<commit_message>
data: oportunidades Visión Circular 2026-05-29
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-06-01
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI24"/>
+  <dimension ref="A1:AI51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4661,6 +4661,4785 @@
       <c r="AI24" t="inlineStr">
         <is>
           <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>VC-0024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Convocatoria Visión Circular 2025-2026 - ANDI</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ANDI (Asociación Nacional de Empresarios de Colombia) / Programa Visión Circular</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Gremio</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Reciclaje, envases y empaques, plásticos flexibles, PET, residuos posconsumo, transformación de materiales</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Cofinanciación; Piloto demostrativo; Investigación aplicada</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Aproximadamente 248-250 millones de pesos por proyecto (ejemplos documentados)</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>https://www.andi.com.co/Uploads/Conv.%20Visi%C3%B3n%20Circular%202025-2026.pdf</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Convocatoria de ANDI para financiar proyectos piloto de economía circular en Colombia que permitan recuperar, transformar y reincorporar residuos de envases y empaques (especialmente PET y plásticos posconsumo) en nuevos productos. Incluye casos como el de Plastilene (recuperación de bandejas PET clamshell) y Pontificia Universidad Javeriana (materiales constructivos con plásticos posconsumo). Ejemplos documentados muestran montos cercanos a 249 millones de pesos por proyecto.</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Es una convocatoria directa del programa Visión Circular de la ANDI, totalmente alineada con sus objetivos de reciclaje, recuperación de plásticos flexibles y envases, innovación en materiales circulares e integración de actores de la cadena de valor.</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>Modelos operativos de recuperación y reciclaje de bandejas PET y clamshell; desarrollo de materiales constructivos con plásticos posconsumo; validación técnica de procesos de transformación; integración de recicladores y actores de cadena de valor</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>No especificado en el extracto</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>No especificado en el extracto</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>Universidades (caso Javeriana), empresas transformadoras de plásticos (caso Plastilene), asociaciones de recicladores, cadena de valor de envases</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Falta claridad sobre fechas de cierre y apertura de próximas convocatorias; documento parece mostrar proyectos aprobados, se requiere confirmar si hay nuevas ventanas abiertas en 2026</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Contactar directamente con Visión Circular ANDI para confirmar si hay convocatoria activa en 2026 y conocer términos de referencia completos.</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>Solicitar TdR actualizados a contacto Visión Circular (info en www.andi.com.co); revisar elegibilidad de proyectos en cartera de Visión Circular para postular</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos Visión Circular ANDI</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>El documento muestra proyectos ya aprobados con códigos PI35, PI29, montos específicos. Es necesario confirmar si la convocatoria 2025-2026 sigue abierta o si habrá nuevas ventanas. | Fuente fuera del listado oficial conocido (andi.com.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>34dd561cb48a5444</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>VC-0025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia Innovation Challenge 2024</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>AgriTech Challenge</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Gestión de residuos, sector agroalimentario, conservación ambiental, reducción de deforestación</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Financiamiento; Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/es/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Desafío de innovación para soluciones circulares en el sector agroalimentario de Colombia. Ofrece acceso a mentores expertos, capacitación en negocios, oportunidades de financiamiento y red de líderes de la industria e inversores. Alineado con el Plan Nacional de Desarrollo 2022-2026 y objetivos de la COP 16 Colombia.</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Enfocado en economía circular y gestión de residuos en el sector agroalimentario, con oportunidad de aplicar principios circulares a empaques agroalimentarios, reciclaje de envases del sector y reducción de residuos.</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>Reciclaje de empaques del sector agroalimentario; tecnologías de valorización de residuos orgánicos; envases compostables o reutilizables para alimentos; modelos de retorno de envases</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Empresas del sector agroalimentario, gremios como SAC, universidades con áreas agroindustriales, cooperativas de recicladores</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>La convocatoria parece haber sido lanzada en 2024; no está claro si sigue abierta en 2026 o si habrá una nueva edición.</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Contactar a AgriTech Challenge para verificar si hay edición 2026 activa o próxima a lanzarse.</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>Visitar el sitio web oficial y contactar vía formulario o email (info disponible en el sitio) para confirmar vigencia y próximas convocatorias</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas empresariales</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>El título menciona 2024, lo que genera incertidumbre sobre vigencia actual. El enfoque agroalimentario es relevante para envases, pero menos central que plásticos flexibles urbanos. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>c75ab3c2ad8e4ed8</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>VC-0026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Convocatoria Fundación AlEn 2026</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Fundación AlEn</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Fundación</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Desarrollo comunitario, reciclaje, protección ambiental</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>https://www.asocapitales.co/sites/default/files/files/technical_documents/boletin-cooperacion-internacional-marzo-2026-2.pdf</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Grant para proyectos de desarrollo comunitario, reciclaje y protección ambiental. Dirigido a organizaciones civiles y gestores locales de sostenibilidad. Ofrece recursos económicos para ejecución de proyectos de impacto ambiental. Fecha límite: 25 de marzo de 2026.</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Directamente alineado con reciclaje y protección ambiental. Aplicable a proyectos comunitarios de reciclaje inclusivo, fortalecimiento de recicladores de base, o pilotos de gestión circular territorial.</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de organizaciones de recicladores; proyectos comunitarios de reciclaje; educación ambiental y separación en la fuente; infraestructura para economía circular territorial</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>Organizaciones civiles y gestores locales de sostenibilidad</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>Asociaciones de recicladores, organizaciones comunitarias, alcaldías locales, universidades con extensión comunitaria</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>No se especifica URL oficial ni monto disponible; falta información sobre elegibilidad geográfica y requisitos detallados</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Buscar información oficial en sitio web de Fundación AlEn o contactar a Asocapitales para obtener términos de referencia completos.</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>Investigar sitio web de Fundación AlEn; contactar a Asocapitales (info@asocapitales.co) para TdR; evaluar elegibilidad para Colombia</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>Coordinación de inclusión social / alianzas con recicladores</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>Fuente secundaria (boletín de Asocapitales). No hay URL oficial de la convocatoria ni confirmación de elegibilidad para Colombia. Fecha de cierre cercana (25 marzo 2026). | Fuente fuera del listado oficial conocido (asocapitales.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>4b69b2552677574d</t>
+        </is>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>VC-0027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Google.org - Financiación para proyectos con Inteligencia Artificial</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Google.org</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Fundación</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Global (incluye Colombia y América Latina)</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Innovación</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Inteligencia artificial aplicada a problemas científicos y sociales</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>No especificado (fondos globales)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>https://www.asocapitales.co/sites/default/files/files/technical_documents/boletin-cooperacion-internacional-marzo-2026-2.pdf</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Grant y asistencia técnica de Google.org para proyectos que usen inteligencia artificial para resolver problemas científicos y sociales. Dirigido a universidades, ONGs y entidades del Estado con áreas de innovación. Incluye fondos globales y acompañamiento de expertos de Google. Cierre: 17 de abril de 2026.</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Aplicable si se desarrollan proyectos que usen IA para optimizar procesos de reciclaje, trazabilidad de materiales, clasificación automatizada de residuos, ecodiseño predictivo o mejora de cadenas circulares.</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>IA para clasificación automatizada de residuos plásticos; sistemas de trazabilidad blockchain+IA para envases; plataformas de ecodiseño asistidas por IA; optimización de rutas de recolección con machine learning</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>Universidades, ONGs y entidades del Estado con áreas de innovación</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>Universidades con centros de IA (Andes, Nacional, Javeriana), centros de investigación tecnológica, empresas tech, entidades públicas de innovación</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>Altamente competitivo a nivel global; requiere capacidad técnica avanzada en IA; no está claro si hay priorización regional</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Evaluar si hay proyectos en cartera de Visión Circular con componente de IA que puedan ser postulados; explorar alianzas con universidades y centros de investigación.</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>Buscar URL oficial de convocatoria Google.org; contactar área de innovación de universidades aliadas; revisar si hay sesiones informativas</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Coordinación de innovación / alianzas con universidades</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>Fuente secundaria (boletín Asocapitales). Relevancia indirecta para Visión Circular (requiere enfoque en IA). Alta competitividad global. Fecha de cierre próxima (17 abril 2026). | Fuente fuera del listado oficial conocido (asocapitales.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>43e1da2484895a5c</t>
+        </is>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>VC-0028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Programa de innovación para la circularidad de los plásticos en América Latina 2025 - WRAP</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>WRAP (The Waste and Resources Action Programme) / Pacto por los Plásticos Colombia, Chile y México</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ONG</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Reino Unido</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Colombia, Chile, México</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Plásticos flexibles, reciclaje, sachets, empaques multilaminados, etiquetas, bolsas plásticas</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Aceleración; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Hasta USD 10.000 por solución seleccionada</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Noviembre de 2025</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>https://www.pactoglobal-colombia.org/news/convocatoria-regional-otorgara-hasta-usd-10-000-a-soluciones-innovadoras-en-plasticos-en-colombia-chile-y-mexico.html</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Programa desarrollado por WRAP en alianza con Pacto por los Plásticos de Colombia, Chile y México. Busca apoyar hasta 10 soluciones innovadoras que prevengan la contaminación por plásticos, con énfasis en plásticos flexibles (sachets, empaques multilaminados, etiquetas, bolsas). Ofrece hasta USD 10.000 por solución seleccionada, más apoyo técnico de WRAP y la Red Global de Pactos por los Plásticos. Convocatoria lanzada en noviembre de 2025.</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Altamente alineado con Visión Circular: enfoque específico en plásticos flexibles (uno de los principales desafíos del programa), soluciones innovadoras de reciclaje, prevención de contaminación y circularidad de envases y empaques.</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Tecnologías de reciclaje de plásticos flexibles; soluciones de recolección de sachets y multilaminados; alternativas de diseño para envases flexibles reciclables; modelos de negocio para circularidad de empaques flexibles</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>No especificado en la fuente (ver URL oficial)</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>No especificado en la fuente (ver URL oficial)</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>Pacto Global Red Colombia, Pacto por los Plásticos Colombia, empresas de envases flexibles, transformadores de plástico, recicladores especializados, universidades</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>El monto de USD 10.000 es relativamente bajo para pilotos de gran escala; se requiere verificar si la convocatoria aún está abierta (anuncio de noviembre 2025)</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Verificar urgentemente si la convocatoria sigue abierta; contactar a Pacto Global Red Colombia para obtener TdR; identificar soluciones innovadoras en plásticos flexibles de empresas de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>Contactar a Pacto Global Red Colombia (info@pactoglobal-colombia.org, tel. 601 636 3638); revisar formulario de aplicación en enlace oficial; preparar ficha de proyecto</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / área de envases y empaques</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>Convocatoria altamente relevante y alineada. Anunciada en noviembre de 2025, pero no se especifica fecha de cierre. Requiere verificación urgente de vigencia. Monto limitado pero con alto valor de acompañamiento técnico. | Fuente fuera del listado oficial conocido (pactoglobal-colombia.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>989708219a39fd28</t>
+        </is>
+      </c>
+      <c r="AI29" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>VC-0029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Programa Vincúlate y Crece Sostenible - Bancóldex / Swisscontact</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Bancóldex / Swisscontact / Banca de las Oportunidades</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Financiamiento verde, instituciones microfinancieras</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Asistencia técnica; Fortalecimiento institucional; Financiamiento concesional</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>https://www.bancoldex.com/soluciones-de-fortalecimiento-empresarial/programa-vinculate-y-crece-sostenible</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Programa de Bancóldex, Swisscontact y Banca de las Oportunidades para seleccionar hasta 5 Instituciones Microfinancieras con límite de exposición de crédito en Bancóldex, con el fin de promover el financiamiento verde. Busca fortalecer capacidades de IMFs para financiar proyectos sostenibles.</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Aplicable si Visión Circular articula con instituciones microfinancieras para financiar emprendimientos circulares, recicladores formalizados, o pequeñas empresas del sector. Fortalece el eslabón financiero de la economía circular.</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Financiamiento a organizaciones de recicladores; crédito verde para MiPymes del sector de reciclaje; fortalecimiento de IMFs que financian economía circular; inclusión financiera de actores circulares</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Instituciones Microfinancieras con límite de exposición de crédito en Bancóldex</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>Instituciones microfinancieras (Bancamía, Contactar, etc.), organizaciones de recicladores, cooperativas, Banca de las Oportunidades</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>Dirigido específicamente a IMFs, no directamente a proyectos; requiere articulación con intermediarios financieros</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Identificar IMFs que trabajen con recicladores o MiPymes circulares; explorar alianzas para canalizar financiamiento verde hacia actores de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>Contactar a Bancóldex para conocer TdR y lista de IMFs participantes; explorar alianzas con IMFs para financiamiento de recicladores y empresas circulares</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>Coordinación de inclusión social / alianzas financieras</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>Dirigido a IMFs, no directamente a proyectos. Relevancia indirecta para Visión Circular. No se especifican fechas de convocatoria. | Fuente fuera del listado oficial conocido (bancoldex.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>6231f4a7d6b23915</t>
+        </is>
+      </c>
+      <c r="AI30" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>VC-0030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Líneas de Crédito para Desarrollo Sostenible - Bancóldex</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Bancóldex</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Eficiencia energética, energía renovable, construcción sostenible, certificaciones ambientales</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Hasta COP 1.500 millones para eficiencia energética y energía renovable; hasta COP 2.000 millones para Desarrollo Sostenible</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>https://www.bancoldex.com/creditos-para-el-desarrollo-sostenible-de-las-empresas</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Líneas de crédito de Bancóldex para empresas colombianas que desarrollen proyectos de eficiencia energética, energía renovable, construcción sostenible y obtención de certificaciones ambientales (ISO 14001, Sello Ambiental Colombiano, etc.). Montos hasta COP 1.500 millones para eficiencia energética/renovables y hasta COP 2.000 millones para desarrollo sostenible. Convocatoria permanente.</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Aplicable a empresas de Visión Circular que requieran financiamiento para infraestructura sostenible, plantas de reciclaje con eficiencia energética, certificaciones ambientales o proyectos de energía renovable en sus operaciones.</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>Infraestructura de reciclaje con eficiencia energética; plantas de transformación de residuos; certificaciones ISO 14001 para empresas del sector; energías renovables en centros de acopio y transformación</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Empresas colombianas; proyectos enmarcados en eficiencia energética, energía renovable, construcción sostenible o certificaciones ambientales</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>No especificado (consultar con Bancóldex)</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>Bancóldex, bancos comerciales intermediarios, empresas del sector de reciclaje y transformación, consultores en eficiencia energética</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>Es crédito, no grant (requiere capacidad de pago); montos pueden ser insuficientes para proyectos de gran escala</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Difundir entre empresas de Visión Circular la disponibilidad de estas líneas de crédito; apoyar en preparación de solicitudes para proyectos elegibles.</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>Contactar a Bancóldex para conocer requisitos y proceso de solicitud; identificar empresas de Visión Circular interesadas; preparar fichas de proyecto</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Coordinación de empresas / área de financiamiento</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>Línea de crédito permanente, no convocatoria competitiva. Relevancia indirecta para economía circular (enfoque en eficiencia energética y certificaciones, no en reciclaje per se). | Fuente fuera del listado oficial conocido (bancoldex.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>7a8276010755790f</t>
+        </is>
+      </c>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>VC-0031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Aceleradora de Financiamiento Climático Colombia 2026</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator (CFA) Colombia</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Residuos y economía circular</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>A partir de USD 1 millón (requerimiento mínimo del proyecto)</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>https://www.emprendemejor.org/post/convocatoria-de-financiamiento-clim%C3%A1tico-2026-en-colombia</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DT_Qk01FT3L</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>La Aceleradora de Financiamiento Climático Colombia 2026 busca proyectos consolidados o en fase de crecimiento con requerimientos de financiamiento desde USD 1 millón. Ofrece fortalecimiento de casos de inversión, estrategias de levantamiento de capital y relacionamiento con inversionistas. Prioriza cinco sectores, incluyendo Residuos y economía circular.</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Directamente relevante para Visión Circular ANDI al priorizar proyectos de residuos y economía circular con potencial de mitigación climática. Permite fortalecer proyectos empresariales de reciclaje, aprovechamiento y circularidad para acceder a financiamiento climático.</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Proyectos de aprovechamiento de residuos de envases y empaques; infraestructura para reciclaje inclusivo; captura de metano; modelos de negocio circulares empresariales; pilotos de circularidad en cadenas de valor; proyectos REP con impacto climático medible</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Proyectos consolidados o en fase de crecimiento; estructura financiera y modelo operativo robusto o en etapa de factibilidad; requerimientos de financiamiento mínimo USD 1 millón; potencial de mitigación o adaptación climática; resultados medibles</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>Caso de inversión; modelo financiero; estructura operativa del proyecto; indicadores de impacto climático; No especificado documentación completa</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>Empresas ANDI sector envases y empaques; gremios productivos; inversionistas de impacto; fondos climáticos; centros tecnológicos; organizaciones de recicladores formalizadas</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>Fecha de cierre cercana (20 feb 2026); requiere proyecto con madurez avanzada y estructura financiera robusta; monto mínimo alto puede excluir proyectos pequeños; competencia por cupos (10 proyectos seleccionados en cohorte actual)</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Identificar inmediatamente 2-3 proyectos empresariales de Visión Circular con potencial de financiamiento superior a USD 1 millón y comenzar preparación de caso de inversión. Priorizar proyectos con datos de reducción de emisiones o captura de metano.</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>Mapear proyectos empresariales en curso dentro de Visión Circular con potencial de escalamiento; contactar a organizadores de CFA Colombia para confirmar requisitos exactos y proceso de postulación; preparar preconcepto ejecutivo para validación interna ANDI esta semana</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Dirección Ejecutiva Visión Circular con apoyo de Coordinación de proyectos y Alianzas empresariales</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>Sectores priorizados incluyen explícitamente 'Residuos y economía circular'. La fecha de cierre es febrero 2026 (en 13 días aprox si hoy es inicio feb 2026). Se infiere que es convocatoria anual basada en cohorte 2026. Requiere validación urgente de si la fecha límite es real o si hay extensión. | Fuente fuera del listado oficial conocido (emprendemejor.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>a46412d5663e5919</t>
+        </is>
+      </c>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>VC-0032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Programa de innovación para la economía circular de los plásticos en América Latina 2025 (Cempre-WRAP)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Cempre Colombia, WRAP (Waste and Resources Action Programme), Red Global de Pactos por los Plásticos</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Internacional (Reino Unido WRAP) / Colombia Cempre</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Colombia, Chile, México</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Plásticos flexibles, Envases y empaques</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Asistencia técnica; Aceleración; Innovación</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>2025-09-22</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>https://cempre.org.co/nuevo-programa-de-innovacion-para-la-economia-circular-de-los-plasticos-en-america-latina-2025</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Convocatoria para seleccionar 10 soluciones empresariales innovadoras enfocadas en envases y empaques plásticos flexibles en Colombia, Chile y México. Ofrece programa de fortalecimiento de capacidades, apoyo técnico, talleres especializados y acceso a redes empresariales para impulsar escalabilidad y expansión a nuevos mercados.</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular ANDI dado el enfoque en envases y empaques plásticos flexibles, uno de los retos centrales del programa. Permite conectar empresas colombianas con red internacional y fortalecer capacidades en economía circular de plásticos.</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Innovación en reciclaje de flexibles; ecodiseño de empaques; sustitución de plásticos problemáticos; nuevos modelos de negocio para envases retornables; tecnologías de clasificación y aprovechamiento de flexibles; proyectos piloto empresariales</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Empresas de cualquier tamaño; organizaciones legales con capacidad de operar en Colombia, Chile o México; soluciones enfocadas en retos de envases y empaques flexibles; innovación demostrable</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>Empresas ANDI del sector empaques; productores de resinas; transformadores de plásticos; empresas de consumo masivo; recicladores especializados; universidades con líneas de investigación en materiales</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>Convocatoria regional con alta competencia; no especifica monto de apoyo económico directo, solo asistencia técnica; se infiere que es más aceleración que financiamiento; requiere capacidad operativa en países priorizados</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Mapear empresas colombianas del programa Visión Circular con soluciones innovadoras en plásticos flexibles y promover su postulación. Considerar postulación conjunta ANDI-empresa como mecanismo de apoyo.</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>Solicitar términos de referencia completos a Cempre Colombia; identificar 3-5 empresas o startups candidatas dentro del ecosistema Visión Circular; preparar carta de apoyo institucional ANDI para fortalecer postulaciones</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>Coordinación técnica de Visión Circular con apoyo de área de Innovación y Alianzas empresariales</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>Fecha de cierre septiembre 2025 da ventana amplia. Cempre Colombia es aliado conocido de ANDI. WRAP es organización internacional reconocida. No queda claro si hay financiamiento directo o solo asistencia técnica, pero el apoyo en capacidades y redes es valioso. | Fuente fuera del listado oficial conocido (cempre.org.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>df72dc0a738ed612</t>
+        </is>
+      </c>
+      <c r="AI33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>VC-0033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Convocatoria EcoCiclo - Agencia ATENEA Bogotá</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Agencia ATENEA - Agencia Distrital para la Educación Superior, la Ciencia y la Tecnología (Bogotá)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Gobierno</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Bogotá D.C., Colombia</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Ecodiseño, Envases y empaques, Reciclaje, Plásticos de un solo uso</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Cofinanciación; Innovación; Investigación aplicada</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Sí, requiere alianza entre centros de investigación y empresas</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2025-09-25</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>https://agenciaatenea.gov.co/noticias/agencia-atenea-lanza-convocatoria-para-promover-la-sustitucion-de-plasticos-de-un-solo-uso-y-el</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Convocatoria EcoCiclo busca conformar un Banco de Proyectos de investigación e innovación en alianzas entre centros de investigación y empresas que utilizan empaques y envases. Financia proyectos en ecodiseño, alternativas sostenibles, sustitución de plásticos de un solo uso, aprovechamiento de residuos y economía circular. Los proyectos financiables definitivos se conocerán el 3 de noviembre 2025.</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Muy pertinente para Visión Circular ANDI al enfocarse en ecodiseño de envases y empaques, sustitución de plásticos de un solo uso y aprovechamiento de residuos. Permite articular empresas ANDI con centros de investigación bogotanos para proyectos de I+D+i aplicada.</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>Ecodiseño de envases y empaques; sustitución de plásticos de un solo uso por alternativas sostenibles; aprovechamiento de residuos de empaques; vigilancia tecnológica en soluciones circulares; desarrollo de materiales alternativos; procesos de reciclaje mejorado</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Alianza estratégica entre centros de investigación y empresas que utilizan empaques y envases; proyecto de investigación e innovación aplicada; enfoque en las temáticas priorizadas; localización o capacidad de ejecución en Bogotá</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>Términos de referencia deben consultarse en plataforma de Agencia ATENEA; se infiere que requiere propuesta técnica, presupuesto, acuerdos de colaboración, justificación de innovación</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>Universidades bogotanas (Andes, Nacional, Javeriana, EAN, etc.); centros de investigación (Corporación Innovar, CIAB); empresas ANDI del sector empaques (Alquería, Alpina, Bavaria, empresas de transformación de plásticos); Sena - Centro de Tecnología de Manufactura Avanzada</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>Convocatoria distrital limitada a Bogotá; requiere alianza previa con centro de investigación; proceso competitivo; fecha de resultado (nov 2025) implica ejecución 2026; no especifica montos disponibles</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Difundir convocatoria entre empresas ANDI en Bogotá con retos en envases y empaques. Facilitar ruedas de conexión entre empresas y centros de investigación. Preparar carta de apoyo institucional ANDI para proyectos alineados con Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>Descargar términos de referencia completos de EcoCiclo; organizar webinar informativo para empresas ANDI; mapear centros de investigación disponibles para alianzas; identificar 5 empresas prioritarias con retos concretos en envases</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos Visión Circular con apoyo de área de Innovación y relacionamiento con academia</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>Convocatoria cerrada en septiembre 2025 pero con ventana amplia. La fuente es oficial (sitio web Agencia ATENEA). No especifica montos pero siendo agencia distrital de CTI se infiere financiamiento significativo. Requiere presencia o capacidad de ejecución en Bogotá. | Fuente fuera del listado oficial conocido (agenciaatenea.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>000232e27d75cf67</t>
+        </is>
+      </c>
+      <c r="AI34" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>VC-0034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Programa de Pequeñas Donaciones del GEF Colombia (PPD-GEF)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) / PNUD Colombia</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Internacional / Colombia</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Biodiversidad y ambiente</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Gestión comunitaria, Producción sostenible, Negocios verdes</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Pequeñas donaciones (fondos no reembolsables)</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente (convocatorias periódicas)</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/es/colombia/projects/programa-pequenas-donaciones-gef</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>El Programa de Pequeñas Donaciones del GEF en Colombia fortalece la gestión ambiental comunitaria mediante fondos no reembolsables. Trabaja en conservación de biodiversidad, cambio climático, producción sostenible y negocios verdes con enfoque comunitario y territorial. Cobertura nacional con tres líneas temáticas priorizadas.</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Pertinencia indirecta para Visión Circular: permite apoyar proyectos comunitarios de aprovechamiento de residuos, negocios verdes de reciclaje, producción sostenible con enfoque circular y fortalecimiento de organizaciones de recicladores de base con impacto en conservación y clima.</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Negocios verdes de aprovechamiento de residuos orgánicos; fortalecimiento de cooperativas de recicladores en territorios priorizados; producción sostenible con cierre de ciclo de materiales; proyectos comunitarios de economía circular rural; emprendimientos de economía circular con comunidades</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>Enfoque comunitario; contribución a conservación de biodiversidad y/o cambio climático; fortalecimiento de capacidades locales; mejoramiento de modos de vida; alineación con una de las tres líneas temáticas del programa</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>No especificado en la fuente; típicamente requiere propuesta de proyecto comunitario, presupuesto, aval comunitario, carta de compromiso organizacional</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>Organizaciones de recicladores de base; cooperativas rurales; autoridades ambientales regionales; alcaldías municipales; ONGs locales; organizaciones comunitarias; resguardos indígenas con proyectos de manejo de residuos</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>Programa orientado principalmente a conservación de biodiversidad, no específicamente a economía circular urbana o envases; montos pequeños pueden no ajustarse a proyectos empresariales; proceso puede ser lento; requiere fuerte componente comunitario</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>Explorar si el PPD-GEF puede financiar componentes de inclusión de recicladores de base en iniciativas de Visión Circular, especialmente en territorios priorizados. Considerar para proyectos piloto comunitarios de aprovechamiento de residuos con enfoque de biodiversidad o clima.</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>Contactar al coordinador del PPD-GEF Colombia en PNUD para entender mejor elegibilidad de proyectos de economía circular y reciclaje inclusivo; revisar si hay convocatorias abiertas actualmente; explorar alianza para componente comunitario de proyectos mayores de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>Coordinación de Inclusión social o Coordinación de proyectos territoriales de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>Programa permanente pero convocatorias son periódicas (no especifica fechas actuales). Pertinencia indirecta porque prioriza biodiversidad sobre circularidad industrial, pero puede ser relevante para componentes de inclusión de recicladores y proyectos comunitarios. Requiere validar si proyectos de reciclaje urbano son elegibles bajo línea de negocios verdes.</t>
+        </is>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>06e771a455944223</t>
+        </is>
+      </c>
+      <c r="AI35" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>VC-0035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Green Climate Fund - Ventana de financiamiento para Colombia</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Colombia y otros países en desarrollo</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Mitigación y adaptación climática, Movilidad sostenible, Agricultura sostenible, Gestión forestal</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Grant no reembolsable; Financiamiento concesional</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Variable por proyecto (millones de USD)</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Sí, típicamente requiere cofinanciamiento</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Permanente</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Permanente (proceso continuo de propuestas)</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/countries/colombia</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>El Green Climate Fund mantiene una cartera activa en Colombia con múltiples proyectos aprobados y en ejecución. Financia proyectos de gran escala en mitigación y adaptación climática, incluyendo movilidad sostenible, agricultura climáticamente inteligente y conservación forestal. Acceso vía entidades acreditadas (Banco Mundial, BID, Findeter, etc.).</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Pertinencia moderada para Visión Circular: proyectos de economía circular con alto impacto climático (ej. captura de metano, reducción de emisiones industriales, gestión de residuos con mitigación) podrían ser elegibles. Requiere escala grande y demostración de impacto climático medible y alineación con NDC de Colombia.</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Infraestructura de gestión de residuos con captura de metano; proyectos de economía circular industrial con reducción de emisiones; sistemas de aprovechamiento de residuos orgánicos a gran escala; infraestructura para reciclaje inclusivo con componente climático; modelos circulares en agricultura (envases agrícolas)</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>Acceso vía entidad acreditada (BID, Banco Mundial, Findeter, etc.); proyecto de gran escala; impacto climático demostrable y medible; alineación con NDC de Colombia; cambio transformacional; cofinanciamiento robusto; sostenibilidad financiera</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>Concept Note; Funding Proposal completo; estudios de factibilidad; evaluación de impacto climático; plan de género; salvaguardas ambientales y sociales; plan financiero; cartas de no objeción de la AND (Autoridad Nacional Designada)</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>Entidades acreditadas: Findeter, BID, Banco Mundial, CAF; Ministerio de Ambiente (AND Colombia); DNP; empresas grandes del sector residuos; autoridades ambientales regionales; gremios empresariales ANDI</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>Proceso largo y complejo (12-24 meses); requiere entidad acreditada como intermediario; altamente competitivo; requiere escala muy grande; foco principal no es economía circular sino clima; costos de preparación altos</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Explorar si proyectos grandes de economía circular dentro de Visión Circular (ej. infraestructura nacional de reciclaje, sistema de captura de metano de residuos) pueden estructurarse para GCF vía Findeter o BID. Requiere componente climático robusto y escala significativa.</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>Contactar a Findeter (entidad acreditada colombiana) y al DNP (punto focal AND) para explorar ventanas de financiamiento aplicables a economía circular; revisar proyectos aprobados de GCF en residuos/economía circular en otros países para aprender; evaluar factibilidad de estructurar megaproyecto</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>Dirección Ejecutiva de Visión Circular en coordinación con Vicepresidencia de Asuntos Corporativos ANDI</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>GCF es fuente de financiamiento climático de largo plazo, no convocatoria específica. La página muestra proyectos aprobados en Colombia pero ninguno específicamente en residuos/economía circular. La elegibilidad depende de demostrar impacto climático transformacional. Proceso complejo que requiere alianza con entidad acreditada. Más una oportunidad estratégica de largo plazo que una convocatoria inmediata.</t>
+        </is>
+      </c>
+      <c r="AH36" t="inlineStr">
+        <is>
+          <t>dfeb9b9bdec01376</t>
+        </is>
+      </c>
+      <c r="AI36" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>VC-0036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Proyecto de Gestión Circular de Residuos y Reducción de Gases de Efecto Invernadero en Medellín</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>KOICA (Agencia de Cooperación de Corea) y Alcaldía de Medellín</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Corea del Sur</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Colombia (Medellín)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Gestión circular de residuos, Reducción de GEI</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Financiamiento concesional; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>16.4 millones</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>2031</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DXGKUEACqjn</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>KOICA y la Alcaldía de Medellín firmaron el Acta de Discusiones (ROD) para un proyecto de USD 16.4 millones que impulsará la gestión circular de residuos y la reducción de gases de efecto invernadero entre 2026 y 2031. Este proyecto busca posicionar a Colombia como referente en soluciones innovadoras frente al cambio climático.</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular ANDI: aborda economía circular territorial, gestión de residuos, reducción de emisiones y posiciona a Colombia como líder regional. Oportunidad de replicar aprendizajes de Medellín en otras ciudades.</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>Articulación con modelo Medellín para replicar en otras ciudades; Sistematización de aprendizajes en gestión circular municipal; Desarrollo de pilotos empresariales alineados con el proyecto; Fortalecimiento de cadenas de reciclaje inclusivo; Innovación en reducción de emisiones desde envases y empaques</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>Alcaldía de Medellín, KOICA Colombia, Área Metropolitana del Valle de Aburrá, empresas de envases y empaques asociadas a ANDI, universidades locales, recicladores organizados</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>El proyecto ya está en fase de implementación (no es convocatoria abierta). Requiere articulación temprana con ejecutores para identificar espacios de colaboración.</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>Contactar a KOICA Colombia y Alcaldía de Medellín para identificar espacios de colaboración, asistencia técnica o réplica del modelo en otras ciudades o sectores (envases y empaques).</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>Solicitar reunión con KOICA Colombia y Secretaría de Medio Ambiente de Medellín para explorar alianzas y oportunidades de articulación con Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas de Visión Circular ANDI</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG37" t="inlineStr">
+        <is>
+          <t>El proyecto ya fue firmado y está en fase de implementación 2026-2031. No es una convocatoria abierta, pero representa una oportunidad estratégica de articulación y réplica. La fuente es una red social oficial (Instagram APC Colombia), se recomienda verificar en fuentes oficiales de KOICA o Alcaldía. | Fuente fuera del listado oficial conocido (instagram.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH37" t="inlineStr">
+        <is>
+          <t>110cc8b6274bf352</t>
+        </is>
+      </c>
+      <c r="AI37" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>VC-0037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia: Agrichallenge</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CGIAR y aliados del Agritech Challenge</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Colombia (nacional y global con soluciones aplicables a Colombia)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Valorización de residuos agroindustriales, Economía circular agroalimentaria, Conversión de residuos en alimento animal y energía renovable</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Financiamiento; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>El CircularEconomy4Colombia Innovation Challenge busca acelerar la transición a la economía circular en el sector agroalimentario de Colombia, alineado con el Plan Nacional de Desarrollo 2022-2026 y los objetivos de la COP 16. Ofrece mentoría, capacitación empresarial, oportunidades de financiación y red de líderes e inversionistas para soluciones en valorización de residuos, tratamiento de aguas residuales, conversión de residuos en alimento animal y energía renovable.</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular: aborda valorización de residuos, economía circular territorial y modelos de negocio circulares. Aunque enfocado en agro, hay sinergias con envases de alimentos, empaques biodegradables y cierre de ciclo en cadenas agroindustriales.</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>Innovación en empaques biodegradables para agroindustria; Valorización de residuos de envases alimentarios; Modelos circulares en cadena de valor agroalimentaria; Integración de recicladores en cadenas agroindustriales; Ecodiseño de empaques para productos agrícolas</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>Soluciones en etapa temprana aplicables a Colombia; innovadores nacionales o globales; científicos de CGIAR con enfoque emprendedor; alineación con áreas prioritarias (valorización de residuos, tratamiento de aguas, conversión de residuos, energía renovable).</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>CGIAR, empresas de agroindustria asociadas a ANDI, universidades con programas de agroindustria y empaques, centros tecnológicos, cooperativas de recicladores</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>Fechas de convocatoria no especificadas. Enfoque principal en agroindustria puede requerir adaptación para envases y empaques de uso general.</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>Verificar fechas de convocatoria en la página oficial. Explorar alianzas con empresas de empaques de alimentos para presentar soluciones conjuntas en economía circular.</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>Visitar el sitio web oficial para confirmar si la convocatoria está abierta, fechas límite y requisitos de aplicación. Contactar al equipo del Challenge.</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>Área de innovación y desarrollo de proyectos de Visión Circular ANDI</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>La página menciona 'aplicar' pero no especifica fechas ni si la convocatoria está actualmente abierta. Parece ser un programa recurrente o con ventanas específicas. Se infiere que es aplicable a Colombia porque está centrado en el país. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH38" t="inlineStr">
+        <is>
+          <t>27e92b16a02cd01c</t>
+        </is>
+      </c>
+      <c r="AI38" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>VC-0038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Too Good to Waste - Llamado a Propuestas BID</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Banco Interamericano de Desarrollo (BID), Global Methane Hub, AquaFund</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Regional (América Latina y el Caribe)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (18 finalistas de 12 países fueron seleccionados de 156 propuestas elegibles)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Residuos</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Gestión de residuos sólidos, Reducción de emisiones de metano, Economía circular</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Cofinanciación; Cooperación técnica; Financiamiento concesional; Fortalecimiento institucional; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>37 millones (demandados solo para estudios de pre-inversión); 4 mil millones anuales requeridos para inversión, operación, mantenimiento y fortalecimiento institucional en LAC</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Sí, el BID explora cofinanciación con GEF (ISLANDS Caribbean Incubator Facility) y #SinDesperdicio (sector privado)</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>https://www.ccap.org/post/latin-america-and-the-caribbean-countries-seek-to-reduce-methane-emissions-in-the-solid-waste-sector</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Too Good to Waste es una iniciativa del BID financiada por Global Methane Hub y AquaFund para mejorar la gestión de residuos sólidos y reducir emisiones de metano en LAC. De 156 propuestas elegibles, se seleccionaron 18 finalistas de 12 países. El BID está explorando cofinanciación con GEF y sector privado. La demanda supera los USD 37 millones para pre-inversión y USD 4 mil millones anuales para inversión total.</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular: aborda gestión de residuos, economía circular, participación del sector privado y fortalecimiento institucional. Es una oportunidad regional con enfoque en reciclaje, valorización y cierre de ciclo.</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Proyectos de pre-inversión en gestión circular de envases y residuos; Modelos de financiamiento para infraestructura de reciclaje; Fortalecimiento de cadenas de reciclaje inclusivo; Reducción de emisiones en gestión de residuos de envases; Alianzas público-privadas para economía circular</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>No especificado en la fuente; se infiere que requiere propuestas de pre-inversión, inversión o fortalecimiento institucional en gestión de residuos con potencial de reducción de metano.</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>BID, Global Methane Hub, AquaFund, GEF, sector privado (#SinDesperdicio), gobiernos locales, empresas de envases y empaques, gremios, recicladores</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>No se especifica si habrá nuevas convocatorias o si el proceso ya cerró con los 18 finalistas. Alta demanda de recursos podría limitar acceso.</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>Contactar al BID para confirmar si habrá nuevas ventanas de aplicación de Too Good to Waste o mecanismos de cofinanciación con GEF o sector privado. Explorar alianza con empresas del sector privado ya vinculadas (#SinDesperdicio).</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>Escribir al BID (División de Agua y Saneamiento / Cambio Climático) para confirmar próximas convocatorias y requisitos. Explorar alianza con finalistas colombianos si los hay.</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas estratégicas y financiamiento de Visión Circular ANDI</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>La fuente describe un proceso ya en marcha (18 finalistas seleccionados) pero menciona que el BID está explorando cofinanciación, lo que sugiere oportunidades futuras. Se requiere verificar si habrá nuevas convocatorias y si Colombia tuvo finalistas. | Fuente fuera del listado oficial conocido (ccap.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH39" t="inlineStr">
+        <is>
+          <t>acbe8ac1b8f5dbd1</t>
+        </is>
+      </c>
+      <c r="AI39" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>VC-0039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Unlocking Innovation in Circular Plastics in the LATAM region 2025</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>WRAP (Waste and Resources Action Programme) y Plastics Pacts Network</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ONG</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Reino Unido / Red global</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>América Latina (Chile, Colombia, México prioritarios; 19 países en la red)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Plásticos circulares, innovación, reciclaje, modelos de negocio circulares</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Aceleración; Fortalecimiento institucional; Grant no reembolsable; Asistencia técnica; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Hasta 3 mini-grants de USD 10,000 cada uno (USD 30,000 total en grants); programa de capacitación y asistencia técnica sin costo</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>No especificado (anunciado para 2025)</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>https://www.wrap.ngo/take-action/plastic-pact-network/innovation-circular-plastics-latam-2025</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>WRAP y la Red de Pactos por los Plásticos otorgarán apoyo a 10 soluciones innovadoras que aborden desafíos críticos en circularidad de plásticos en América Latina. Las soluciones seleccionadas recibirán capacitación intensiva, acceso a redes de inversores, empresas y potenciales pilotos; además, hasta 3 soluciones recibirán mini-grants de USD 10,000 para preparación para inversión y testeo. El programa busca fortalecer modelos de negocio, escalabilidad e impacto real.</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular ANDI: aborda circularidad de plásticos, envases/empaques, innovación empresarial, modelos de negocio circulares y acceso a redes empresariales en Colombia (país prioritario). Alineado con REP, ecodiseño, reciclaje y escalamiento de soluciones.</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Desarrollo de pilotos empresariales de envases circulares; soluciones de reciclabilidad de plásticos flexibles; modelos de negocio circulares escalables; articulación con empresas y gremios afiliados a ANDI; fortalecimiento de cadenas de reciclaje inclusivas; proyectos de ecodiseño aplicado a envases.</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>Soluciones innovadoras enfocadas en circularidad de plásticos; ubicación/operación en América Latina (Chile, Colombia, México priorizados); modelo de negocio escalable; capacidad de participar en programa de capacitación; apertura a pilotos comerciales.</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>No especificado (probablemente: descripción de la solución, modelo de negocio, impacto esperado, equipo)</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Pacto Plásticos Colombia, empresas afiliadas a ANDI con compromisos de envases circulares, universidades con investigación en materiales, centros tecnológicos (ICIPC, SENA), cooperativas de recicladores, inversionistas de impacto</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Fecha de apertura/cierre no especificada; alta competencia regional; mini-grants limitados a 3 soluciones; requiere capacidad de ejecución rápida y escalamiento; dependencia de match con empresas de la red para pilotos</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>Monitorear apertura de convocatoria en página oficial; preparar portafolio de soluciones innovadoras de Visión Circular (ecodiseño, plásticos flexibles, modelos circulares); identificar empresas ANDI con necesidades de innovación en envases; diseñar propuestas escalables con potencial de piloto comercial</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>Suscribirse a actualizaciones en página oficial de WRAP; contactar a Pacto Plásticos Colombia para información privilegiada; preparar pre-propuesta con caso de negocio y equipo; mapear empresas ANDI interesadas en codesarrollo</t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>Coordinación de Innovación y Proyectos, Alianzas Empresariales, Coordinación Técnica Visión Circular</t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG40" t="inlineStr">
+        <is>
+          <t>Oportunidad estratégica altamente alineada. Colombia es país prioritario de la red. ANDI/Visión Circular tiene empresas afiliadas con compromisos de circularidad que pueden ser co-aplicantes o socios comerciales. El formato de aceleración + mini-grant + acceso a red empresarial es ideal para escalar pilotos. Requiere verificar fechas exactas de apertura 2025. | Fuente fuera del listado oficial conocido (wrap.ngo): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH40" t="inlineStr">
+        <is>
+          <t>21214db28bbfbf14</t>
+        </is>
+      </c>
+      <c r="AI40" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>VC-0040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>IFC &amp; BFS Industrial Plastic Circularity in Latin America Initiative</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>International Finance Corporation (IFC) y BFS (Business Finance Solutions)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Global (IFC - Banco Mundial)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>América Latina</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Circularidad industrial de plásticos, inversión sostenible, cadenas de suministro circulares, responsabilidad extendida del productor (REP)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Investigación aplicada; Asistencia técnica; Financiamiento concesional; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>No especificado (enfocado en identificar oportunidades de inversión para pipeline de IFC)</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026 (anunciado)</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>https://rainbowforest.org/bfs/ifc-bfs-plastic-circularity-latin-america-2026</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>IFC y BFS lanzaron en 2026 una iniciativa para mapear oportunidades de circularidad industrial de plásticos en América Latina, desarrollar herramientas de diagnóstico empresarial para reducción de plástico virgen, pilotar hojas de ruta de circularidad con empresas seleccionadas, e identificar oportunidades de inversión para el pipeline de IFC. La iniciativa busca cerrar la brecha entre compromisos de sostenibilidad y acción real, validando ventures con potencial comercial e impacto socioambiental.</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular: enfoque en REP, cadenas circulares de plásticos/envases, diagnóstico empresarial, hojas de ruta de circularidad y acceso a financiamiento de desarrollo. Puede facilitar acceso de empresas ANDI a financiamiento IFC y asistencia técnica para circularidad industrial.</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Diagnóstico de línea base de plástico virgen en empresas afiliadas ANDI; desarrollo de hojas de ruta de circularidad empresarial; diseño de proyectos de inversión en infraestructura de reciclaje o economía circular; pilotos de cadenas de suministro circulares; acceso a financiamiento IFC para escalamiento de soluciones circulares.</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>Empresas con operaciones en América Latina; compromiso de reducción de plástico virgen; disposición a participar en diagnóstico y hoja de ruta; potencial de inversión y escalamiento comercial; datos verificables de uso de plásticos.</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>No especificado (probablemente: datos de consumo de plásticos, compromisos de sostenibilidad, modelo de negocio, capacidad financiera)</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Empresas grandes y medianas afiliadas a ANDI con compromisos de envases sostenibles, IFC Colombia, centros de investigación aplicada, proveedores de tecnología de reciclaje, inversionistas de impacto</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Iniciativa en fase de mapeo (lanzada en 2026 según fuente); no es convocatoria abierta sino selección dirigida de empresas; acceso limitado a empresas con escala y capacidad de inversión; proceso largo de diagnóstico a inversión; no hay grant directo, enfocado en préstamos/equity IFC</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>Contactar a IFC Colombia para expresar interés de empresas ANDI; proponer Visión Circular como plataforma de articulación empresarial; ofrecer datos agregados de sector de envases/empaques; posicionar empresas afiliadas para pilotos de hojas de ruta; explorar cofinanciamiento IFC para proyectos de infraestructura circular</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>Establecer contacto con IFC Colombia y BFS; preparar portafolio de empresas ANDI con potencial de circularidad industrial; solicitar reunión para explorar participación de Visión Circular como hub de articulación; preparar datos sectoriales de plásticos/envases</t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>Dirección Visión Circular, Coordinación de Alianzas Estratégicas, Financiación de Proyectos</t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG41" t="inlineStr">
+        <is>
+          <t>Iniciativa estratégica de largo plazo enfocada en empresas con capacidad de inversión. No es grant abierto sino mapeo y pipeline de inversión IFC. Visión Circular/ANDI puede posicionarse como articulador de empresas para diagnóstico y hojas de ruta. Acceso a financiamiento IFC requiere empresas con solidez financiera. La fuente menciona 2026 como lanzamiento, lo que sugiere que la iniciativa está activa o por activarse. | Fuente fuera del listado oficial conocido (rainbowforest.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH41" t="inlineStr">
+        <is>
+          <t>0094f4dd5f5f76d2</t>
+        </is>
+      </c>
+      <c r="AI41" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>VC-0041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PREVEC II - Circular Economy and Green Jobs (GIZ Colombia)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Deutsche Gesellschaft für Internationale Zusammenarbeit (GIZ)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Empleos verdes, modelos de negocio circulares, inclusión de género, reducción de emisiones GEI, capacidad institucional</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Fortalecimiento institucional; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>https://www.giz.de/en/downloads/giz2024-en-colombia-circular-economy.pdf</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>PREVEC II es un proyecto de cooperación alemana (GIZ) con Colombia que fortalece capacidades técnicas e institucionales de actores gubernamentales y privados para implementar medidas de economía circular relacionadas con clima y empleo a nivel local y nacional. Apoya 15 modelos de negocio circulares (7 con alto potencial de reducción de GEI, liderados por pequeñas empresas/organizaciones, 6 por mujeres) y promueve instrumentos de empleo verde con enfoque de género en el sector de economía circular, especialmente recicladores.</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Altamente relevante: GIZ es socio estratégico clave en economía circular en Colombia. PREVEC II trabaja directamente con sector privado en modelos de negocio circulares, inclusión de recicladores, empleo verde y capacidad institucional, temas centrales de Visión Circular ANDI. Oportunidad de articulación directa.</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>Desarrollo/escalamiento de modelos de negocio circulares con empresas ANDI; fortalecimiento de capacidades en REP; inclusión de recicladores en cadenas circulares empresariales; análisis de potencial de empleo verde en economía circular; instrumentos de promoción de empleo circular con enfoque de género; medición de reducción de GEI en iniciativas circulares</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>Actores gubernamentales o privados en Colombia; enfoque en economía circular con impacto climático y de empleo; modelos liderados por pequeñas empresas o con liderazgo de mujeres priorizados; potencial de reducción de GEI; inclusión de recicladores</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>GIZ Colombia, Agencia Presidencial de Cooperación Internacional (APC-Colombia), Ministerio de Ambiente y Desarrollo Sostenible, Ministerio de Vivienda Ciudad y Territorio, municipios, empresas afiliadas a ANDI, organizaciones de recicladores, organizaciones lideradas por mujeres</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>Documento de 2024 no especifica si PREVEC II está activo o en qué fase; no hay convocatoria abierta identificada; cooperación técnica puede ser dirigida/por invitación; tiempos de GIZ pueden ser largos</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>Contactar a GIZ Colombia para explorar articulación formal entre PREVEC II y Visión Circular ANDI; proponer empresas/proyectos de Visión Circular para apoyo técnico en modelos de negocio circulares; alinear agendas en inclusión de recicladores y empleo verde; solicitar asistencia técnica para empresas afiliadas en REP y circularidad</t>
+        </is>
+      </c>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>Identificar punto focal PREVEC II en GIZ Colombia; solicitar reunión de articulación; preparar portafolio de proyectos de Visión Circular alineados con objetivos PREVEC II; explorar cofinanciamiento/coejección de iniciativas</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>Dirección Visión Circular, Coordinación de Alianzas Estratégicas, Cooperación Internacional</t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr">
+        <is>
+          <t>PREVEC II es proyecto de cooperación técnica activo de GIZ en Colombia, altamente alineado con Visión Circular. Aunque no es convocatoria abierta, GIZ busca socios estratégicos del sector privado para implementación. ANDI/Visión Circular puede ser socio ideal por su convocatoria empresarial y enfoque en circularidad y recicladores. Requiere articulación directa proactiva.</t>
+        </is>
+      </c>
+      <c r="AH42" t="inlineStr">
+        <is>
+          <t>aa78fc8c5989b560</t>
+        </is>
+      </c>
+      <c r="AI42" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>VC-0042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>IFC Regional Initiative - Industrial Plastic Circularity Opportunities in Latin America and the Caribbean</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>IFC (International Finance Corporation) - World Bank Group, en alianza con BlackForest Solutions GmbH y ABIPLAST</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Estados Unidos (sede IFC)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Brasil y América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Plásticos - circularidad, reducción de huella de plástico virgen y fósil, oportunidades de inversión en cadena de valor</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Investigación aplicada; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>USD 1.9 mil millones (estimado basado en Harmonized Circular Economy Guidelines)</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>https://www.ifc.org/en/pressroom/2026/ifc-launches-regional-initiative-to-accelerate-investment-ready-industrial-plastic</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>IFC lanza iniciativa regional en alianza con ABIPLAST y BlackForest Solutions para identificar y acelerar oportunidades de inversión listas para financiación en circularidad de plásticos industriales en Brasil y América Latina. La iniciativa cuantifica huellas de plástico virgen y fósil, prioriza palancas de reducción factibles y traduce ambiciones circulares en oportunidades de inversión financiables para grandes usuarios de plástico, convertidores y actores clave de la cadena de valor.</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI: aborda directamente circularidad de plásticos, cuantificación de huellas, ecodiseño implícito, y financiamiento de proyectos circulares con actores industriales, alineado con REP, reciclaje y modelos de negocio circulares en el sector de envases y empaques.</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>Diagnóstico de huella de plásticos en empresas asociadas ANDI; desarrollo de business cases para inversión en reciclaje químico o mecánico de plásticos flexibles; articulación con ABIPLAST para aprendizaje regional; preparación de proyectos financiables para reducción de plástico virgen en envases.</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>Ser actor relevante en cadena de valor de plásticos (usuarios, convertidores, recicladores); capacidad de cuantificar huella de plástico; interés en traducir estrategias circulares en proyectos de inversión.</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>ABIPLAST (Brasil), empresas transformadoras de plástico ANDI, gremios de envases, universidades con investigación en materiales, IFC Colombia, Ministerio de Ambiente</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>Foco inicial en Brasil podría limitar acceso directo; requiere capacidad técnica para cuantificación; dependencia de interés de IFC en proyectos específicos</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>Contactar oficina IFC Colombia y expresar interés de ANDI/Visión Circular en participar como socio estratégico; identificar empresas miembro interesadas en diagnósticos de circularidad de plásticos; explorar articulación con ABIPLAST.</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>Enviar carta de interés a IFC Colombia y a BlackForest Solutions; solicitar reunión exploratoria; identificar 3-5 empresas miembro ANDI para piloto.</t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos internacionales y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>Iniciativa recién lanzada (marzo 2026), aún en fase de implementación. No se especifica proceso de postulación formal, pero la naturaleza de cooperación técnica sugiere que actores regionales pueden expresar interés. Estimación de USD 1.9 mil millones aparece en el texto como potencial de la economía circular aplicando las guías armonizadas, no necesariamente como presupuesto del programa.</t>
+        </is>
+      </c>
+      <c r="AH43" t="inlineStr">
+        <is>
+          <t>c5d502e880cd4a2b</t>
+        </is>
+      </c>
+      <c r="AI43" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>VC-0043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>IDB Lab - Caribbean Loans Call for Proposals</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>IDB Lab (Banco Interamericano de Desarrollo)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Regional - América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Países del Caribe</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Clima, inclusión financiera, impacto social</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Resiliencia climática, economía circular implícita, financiamiento a PyMEs y organizaciones de base</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Cofinanciación</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>No especificado (producto de deuda para PyMEs y organizaciones de base)</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>No especificado; se menciona demostrar sostenibilidad financiera</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>https://bidlab.org/en/home/caribbean-loans-call-proposals</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>IDB Lab busca identificar candidatos elegibles para su producto de financiamiento de deuda (préstamos) en el Caribe, dirigido a PyMEs y organizaciones de base que trabajen en inclusión financiera, resiliencia climática e impacto social. Los solicitantes deben demostrar modelo de negocio sólido, tracción, potencial de crecimiento, sostenibilidad financiera, y contar con estados financieros auditados de los últimos 3 años completos y cuentas de gestión recientes en 2025.</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Relevancia indirecta pero aprovechable: aunque no menciona economía circular explícitamente, la convocatoria busca soluciones de resiliencia climática e impacto social, donde se pueden enmarcar proyectos de gestión de residuos, reciclaje, inclusión de recicladores y cadenas circulares en contexto caribeño.</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>Financiamiento de infraestructura de reciclaje en Caribe colombiano (San Andrés, Providencia); proyectos de inclusión de organizaciones de recicladores; soluciones circulares para gestión de residuos en islas; modelos de economía circular en turismo sostenible.</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>PyME u organización de base en el Caribe; modelo de negocio sólido con tracción; enfoque en inclusión financiera, resiliencia climática o impacto social; estados financieros auditados (3 años completos) y cuentas de gestión 2025; sostenibilidad financiera demostrable.</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>Estados financieros auditados (últimos 3 años completos); cuentas de gestión más recientes (2025); documentos sobre modelo de negocio, impacto y sostenibilidad (formato no especificado)</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>Organizaciones de recicladores del Caribe colombiano; PyMEs de gestión de residuos; alcaldías de San Andrés, Providencia; universidades regionales; cooperación caribeña</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>Foco exclusivo en Caribe puede limitar alcance; requisito de estados financieros auditados excluye a organizaciones informales o pequeñas; no especifica montos ni condiciones de préstamo</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>Explorar si organizaciones de recicladores o PyMEs de economía circular en Caribe colombiano califican; preparar propuesta de concepto si existe piloto en San Andrés o Providencia; consultar con IDB Lab sobre elegibilidad específica.</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>Revisar portafolio de Visión Circular en Caribe colombiano; contactar IDB Lab para aclarar elegibilidad de organizaciones colombianas con operaciones caribeñas; identificar socios locales con capacidad financiera.</t>
+        </is>
+      </c>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas estratégicas y proyectos territoriales</t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>Convocatoria abierta permanentemente pero enfocada exclusivamente en Caribe. Aunque Colombia tiene territorios caribeños (San Andrés, Providencia, costa Caribe), la elegibilidad depende de la interpretación de 'Caribbean' por IDB Lab (puede referirse a países insulares caribeños, excluyendo costas continentales). Requiere verificación de elegibilidad para Colombia. No menciona economía circular explícitamente, pero resiliencia climática puede incluirla.</t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr">
+        <is>
+          <t>97fe4eee9f460e9b</t>
+        </is>
+      </c>
+      <c r="AI44" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>VC-0044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>IDB Lab &amp; Circulate Capital - Ocean-Bound Plastics Initiative LAC</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>IDB Lab (Banco Interamericano de Desarrollo) y Circulate Capital</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Banca multilateral | Plataforma</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Regional - América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Plásticos ocean-bound, reciclaje, gestión de residuos, infraestructura de recolección, procesamiento, materiales innovadores</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Cofinanciación; Innovación; Escalamiento; Aceleración</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>No especificado; se menciona catalización de capital institucional a escala</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Sí; se menciona programa de desarrollo de capacidades para el Caribe combinado con la inversión</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>No especificado (anuncio de alianza, iniciativa en curso)</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/news/idb-lab-partners-circulate-capital-combat-ocean-bound-plastics</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>IDB Lab y Circulate Capital se asocian para combatir la contaminación por plásticos ocean-bound en América Latina y el Caribe, financiando principalmente startups y PyMEs en etapa temprana (Series A y B) que desarrollen soluciones escalables en economía circular de plásticos: materiales innovadores, reducción de residuos, infraestructura de gestión (recolección, clasificación, procesamiento, reciclaje, manufactura). Incluye programa de desarrollo de capacidades específico para el Caribe. La estrategia busca catalizar inversión institucional a gran escala.</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Altamente relevante: aborda directamente economía circular de plásticos, reciclaje, infraestructura de recolección, procesamiento, materiales innovadores, y reducción de residuos; alineado con REP, envases y empaques, y modelos de negocio circulares de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>Financiamiento de startups de reciclaje de plásticos flexibles; infraestructura de recolección y clasificación de envases; desarrollo de materiales alternativos o reciclados; modelos de negocio de inclusión de recicladores con tecnología; pilotos de economía circular en zonas costeras colombianas.</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>Startups o PyMEs en etapa temprana (Series A, B); soluciones escalables en economía circular de plásticos; enfoque en reducción de plásticos ocean-bound; potencial de atracción de inversión institucional</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>Startups de tecnología de reciclaje; empresas de recolección y clasificación; gremios de recicladores; universidades con I+D en materiales; organizaciones ambientales costeras; gobiernos locales de zonas costeras</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Foco en etapa temprana (Series A/B) puede excluir proyectos más maduros o en pre-semilla; no se especifica proceso de aplicación ni fechas; dependencia de criterios de Circulate Capital para inversión</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>Contactar IDB Lab Colombia y Circulate Capital para conocer proceso de postulación y criterios de inversión; identificar startups y PyMEs en ecosistema ANDI que califiquen; explorar alianza estratégica para presentar portafolio de proyectos.</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>Solicitar reunión con IDB Lab Colombia; mapear startups/PyMEs de reciclaje de plásticos en ecosistema Visión Circular; preparar pitch de cartera de proyectos elegibles.</t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de innovación y emprendimiento circular</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>Es un anuncio de alianza estratégica, no una convocatoria con fechas específicas. La iniciativa está en curso, pero no se especifica si hay ventanas de aplicación abiertas o proceso formal de postulación. Se infiere que es una iniciativa de inversión (equity o deuda) más que grant, pero orientada a economía circular. Requiere confirmar mecanismos de acceso.</t>
+        </is>
+      </c>
+      <c r="AH45" t="inlineStr">
+        <is>
+          <t>067ec89b013504b6</t>
+        </is>
+      </c>
+      <c r="AI45" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>VC-0045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme (SGP) 2.0 - CSO Challenge Program (IUCN) y Microfinance Initiative (World Bank)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) - implementado por IUCN (CSO Challenge) y World Bank (Microfinance Initiative)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Fondo ambiental | Agencia ONU | Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>25 países para CSO Challenge; 7 países específicos para Microfinance Initiative: Brasil, Colombia, Madagascar, Nigeria, Sudáfrica, Tanzania, Turquía</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Medio ambiente (biodiversidad, cambio climático, degradación de tierras, aguas internacionales, químicos)</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Iniciativas comunitarias lideradas por sociedad civil, pueblos indígenas, mujeres, jóvenes; resiliencia, acción ambiental local</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Microfinanciamiento; Innovación; Fortalecimiento institucional; Inclusión social</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>CSO Challenge: hasta USD 300,000 por iniciativa (mínimo 30 iniciativas en 25 países); Microfinance Initiative: USD 1.4 mil millones en cofinanciamiento (ratio 150:1)</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Microfinance Initiative: Sí, integrado en programas del World Bank con cofinanciamiento de 150:1. CSO Challenge: No especificado</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>GEF-8 (ciclo actual)</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>No especificado; programas en curso</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/localactionglobalimpact (menciona grants de hasta USD 75,000 para CSOs/CBOs)</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>GEF SGP 2.0 introduce dos iniciativas innovadoras complementarias: (1) CSO Challenge Program (liderado por IUCN) con grants de hasta USD 300,000 para al menos 30 iniciativas en 25 países, enfocado en apoyar directamente a OSCs, pueblos indígenas, mujeres y jóvenes; (2) Microfinance Initiative (liderado por World Bank) integrada en programas nacionales del Banco en 7 países (incluyendo Colombia), con USD 1.4 mil millones en cofinanciamiento. Ambas buscan catalizar acción local para enfrentar degradación ambiental y promover desarrollo sostenible.</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Relevancia directa para inclusión de recicladores y economía circular comunitaria: GEF SGP financia iniciativas de base comunitaria en gestión de residuos, economía circular, fortalecimiento de organizaciones de recicladores, y proyectos ambientales con enfoque de inclusión social, especialmente de mujeres y jóvenes.</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de organizaciones de recicladores de oficio; proyectos comunitarios de gestión de residuos y reciclaje; inclusión de mujeres recicladoras; innovación en reciclaje comunitario; economía circular territorial con pueblos indígenas; articulación con políticas REP desde la base.</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>CSO Challenge: OSC, CBO, con enfoque en pueblos indígenas, mujeres, jóvenes; acción ambiental local con impacto en biodiversidad, clima, tierras, aguas o químicos. Microfinance: integración en programas del World Bank Colombia (requisitos específicos por definir con el Banco)</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>Concepto de proyecto (formato GEF SGP); capacidad organizacional demostrable; enfoque de inclusión social y género; medición de impacto ambiental</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>Organizaciones de recicladores de base; asociaciones de mujeres recicladoras; comunidades indígenas con gestión territorial; ONGs ambientales locales; UNDP Colombia (implementador GEF SGP en Colombia); World Bank Colombia; alcaldías</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>CSO Challenge: No se especifica si Colombia está entre los 25 países elegibles; Microfinance Initiative: depende de ventanas del World Bank en Colombia, no es postulación directa a GEF; límite de USD 300,000 puede ser insuficiente para proyectos de mayor escala</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>Confirmar si Colombia está en los 25 países del CSO Challenge contactando a IUCN y UNDP Colombia (focal point GEF SGP); explorar con World Bank Colombia las ventanas de Microfinance Initiative; preparar portafolio de organizaciones de recicladores elegibles para grants pequeños (hasta USD 75,000).</t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>Contactar UNDP Colombia (implementador GEF SGP) para confirmar ventanas abiertas en Colombia; solicitar información sobre CSO Challenge a IUCN; mapear organizaciones de recicladores que cumplan requisitos; contactar World Bank Colombia sobre Microfinance Initiative.</t>
+        </is>
+      </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>Coordinación de inclusión social y fortalecimiento de recicladores</t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>GEF SGP tiene larga trayectoria en Colombia (ver resultado [14]: lanzamiento en 2014 con grants de hasta USD 15,000-35,000). Las dos nuevas iniciativas SGP 2.0 (CSO Challenge y Microfinance) son del ciclo GEF-8 (actual), pero no se especifica si Colombia está entre los 25 países del CSO Challenge ni las ventanas específicas de la Microfinance Initiative del WB. En Instagram se menciona hasta USD 75,000 para CSOs/CBOs, lo que sugiere ventanas activas pero requiere verificación de elegibilidad y fechas para Colombia. Microfinance Initiative no es postulación directa a GEF, sino integrada en programas del Banco Mundial.</t>
+        </is>
+      </c>
+      <c r="AH46" t="inlineStr">
+        <is>
+          <t>19f9beae7237003b</t>
+        </is>
+      </c>
+      <c r="AI46" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>VC-0046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF) - FP261: Improving Climate Resilience by Increasing Water Security in the Amazon Basin</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Colombia, Brasil, Bolivia, Ecuador, Perú, Suriname (región Amazónica)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Clima - adaptación y resiliencia</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Seguridad hídrica, manejo integrado de recursos hídricos (IWRM), infraestructura de agua, saneamiento y residuos (WSW) resiliente al clima, sistemas de alerta temprana, comunidades indígenas</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Cooperación técnica; Fortalecimiento institucional; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>USD 391 millones totales, incluyendo más de USD 160 millones de financiamiento GCF</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Sí; el programa incluye cofinanciamiento por aproximadamente USD 231 millones (391 - 160)</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>No especificado (programa aprobado, en fase de implementación)</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/project/fp261</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>https://www.agroberichtenbuitenland.nl/actueel/nieuws/2025/05/15/new-green-climate-fund-programme-in-the-amazon-basin-opens-doors-for-dutch-water-expertise</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>GCF aprobó programa regional FP261 (USD 391 millones, incluyendo USD 160 millones GCF) para mejorar resiliencia climática mediante seguridad hídrica en la cuenca Amazónica de Colombia, Brasil, Bolivia, Ecuador, Perú y Suriname. Implementado por IDB, enfoca manejo integrado de agua, infraestructura resiliente de agua, saneamiento y residuos (WSW), sistemas de alerta temprana, información hidro-climática, y apoyo a comunidades indígenas vulnerables. En fase de implementación desde mayo 2025.</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Relevancia indirecta pero estratégica: el componente de infraestructura de agua, saneamiento y residuos (WSW) resiliente al clima incluye gestión de residuos en territorios amazónicos, donde puede integrarse economía circular, reciclaje comunitario, gestión de residuos orgánicos e inorgánicos, y modelos circulares en comunidades indígenas.</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>Gestión integral de residuos en territorios amazónicos colombianos; modelos de economía circular adaptados a comunidades indígenas; infraestructura de reciclaje y compostaje resiliente al clima en la Amazonía; articulación con planes de gestión de residuos municipales en zona amazónica; inclusión de recicladores indígenas y comunidades de base.</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>Programa ya aprobado y en implementación; las oportunidades de participación serían como ejecutor, contratista o socio implementador en componentes de gestión de residuos (WSW) dentro del programa; requiere articulación con IDB (implementador) y autoridades nacionales/locales colombianas en Amazonía</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>No aplica para postulación directa (programa ya aprobado); para participar como contratista o socio: capacidad técnica en gestión de residuos, experiencia en comunidades indígenas, enfoque de género y resiliencia climática</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>IDB (implementador); autoridades ambientales de la Amazonía colombiana (CDA, Corpoamazonía); gobiernos locales amazónicos; organizaciones de pueblos indígenas; ONGs con presencia en Amazonía; Ministerio de Ambiente Colombia; universidades regionales</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>Programa ya aprobado y en implementación, no es convocatoria abierta; participación requiere articulación con IDB y autoridades, no postulación directa; foco en agua puede limitar componente de residuos; contexto amazónico (acceso, logística) es desafiante</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>Contactar IDB Colombia y unidad implementadora del programa FP261 para explorar oportunidades de participación en componente WSW (agua, saneamiento, residuos); ofrecer experticia de Visión Circular en economía circular territorial y gestión de residuos; articularse con autoridades ambientales amazónicas.</t>
+        </is>
+      </c>
+      <c r="AB47" t="inlineStr">
+        <is>
+          <t>Solicitar reunión con IDB Colombia y equipo FP261; identificar municipios amazónicos colombianos incluidos en el programa; preparar propuesta de valor de Visión Circular para componente de gestión de residuos resiliente al clima.</t>
+        </is>
+      </c>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos territoriales y economía circular amazónica</t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG47" t="inlineStr">
+        <is>
+          <t>El programa FP261 fue aprobado por GCF y está en fase de implementación desde mayo 2025 (anuncio de mayo 2025 en fuente holandesa). No es una convocatoria abierta, sino un programa aprobado implementado por IDB en 6 países amazónicos (incluyendo Colombia). La participación de Visión Circular sería como socio técnico, contratista o aliado implementador en el componente de infraestructura de agua, saneamiento y residuos (WSW), no como receptor directo de grants. El foco principal es agua y resiliencia climática; gestión de residuos es secundaria pero incluida.</t>
+        </is>
+      </c>
+      <c r="AH47" t="inlineStr">
+        <is>
+          <t>66ebdf5e202e51e9</t>
+        </is>
+      </c>
+      <c r="AI47" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>VC-0047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Euroclima - Programa de Cooperación UE-ALC en Economía Circular y Transición Energética</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Unión Europea (UE) y Gobierno Federal de Alemania</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Unión Europea y Alemania</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Cambio climático, biodiversidad, transición verde</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Economía circular, transición energética, finanzas sostenibles, gestión de residuos, aguas residuales, eficiencia de recursos, modelos de negocio sostenibles, energías renovables</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Cofinanciación; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>EUR (presumiblemente)</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>No especificado; programa de cooperación con enfoque en asistencia técnica y diálogo</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Programa en curso; Encuentro Anual realizado 24-26 marzo 2026</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Período de implementación 2026-2027 (según prioridades confirmadas en encuentro)</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>https://www.fiap.gob.es/noticias/euroclima-impulsa-la-coordinacion-regional-para-avanzar-en-la-transicion-verde-en-america-latina-y-el-caribe</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>https://www.cepal.org/es/eventos/encuentro-anual-euroclima-construyendo-ndc-la-implementacion-global-gateway</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Euroclima es programa de cooperación UE-ALC cofinanciado por UE y Alemania que fortalece acción climática y pérdida de biodiversidad mediante asistencia técnica, diálogo y coordinación regional. En su encuentro anual 2026 (Panamá, 24-26 marzo), estableció prioridades 2026-2027 en dos ejes: (1) Economía Circular (gestión residuos, aguas residuales, eficiencia de recursos, modelos de negocio sostenibles), y (2) Transición Energética (renovables, integración regional, seguridad energética), con finanzas sostenibles como tema transversal, alineado con Global Gateway UE-ALC.</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Altamente relevante: Euroclima tiene economía circular como eje estratégico central 2026-2027, incluyendo gestión de residuos, eficiencia de recursos y modelos de negocio sostenibles. Su metodología de diálogo país y asistencia técnica se alinea perfectamente con enfoque de Visión Circular ANDI en articulación institucional, REP, reciclaje y circularidad empresarial.</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Asistencia técnica para implementación de REP en Colombia; fortalecimiento de cadenas de reciclaje de envases y empaques; modelos de negocio circular empresariales; financiamiento de economía circular (finanzas sostenibles); gestión de residuos plásticos (ver iniciativa Guatemala en resultado [20]); diálogo político para economía circular territorial.</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>Alineación con prioridades de economía circular Euroclima; articulación con autoridades nacionales (Ministerio de Ambiente Colombia, DNP); enfoque en diálogo político-institucional; capacidad de cofinanciamiento o contrapartida</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>Concepto de proyecto alineado con prioridades Euroclima 2026-2027; cartas de respaldo institucional; plan de diálogo político-técnico</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>Delegación UE en Colombia; Ministerio de Ambiente; DNP; AECID Colombia; Expertise France; agencias implementadoras Euroclima (FIIAPP, GIZ, AFD); gremios empresariales; gobiernos locales</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>No se especifica proceso de postulación abierto; acceso puede requerir invitación o articulación con autoridades nacionales; foco en diálogo político puede limitar financiamiento directo a proyectos</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>Contactar Delegación UE en Colombia y AECID Colombia para conocer mecanismos de participación en Euroclima; expresar interés de ANDI/Visión Circular en diálogo de economía circular; preparar propuesta de concepto en línea con prioridades 2026-2027; participar en espacios de diálogo país.</t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>Solicitar reunión con Delegación UE Colombia y coordinación Euroclima Colombia; identificar punto focal Euroclima en Ministerio de Ambiente; preparar propuesta de diálogo/asistencia técnica en economía circular de envases.</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>Coordinación de cooperación internacional y diálogo político</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG48" t="inlineStr">
+        <is>
+          <t>Euroclima es programa de cooperación técnica, no grants directos. El resultado [20] menciona específicamente una iniciativa en Guatemala sobre economía circular y reciclaje de plásticos (cuenca Motagua) con Expertise France, lo que confirma que Euroclima financia asistencia técnica en economía circular. El resultado [21] confirma proyecto en Chile (acción climática local y economía circular) también bajo Euroclima. Encuentro Anual 2026 confirmó economía circular como prioridad 2026-2027, lo que indica ventana de oportunidad. Acceso requiere articulación institucional, no postulación directa abierta. | Fuente fuera del listado oficial conocido (fiap.gob.es): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH48" t="inlineStr">
+        <is>
+          <t>7c783a5aa29b9908</t>
+        </is>
+      </c>
+      <c r="AI48" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>VC-0048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Colombia-UK PACT - Green Finance Call for Proposals</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>UK PACT (Partnerships for Accelerating Climate Transitions)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Reino Unido</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Financiamiento climático y verde</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Finanzas verdes, adaptación de estándares climáticos en sector financiero, estructuración de proyectos verdes, NDC de Colombia</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cooperación técnica; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Hasta £500,000 por año por proyecto</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>https://www.ukpact.co.uk/colombia-country-fund-green-finance-call-for-proposals</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>https://www.ukpact.co.uk/country-programme/colombia/2021-call-for-proposals</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>UK PACT Colombia ofrece financiamiento de hasta £500,000 anuales para proyectos de desarrollo de capacidades en finanzas verdes. Busca cerrar la brecha financiera para alcanzar las metas NDC de Colombia mediante dos áreas de intervención: (1) adopción de prácticas y estándares verdes en el sector financiero, y (2) fortalecimiento de capacidades de estructuración de proyectos verdes para lograr cierre financiero.</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular porque financia estructuración de proyectos verdes y sostenibles que pueden incluir economía circular, reciclaje, envases sostenibles y modelos de negocio circulares como componentes clave de proyectos climáticos elegibles para financiamiento verde en Colombia.</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>Estructuración financiera de proyectos de economía circular para cierre de ciclo de envases; desarrollo de capacidades del sector financiero colombiano para evaluar proyectos de reciclaje inclusivo y plásticos circulares; pilotos de financiamiento verde para empresas implementando REP y ecodiseño; articulación con banca para financiar infraestructura de reciclaje.</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>Proyectos de desarrollo de capacidades alineados con las metas NDC de Colombia; enfoque en sector financiero o estructuración de proyectos verdes; articulación con contrapartes gubernamentales colombianas</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>Terms of Reference, Applicant Handbook, GEDSI guidance, Q&amp;A document (todos disponibles en la URL oficial)</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible, Superintendencia Financiera de Colombia, bancos comerciales colombianos, empresas miembro de ANDI implementando economía circular, universidades con programas de finanzas sostenibles</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>Enfoque principal en finanzas verdes puede requerir articular explícitamente economía circular como componente climático; requiere contrapartes del gobierno colombiano; competencia con otras organizaciones</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>Revisar documentos guía (ToR y Handbook) disponibles en la web; articular propuesta que posicione economía circular de envases/empaques como proyecto verde elegible para financiamiento; contactar UK PACT para confirmar vigencia y próximas ventanas</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>Descargar Terms of Reference y Applicant Handbook; verificar fechas de cierre actuales contactando UK PACT Colombia; preparar concepto de proyecto enfocado en estructuración financiera para economía circular de envases</t>
+        </is>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas de Visión Circular; área de financiamiento sostenible</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>La convocatoria está publicada en la web oficial de UK PACT pero no se especifica fecha de cierre actual. El documento menciona 'Market engagement event' y documentos Q&amp;A de octubre 2024, lo que sugiere actividad reciente. Se requiere verificación de ventanas abiertas. La pertinencia es alta si se articula economía circular como componente de finanzas verdes y NDC.</t>
+        </is>
+      </c>
+      <c r="AH49" t="inlineStr">
+        <is>
+          <t>b71c1460bf9d7f3f</t>
+        </is>
+      </c>
+      <c r="AI49" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>VC-0049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Global Innovation Fund - Open Window for Applications</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Global Innovation Fund (GIF)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Fondo multilateral</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Reino Unido (sede); operación global</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Países de ingresos bajos y medios, incluyendo Colombia y América Latina</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Innovación social con impacto en poblaciones de bajos ingresos</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Reciclaje inclusivo, formalización de recicladores, innovaciones circulares, emprendimientos con impacto social y ambiental</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Equity (capital de riesgo); Deuda; Asistencia técnica; Aceleración; Piloto demostrativo; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Variable según etapa: desde grants pequeños hasta equity de millones USD</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Variable según etapa y tipo de innovación</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Ventana permanente (rolling basis)</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Última ventana cerró 15 enero 2025; próximas fechas pendientes de anuncio</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>https://www.globalinnovation.fund/apply-for-funding</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>https://www.globalinnovation.fund</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>GIF es un fondo multilateral que invierte en innovaciones con potencial de transformar vidas en países de ingresos bajos y medios. Ofrece capital flexible (grants, equity, deuda) en diferentes etapas desde piloto hasta escalamiento. Opera con ventana abierta permanente con revisión continua de aplicaciones. Ha invertido en reciclaje inclusivo (ej. Mr. Green Africa, $1.8M con Unilever) y reduce barreras de aplicación para innovadores locales.</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: GIF ha financiado proyectos de reciclaje inclusivo que formalizan recicladores de base (Mr. Green Africa en Kenia), exactamente el modelo que Visión Circular ANDI promueve. La inclusión de recicladores, modelos circulares de negocio y reducción de residuos plásticos son áreas de interés demostrado de GIF.</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Pilotos de modelos de negocio circulares que integren recicladores de base en Colombia; plataformas tecnológicas para trazabilidad y formalización de recicladores; innovaciones en reciclaje de plásticos flexibles con inclusión social; expansión territorial de modelos exitosos de economía circular inclusiva; soluciones de ecodiseño con impacto en cadenas de reciclaje.</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>Innovación con potencial de escala y transformación; impacto demostrable en poblaciones de bajos ingresos; evidencia de modelo viable; ubicación en países de ingresos bajos y medios (Colombia califica); presentación inicial simplificada para reducir barreras</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>Aplicación inicial simplificada (disponible en sitio web); documentación completa de due diligence en etapas posteriores si pasan selección inicial</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>Organizaciones de recicladores de base (ANR Colombia), empresas productoras de envases miembro de ANDI, Latitud R, universidades para medición de impacto, gobiernos locales para escalamiento</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>Última ventana cerró enero 2025 y próximas fechas no están anunciadas aún; alta competencia global; requiere demostración clara de impacto en poblaciones vulnerables; proceso de due diligence puede ser extenso</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>Monitorear sitio web de GIF para anuncio de próxima ventana; preparar concepto de proyecto piloto de reciclaje inclusivo con métricas claras de impacto social y ambiental; identificar alianza con organización de recicladores para fortalecer componente de inclusión</t>
+        </is>
+      </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>Suscribirse a notificaciones de GIF para próximas convocatorias; revisar caso de éxito de Mr. Green Africa como referencia; preparar borrador de aplicación inicial enfocada en formalización de recicladores y cierre de ciclo de envases en Colombia</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>Coordinación de innovación y pilotos empresariales; área de inclusión social y alianzas con recicladores</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG50" t="inlineStr">
+        <is>
+          <t>GIF tiene track record comprobado en reciclaje inclusivo (Mr. Green Africa) y opera con ventana permanente, lo que es ventajoso. Colombia califica como país de ingresos medios. La última ventana cerró recientemente (enero 2025) y están revisando propuestas; próximas fechas pendientes de anuncio. La aplicación inicial es simplificada intencionalmente para reducir barreras. Alta alineación temática con Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AH50" t="inlineStr">
+        <is>
+          <t>ab5ad8550b338020</t>
+        </is>
+      </c>
+      <c r="AI50" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>VC-0050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Latitud R - Aceleradora de Negocios de Economía Circular Inclusiva</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Latitud R (plataforma liderada por BID Lab, Coca-Cola, PepsiCo, Fundación Avina, Dow, Nestlé, Red Latinoamericana de Recicladores)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Plataforma multilateral público-privada</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Regional América Latina</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>América Latina (presencia confirmada en Colombia, Brasil, México, Perú, Ecuador, Chile, Argentina)</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Economía circular y reciclaje inclusivo</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Inclusión de recicladores de base, formalización, economía circular inclusiva, fortalecimiento de cadenas de valor de reciclables, startups circulares</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Aceleración; Grant no reembolsable; Asistencia técnica; Fortalecimiento institucional; Inclusión social; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>No especificado (variable según programa: Aceleradora de Negocios vs Academia Formativa)</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>https://latitudr.org</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>https://corlab.cordoba.gob.ar/latitud-r-aceleradora-de-negocios-de-economia-circular-inclusiva</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Latitud R es la principal plataforma regional de reciclaje inclusivo en América Latina, respaldada por BID Lab y empresas líderes. Ofrece dos programas: (1) Aceleradora de Negocios para startups y emprendimientos que fortalezcan demanda de reciclables, con apoyo financiero, mentoría y red estratégica; (2) Academia Formativa para capacitación. Tiene presencia activa en Colombia y opera con modelo de colaboración intersectorial que incluye empresas, recicladores y cooperación.</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Máxima pertinencia: Latitud R fue creada específicamente para reciclaje inclusivo y economía circular en América Latina. Fundación Avina la implementa desde 2016. Alineación total con Visión Circular ANDI: inclusión de recicladores, cierre de ciclo de envases, políticas públicas REP, articulación empresas-recicladores-gobierno. Es el aliado natural de Visión Circular a nivel regional.</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>Aceleración de startups de economía circular de envases; fortalecimiento de organizaciones de recicladores en Colombia; pilotos de inclusión de recicladores en cadenas de valor empresariales; articulación para implementación de REP; proyectos territoriales de economía circular; innovación en plásticos flexibles con inclusión social.</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>Startups o emprendimientos innovadores que fortalezcan cadena de valor de reciclables; componente de inclusión social; potencial de escalamiento; alineación con economía circular</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>No especificado en las fuentes; requiere consulta directa con Latitud R</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>Fundación Avina (implementadora de Latitud R), Red Latinoamericana de Recicladores, ANR Colombia, empresas socias de Latitud R (Coca-Cola, PepsiCo, Nestlé, Dow - todas miembros de ANDI), BID Lab, CORLAB Córdoba (Argentina) como referencia de implementación local</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>No se especifican fechas de convocatoria actuales en el sitio web; puede tener ventanas específicas no continuas; requiere verificación de convocatorias abiertas o próximas</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>Contactar directamente a Fundación Avina y Latitud R Colombia para conocer convocatorias vigentes o próximas de la Aceleradora; explorar alianza estratégica formal entre Visión Circular ANDI y Latitud R para articular acciones conjuntas; participar en eventos y espacios de Latitud R</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>Contactar a Latitud R vía su sitio web o Fundación Avina Colombia para consultar estado de convocatorias; solicitar reunión para explorar colaboración ANDI-Latitud R en reciclaje inclusivo y economía circular</t>
+        </is>
+      </c>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas estratégicas y cooperación de Visión Circular; área de inclusión de recicladores</t>
+        </is>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>Latitud R es el aliado estratégico natural de Visión Circular por alineación total de misión y temática. Fundación Avina implementa Latitud R desde 2016 con presencia regional consolidada. El sitio web muestra actividad reciente (publicaciones 2026, COP30) confirmando vigencia. Sin embargo, no se especifican convocatorias abiertas actualmente en el sitio, por lo que se requiere contacto directo. El proyecto BID RG-G1037 muestra financiamiento activo hasta fecha reciente (reporte mayo 2026).</t>
+        </is>
+      </c>
+      <c r="AH51" t="inlineStr">
+        <is>
+          <t>d0fac140bf04fc41</t>
+        </is>
+      </c>
+      <c r="AI51" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-06-05
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI83"/>
+  <dimension ref="A1:AI84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15104,6 +15104,183 @@
       <c r="AI83" t="inlineStr">
         <is>
           <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>VC-0083</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Financing Circular Economy</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>GIZ</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Cooperación internacional</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Financiación de la economía circular</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>https://www.giz.de/en/downloads/giz2022-en-financing-circula-economy-colombia.pdf</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>GIZ ofrece financiación para proyectos de economía circular en Colombia. El objetivo es apoyar la implementación de la economía circular en el país.</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>Este programa se alinea con los objetivos de Visión Circular ANDI, ya que busca apoyar la implementación de la economía circular en Colombia.</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>Economía circular, financiación de proyectos, implementación de la economía circular</t>
+        </is>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>Investigar más sobre el programa y considerar la participación</t>
+        </is>
+      </c>
+      <c r="AB84" t="inlineStr">
+        <is>
+          <t>Visitar la página web oficial de GIZ para obtener más información</t>
+        </is>
+      </c>
+      <c r="AC84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE84" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF84" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG84" t="inlineStr">
+        <is>
+          <t>El programa parece estar enfocado en la financiación de proyectos de economía circular en Colombia, lo que se alinea con los objetivos de Visión Circular ANDI.</t>
+        </is>
+      </c>
+      <c r="AH84" t="inlineStr">
+        <is>
+          <t>199ae3f770ccb468</t>
+        </is>
+      </c>
+      <c r="AI84" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-07-03
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI92"/>
+  <dimension ref="A1:AI112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4837,7 +4837,7 @@
       </c>
       <c r="AI25" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -16697,6 +16697,3546 @@
       <c r="AI92" t="inlineStr">
         <is>
           <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>VC-0092</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Incentivo al Aprovechamiento y Tratamiento de Residuos Sólidos IAT 2026 - Dosquebradas</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Municipio de Dosquebradas (Risaralda, Colombia)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Gobierno</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Colombia (prioridad Dosquebradas, posiblemente Risaralda)</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Residuos sólidos</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Aprovechamiento y tratamiento de residuos, reciclaje, economía circular municipal</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cofinanciación</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Más de COP 1.400.000.000</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>2026 (año en curso, convocatoria abierta recientemente según nota)</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>https://www.dosquebradas.gov.co/web/index.php/dosquebradas/ciudad/sala-de-prensa/noticias/303-vigencia-2026/9546-dosquebradas-abre-convocatoria-por-mas-de-1-400-millones-para-transformar-el-manejo-de-residuos-en-el-municipio</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>Convocatoria municipal lanzada en 2026 por Dosquebradas con más de COP 1.400 millones para financiar proyectos de aprovechamiento, tratamiento de residuos sólidos y economía circular a nivel local. Busca transformar la gestión de residuos y fortalecer actores del reciclaje en el municipio.</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>Alineada con economía circular territorial, inclusión de recicladores y cierre de ciclo de materiales. Oportunidad para pilotos locales de Visión Circular en articulación con gobierno municipal.</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>Pilotos territoriales de reciclaje de envases; inclusión y formalización de recicladores de Dosquebradas; plantas de aprovechamiento de residuos; modelos circulares municipales; articulación empresa-municipio para cierre de ciclo.</t>
+        </is>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>Municipio de Dosquebradas, Gobernación de Risaralda, organizaciones de recicladores locales, empresas con operación en Risaralda, universidades regionales</t>
+        </is>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>Alcance geográfico limitado a Dosquebradas; requisitos y fechas de cierre no especificados en nota de prensa. Requiere consultar términos de referencia oficial.</t>
+        </is>
+      </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>Contactar Secretaría de Ambiente o Desarrollo Económico de Dosquebradas para obtener términos de referencia, requisitos, fechas de cierre y evaluar elegibilidad de actores de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB93" t="inlineStr">
+        <is>
+          <t>Solicitar términos de referencia oficiales de IAT 2026 y explorar alianza con empresas asociadas ANDI con operación en Risaralda.</t>
+        </is>
+      </c>
+      <c r="AC93" t="inlineStr">
+        <is>
+          <t>Coordinación de economía circular territorial / Alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE93" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF93" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG93" t="inlineStr">
+        <is>
+          <t>Convocatoria municipal con monto significativo. Elegibilidad para ANDI/Visión Circular depende de alcance geográfico y si permite participación de actores gremiales o solo locales. Se infiere apertura reciente por fecha 2026 en URL y tono de noticia ('puso en marcha', 'abre convocatoria'). | Fuente fuera del listado oficial conocido (dosquebradas.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH93" t="inlineStr">
+        <is>
+          <t>30690ba74d57a461</t>
+        </is>
+      </c>
+      <c r="AI93" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>VC-0093</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Greentown Labs - Subvenciones para Innovación en Reciclaje de Autopartes y Movilidad</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Greentown Labs</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Empresas de cualquier parte del mundo</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Reciclaje</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Innovación en materiales, reciclaje de autopartes, economía circular</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>25,000 (cofinanciados)</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Sí, recursos cofinanciados</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>https://administrador.nortedesantander.gov.co/wp-content/uploads/2023/01/Conv.-cooperacion-internacional-1.pdf</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>Convocatoria de Greentown Labs dirigida a empresas o startups innovadoras con materiales novedosos en eficiencia automotriz, movilidad compartida y procesos de reciclaje de autopartes. Ofrece subvenciones con cofinanciación de hasta USD $25,000.</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular por su enfoque en reciclaje de materiales (autopartes), innovación en economía circular y modelos de negocio circulares. Aplicable a pilotos empresariales con componentes de reciclaje y cierre de ciclo.</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje de materiales plásticos de autopartes; innovación en ecodiseño de componentes vehiculares reciclables; modelos de negocio circulares en sector automotriz; articulación con empresas del sector para cierre de ciclo de materiales</t>
+        </is>
+      </c>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>Empresas del sector automotriz colombiano (Renault, Sofasa, GM Colmotores), universidades con líneas de materiales e ingeniería (Universidad Nacional, Javeriana, EAFIT), centros tecnológicos, asociaciones de recicladores especializados</t>
+        </is>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>Documento de 2023, vigencia incierta; información incompleta sobre requisitos y proceso de aplicación; necesidad de validar si la convocatoria sigue activa; cofinanciación requerida puede limitar aplicabilidad</t>
+        </is>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>Verificar urgentemente vigencia de la convocatoria contactando a Greentown Labs directamente y a la Secretaría de Fronteras de Norte de Santander (secfronteras@nortedesantander.gov.co); validar términos de referencia completos y plazos actuales</t>
+        </is>
+      </c>
+      <c r="AB94" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a secfronteras@nortedesantander.gov.co y buscar sitio oficial de Greentown Labs para verificar si la convocatoria está activa en 2025</t>
+        </is>
+      </c>
+      <c r="AC94" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD94" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE94" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF94" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG94" t="inlineStr">
+        <is>
+          <t>El documento data de enero 2023 (según URL), por lo que la vigencia actual requiere verificación urgente. La información es fragmentada. Se infiere que Colombia puede aplicar dado que está publicado en sitio gubernamental colombiano. El enfoque en reciclaje de autopartes es indirecto pero aplicable a economía circular de materiales. | Fuente fuera del listado oficial conocido (administrador.nortedesantander.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH94" t="inlineStr">
+        <is>
+          <t>0e3bd2a5b01dfd32</t>
+        </is>
+      </c>
+      <c r="AI94" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>VC-0094</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Programa de Cooperación Triangular 2025 para América Latina y El Caribe</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Agencia Presidencial de Cooperación Internacional de Colombia (APC-Colombia) y socios internacionales</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Colombia (coordinador)</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>América Latina y El Caribe</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Desarrollo sostenible</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Cooperación Sur-Sur, replicabilidad de proyectos exitosos, desarrollo territorial</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Fortalecimiento institucional; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>https://www.apccolombia.gov.co/modalidades-de-cooperacion/convocatorias</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XC2u-6zWtps</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>Convocatoria 2025 del Programa de Cooperación Triangular que impulsa la replicabilidad de proyectos exitosos entre países de América Latina y el Caribe. Incluye la estrategia 'Colombia Enseña Colombia' para intercambio de experiencias regionales y promoción de desarrollo sostenible en territorios del sur global.</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>Aplicable para escalar y replicar experiencias exitosas de Visión Circular (modelos de reciclaje inclusivo, sistemas REP, economía circular territorial) hacia otros países de la región, fortaleciendo el liderazgo de ANDI/Colombia en economía circular regional.</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>Escalamiento de modelos de inclusión de recicladores a otros países de LATAM; transferencia de experiencias en implementación de REP y sistemas de envases/empaques; cooperación técnica en economía circular territorial; articulación de redes regionales de empresas por la circularidad</t>
+        </is>
+      </c>
+      <c r="W95" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>APC-Colombia como contraparte principal, otros gremios empresariales de LATAM (CPC, ANDI capítulos regionales), gobiernos locales, redes de recicladores de base (Red LACRE), universidades con presencia regional</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>Falta información detallada sobre montos, requisitos específicos y fechas límite; probable que requiera articulación institucional compleja con APC-Colombia; tiempos de gestión de cooperación triangular suelen ser extensos</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>Contactar mesa de cooperación de APC-Colombia para obtener términos de referencia específicos de la convocatoria 2025; identificar proyecto exitoso de Visión Circular susceptible de escalamiento regional; preparar perfil de proyecto demostrativo replicable</t>
+        </is>
+      </c>
+      <c r="AB95" t="inlineStr">
+        <is>
+          <t>Solicitar reunión con APC-Colombia (vía página oficial de convocatorias) para conocer alcance, plazos y requisitos exactos de la convocatoria 2025 de cooperación triangular</t>
+        </is>
+      </c>
+      <c r="AC95" t="inlineStr">
+        <is>
+          <t>Dirección ejecutiva / Coordinación de alianzas y cooperación internacional</t>
+        </is>
+      </c>
+      <c r="AD95" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE95" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF95" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG95" t="inlineStr">
+        <is>
+          <t>La convocatoria 2025 aparece mencionada en video reciente, pero no se encontró documento oficial con términos de referencia. Se infiere alta elegibilidad para organizaciones colombianas como ANDI. La pertinencia es indirecta: no financia proyectos nuevos sino que facilita cooperación técnica y escalamiento. Requiere que Visión Circular tenga casos de éxito demostrables para compartir.</t>
+        </is>
+      </c>
+      <c r="AH95" t="inlineStr">
+        <is>
+          <t>f772cc4ebe5313b3</t>
+        </is>
+      </c>
+      <c r="AI95" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>VC-0095</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator Colombia – Call for Proposals 2026</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator (liderado por UK PACT, Foreign, Commonwealth &amp; Development Office del Reino Unido, en alianza con autoridades colombianas)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Reino Unido / Colombia</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Residuos y economía circular, industria y construcción sostenible, energías renovables, transporte sostenible</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Fortalecimiento institucional; Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>2026-01 (inferido por menciones de 'convocatoria abierta 2026' en múltiples fuentes)</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>https://bogota.gov.co/boletin-oferta-internacional/climate-finance-accelerator-colombia-2026-acelera-proyectos-climatico</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>https://lanotaeconomica.com.co/movidas-empresarial/la-aceleradora-de-financiamiento-climatico-lanza-una-nueva-convocatoria-en-colombia-para-impulsar-proyectos-ambientales-de-impacto</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>La Aceleradora de Financiamiento Climático Colombia abre convocatoria 2026 para proyectos climáticos de alto impacto que buscan inversión y escalamiento hacia una economía baja en carbono. El programa ofrece acompañamiento práctico para fortalecer casos de inversión, estrategias de levantamiento de capital y relacionamiento con inversionistas. Prioriza sectores incluyendo residuos y economía circular, además de energías renovables, transporte e industria sostenible.</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>Directamente relevante para Visión Circular: uno de los sectores priorizados es 'residuos y economía circular'. Permite fortalecer proyectos de envases, reciclaje, inclusión de recicladores y modelos circulares para hacerlos atractivos a inversionistas y escalar soluciones de cierre de ciclo.</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje de plásticos flexibles con inclusión de recicladores; escalamiento de modelos de negocio circulares en envases y empaques; proyectos REP con retorno de inversión; innovación en ecodiseño con impacto climático medible; economía circular territorial con potencial de financiamiento privado o blended finance</t>
+        </is>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>Proyectos climáticos de alto impacto que contribuyan a metas nacionales de carbono; potencial de escalamiento; disposición a recibir asistencia técnica para preparación de inversión. Los proyectos deben completar solicitud en línea (criterios de selección en la web de la Aceleradora).</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>No especificado en las fuentes; probablemente incluyen: descripción del proyecto, caso de inversión preliminar, impacto climático esperado, equipo, sostenibilidad financiera</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>ANDI como articulador gremial; empresas asociadas de Visión Circular; Ministerio de Ambiente (entidad nacional involucrada); Secretaría de Ambiente de Bogotá; cooperación UK PACT; inversionistas de impacto y banca de desarrollo</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>La convocatoria no especifica fechas límite claras ni monto de apoyo; puede ser altamente competitiva; requiere preparación técnica y financiera previa; enfoque en 'preparación para inversión' implica que el proyecto debe tener potencial comercial o de sostenibilidad financiera, no solo impacto social</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>Verificar inmediatamente la web oficial de Climate Finance Accelerator Colombia para obtener términos de referencia, fechas exactas de cierre y criterios de selección. Preparar un proyecto de Visión Circular con caso de inversión preliminar en economía circular (ej. modelo de negocio circular en plásticos flexibles con inclusión y retorno financiero).</t>
+        </is>
+      </c>
+      <c r="AB96" t="inlineStr">
+        <is>
+          <t>Contactar al equipo de la Aceleradora vía web o redes (Instagram @climatefinanceacceleratorcolombia según fuente [3]) para confirmar ventana de aplicación y agendar pre-consulta. Paralelamente, identificar un proyecto piloto de Visión Circular con potencial de escalamiento y retorno de inversión para postular.</t>
+        </is>
+      </c>
+      <c r="AC96" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de Visión Circular / Oficial de alianzas y financiamiento / PROJECTABILITY área de innovación y movilización de recursos</t>
+        </is>
+      </c>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE96" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF96" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG96" t="inlineStr">
+        <is>
+          <t>Información confirmada en múltiples fuentes oficiales (Bogotá.gov.co, Cancillería, prensa). Fechas exactas no publicadas en los extractos, pero convocatoria se anuncia como 'abierta 2026'. Se infiere que está activa o próxima a abrir. Requiere verificación de plazos exactos y condiciones de elegibilidad detalladas en la web oficial de la Aceleradora (URL no proporcionada en extractos, pero mencionada en fuente [5]). | Fuente fuera del listado oficial conocido (bogota.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH96" t="inlineStr">
+        <is>
+          <t>519f99704274fbaa</t>
+        </is>
+      </c>
+      <c r="AI96" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>VC-0096</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Programa de Pequeñas Donaciones del FMAM (GEF Small Grants Programme)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Fondo para el Medio Ambiente Mundial (GEF) / PNUMA</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe, incluida Colombia</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Gestión de residuos de plástico, prácticas innovadoras de economía circular</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Donación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>No especificado en documento (típicamente hasta USD 50,000 según histórico del programa)</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/small-grants-programme</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>https://www.chathamhouse.org/sites/default/files/2021-01/2021-01-13-spanish-circular-economy-schroder-et-al.pdf</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>El Programa de Pequeñas Donaciones del FMAM financia proyectos comunitarios e innovadores que implementan prácticas de economía circular para gestión de residuos plásticos en América Latina y el Caribe. Aunque la fuente de búsqueda es de 2021, el programa opera de manera continua con convocatorias nacionales gestionadas por puntos focales en cada país.</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular, especialmente para pilotos de reciclaje de plásticos, innovación en gestión de residuos de envases y empaques, e inclusión de recicladores de base comunitaria en modelos circulares.</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje de plásticos flexibles con inclusión de recicladores; innovación en cierre de ciclo de envases; fortalecimiento de organizaciones de recicladores; modelos territoriales de economía circular</t>
+        </is>
+      </c>
+      <c r="W97" t="inlineStr">
+        <is>
+          <t>Organizaciones comunitarias, ONGs, cooperativas; proyectos de pequeña escala con impacto ambiental y social demostrable; enfoque participativo</t>
+        </is>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto, presupuesto detallado, cartas de apoyo comunitario, plan de sostenibilidad (requisitos específicos varían por país)</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>Organizaciones de recicladores, cooperativas, ONGs ambientales locales, gobiernos municipales, empresas ANDI para cofinanciación o apoyo técnico</t>
+        </is>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>Techo de financiamiento limitado; proceso competitivo; puede requerir contraparte local comunitaria como beneficiario directo (ANDI actuaría como aliado técnico)</t>
+        </is>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>Contactar al punto focal nacional del GEF SGP en Colombia (usualmente operado por PNUD Colombia) para verificar ventanas abiertas o próximas convocatorias 2025. Identificar organizaciones de recicladores como socios aplicantes con ANDI/Visión Circular como aliado técnico.</t>
+        </is>
+      </c>
+      <c r="AB97" t="inlineStr">
+        <is>
+          <t>Contactar PNUD Colombia o punto focal GEF SGP Colombia para conocer estado de convocatorias 2025 y requisitos actuales</t>
+        </is>
+      </c>
+      <c r="AC97" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas territoriales de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AD97" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE97" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF97" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG97" t="inlineStr">
+        <is>
+          <t>Documento fuente es de 2021, pero el Programa de Pequeñas Donaciones del GEF es permanente con convocatorias regulares. Requiere verificar convocatorias actuales en Colombia. La elegibilidad directa de gremios puede ser limitada, pero pueden participar como socios técnicos de organizaciones comunitarias.</t>
+        </is>
+      </c>
+      <c r="AH97" t="inlineStr">
+        <is>
+          <t>54533eae40a8d9d5</t>
+        </is>
+      </c>
+      <c r="AI97" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>VC-0097</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Garantías para Economía Circular - CAF Banco de Desarrollo de América Latina</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>CAF - Banco de Desarrollo de América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (sede en Caracas/Panamá)</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Países miembros de CAF, incluida Colombia</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Inversión privada en iniciativas de economía circular, gestión de residuos, reciclaje</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Otro (garantías)</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>Sí, inversión privada requerida</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>https://www.caf.com</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>https://www.giz.de/en/downloads/giz2024-es-guia-para-el-financiamiento-EC-RD.pdf</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>CAF ofrece instrumentos de garantía para reducir riesgos en inversiones privadas de economía circular. No es financiamiento directo sino mitigación de riesgo que facilita acceso a crédito bancario comercial para proyectos circulares. Aplicable a empresas de diversos tamaños para inversión de capital u operativa en iniciativas de economía circular.</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>Relevante para empresas miembro de ANDI que requieren financiamiento para infraestructura de reciclaje, plantas de procesamiento de residuos de envases, inversiones en ecodiseño o ampliación de capacidad de recolección y procesamiento en el marco de cumplimiento REP.</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>Inversión en infraestructura de reciclaje de envases y empaques; plantas de clasificación y procesamiento; tecnología de reciclaje químico de plásticos flexibles; modelos de negocio de reuso y retorno de envases; infraestructura de logística inversa</t>
+        </is>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>Empresas con proyectos de economía circular que requieren financiamiento bancario; viabilidad financiera demostrable; proyecto alineado con principios de economía circular; capacidad de cofinanciación</t>
+        </is>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>Plan de negocios del proyecto circular, proyecciones financieras, análisis de impacto ambiental, documentación corporativa, garantías complementarias</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>Bancos comerciales colombianos, empresas ANDI con proyectos de inversión circular, gremios para agregación de proyectos</t>
+        </is>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>Requiere capacidad de endeudamiento de la empresa; las garantías no eliminan totalmente el costo financiero; proceso puede ser extenso; requiere proyecto estructurado con viabilidad financiera clara</t>
+        </is>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>Identificar empresas ANDI con proyectos de inversión circular que requieren financiamiento (ej. plantas de reciclaje, infraestructura REP). Realizar sesión informativa con CAF Colombia para entender condiciones y proceso de garantías. Priorizar proyectos de mayor escala y madurez financiera.</t>
+        </is>
+      </c>
+      <c r="AB98" t="inlineStr">
+        <is>
+          <t>Contactar oficina CAF Colombia para agendar sesión sobre instrumentos de garantía para proyectos de economía circular de empresas ANDI</t>
+        </is>
+      </c>
+      <c r="AC98" t="inlineStr">
+        <is>
+          <t>Dirección de Visión Circular ANDI y área de relacionamiento financiero</t>
+        </is>
+      </c>
+      <c r="AD98" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE98" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF98" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG98" t="inlineStr">
+        <is>
+          <t>No es grant sino instrumento de garantía que facilita acceso a crédito. Más apropiado para empresas grandes o medianas con capacidad de endeudamiento. La fuente (GIZ 2024) es reciente y confiable. CAF tiene oficina activa en Colombia.</t>
+        </is>
+      </c>
+      <c r="AH98" t="inlineStr">
+        <is>
+          <t>d3cefea50c1b7e4f</t>
+        </is>
+      </c>
+      <c r="AI98" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>VC-0098</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Financiamiento BID Invest para Economía Circular</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>BID Invest (Grupo Banco Interamericano de Desarrollo)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Internacional (América Latina y el Caribe)</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe, incluida Colombia</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Reciclaje de plásticos, gestión de residuos, empresas circulares</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Cofinanciación; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>No especificado (varía según proyecto, típicamente desde USD 5 millones)</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>Sí, inversión privada requerida</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>https://idbinvest.org</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>https://idbinvest.org/es/blog/transporte/liberando-la-economia-circular-en-america-latina-y-el-caribe</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>BID Invest financia empresas privadas del sector de economía circular en ALC, incluyendo reciclaje de plásticos y gestión de residuos. Ofrece préstamos, equity y asistencia técnica para empresas en crecimiento o consolidación. Enfoque en proyectos escalables con retorno financiero y alto impacto ambiental y social.</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>Relevante para empresas de reciclaje asociadas a ANDI o para agregar proyectos empresariales de economía circular que requieren inversión para escalar. Particularmente útil para empresas de reciclaje de envases y empaques plásticos que buscan expandir capacidad.</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>Escalamiento de empresas de reciclaje de plásticos (incluidos flexibles); plantas de producción de resinas recicladas; infraestructura de recolección y clasificación; empresas de valorización de residuos de envases; modelos B2B de gestión circular de empaques</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>Empresas privadas con modelo de negocio probado; viabilidad financiera; potencial de escalamiento; impacto ambiental y social cuantificable; capacidad de gestión empresarial; generalmente proyectos desde USD 5 millones</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>Business plan detallado, estados financieros auditados, proyecciones financieras, análisis de mercado, due diligence ambiental y social, estructura de gobernanza</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>Empresas ANDI del sector de reciclaje o gestión de residuos, inversionistas privados, fondos de impacto, empresas productoras de envases interesadas en abastecimiento de material reciclado</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>Proceso de evaluación extenso (6-12 meses); montos mínimos relativamente altos; requiere madurez empresarial y financiera; enfoque en empresas más que en programas gremiales; costo de capital aunque concesional</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>Mapear empresas de reciclaje dentro o vinculadas al ecosistema ANDI con potencial de escalamiento. Facilitar contacto con BID Invest para explorar financiamiento. Considerar agregación de empresas medianas si proyectos individuales están bajo montos mínimos.</t>
+        </is>
+      </c>
+      <c r="AB99" t="inlineStr">
+        <is>
+          <t>Identificar 2-3 empresas candidatas del sector reciclaje de envases/empaques con proyectos de expansión. Contactar BID Invest Colombia para sesión exploratoria</t>
+        </is>
+      </c>
+      <c r="AC99" t="inlineStr">
+        <is>
+          <t>Dirección de Visión Circular y área de desarrollo empresarial ANDI</t>
+        </is>
+      </c>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF99" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG99" t="inlineStr">
+        <is>
+          <t>La fuente menciona ejemplo de financiamiento a empresa de reciclaje (Plastech en Haití). BID Invest opera continuamente pero con enfoque en empresas maduras. ANDI actuaría más como facilitador que como aplicante directo. Montos típicamente para empresas medianas-grandes.</t>
+        </is>
+      </c>
+      <c r="AH99" t="inlineStr">
+        <is>
+          <t>8bd66039cd3c8b18</t>
+        </is>
+      </c>
+      <c r="AI99" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>VC-0099</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Convocatoria regional para soluciones innovadoras en plásticos - Colombia, Chile y México</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Pacto Global Red Colombia (en alianza con otros actores regionales)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Colombia (regional)</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Colombia, Chile y México</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Plásticos, Innovación en envases y empaques, Reciclaje</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Aceleración; Innovación</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Hasta 10.000 por solución seleccionada</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>https://www.pactoglobal-colombia.org/news/convocatoria-regional-otorgara-hasta-usd-10-000-a-soluciones-innovadoras-en-plasticos-en-colombia-chile-y-mexico.html</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>Convocatoria regional que otorga hasta USD 10.000 a soluciones innovadoras en plásticos en Colombia, Chile y México. Los recursos se destinan a acelerar el desarrollo de soluciones y su preparación para el mercado. Se seleccionará una solución por cada desafío crítico identificado en el programa.</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI por su enfoque en innovación de soluciones para plásticos, envases y empaques, y su alineación directa con los pilares de economía circular, reciclabilidad y modelos de negocio circulares que impulsa el programa.</t>
+        </is>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>Desarrollo de soluciones innovadoras para plásticos flexibles; Modelos de negocio circulares para envases; Pilotos demostrativos de reciclabilidad mejorada; Ecodiseño de empaques plásticos; Tecnologías de cierre de ciclo para envases</t>
+        </is>
+      </c>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t>Las soluciones deben enfocarse en desafíos críticos de innovación en plásticos (los desafíos específicos no están detallados en el extracto)</t>
+        </is>
+      </c>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>Empresas afiliadas a ANDI del sector de empaques, universidades con líneas de investigación en materiales, centros tecnológicos, Pacto Global Red Colombia, empresas de reciclaje</t>
+        </is>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>Fechas de apertura y cierre no especificadas en la fuente; Requisitos de elegibilidad y desafíos específicos no detallados completamente; Monto limitado (USD 10.000) puede ser insuficiente para proyectos de gran escala</t>
+        </is>
+      </c>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente al Pacto Global Red Colombia para verificar estado de la convocatoria, fechas exactas, requisitos completos y desafíos específicos. Preparar portafolio de soluciones innovadoras de empresas asociadas a Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB100" t="inlineStr">
+        <is>
+          <t>Consultar con Pacto Global Red Colombia el estado actual de la convocatoria y solicitar bases completas. Identificar 2-3 soluciones innovadoras en desarrollo dentro del ecosistema Visión Circular que puedan aplicar.</t>
+        </is>
+      </c>
+      <c r="AC100" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos en alianza con área de Innovación</t>
+        </is>
+      </c>
+      <c r="AD100" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE100" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF100" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG100" t="inlineStr">
+        <is>
+          <t>La fuente es oficial del Pacto Global Red Colombia, pero no especifica fechas de apertura ni cierre. Es necesario verificar vigencia actual. El monto es relativamente pequeño pero puede ser estratégico para validación de conceptos o pilotos. Colombia es explícitamente elegible. | Fuente fuera del listado oficial conocido (pactoglobal-colombia.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH100" t="inlineStr">
+        <is>
+          <t>dc4cadd625c2b50a</t>
+        </is>
+      </c>
+      <c r="AI100" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>VC-0100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Convocatoria Acercar para sostenibilidad empresarial</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>No especificado en el extracto</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Colombia (inferido por fuente colombiana)</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Colombia (inferido)</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Sostenibilidad empresarial, posiblemente economía circular en empaques</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>No especificado (posiblemente Grant no reembolsable o Cofinanciación)</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>https://www.ekologypack.com.co/blog-de-ekologypack-innovacion-ecologica-en-empaques</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>Convocatoria Acercar mencionada en el blog de EkologyPack como oportunidad para la sostenibilidad empresarial. La información disponible es limitada; aparece como título de entrada de blog pero sin detalles sobre entidad financiadora, montos, fechas o requisitos específicos.</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>Potencialmente relevante si está enfocada en sostenibilidad empresarial relacionada con empaques y envases, dado que es mencionada por EkologyPack, empresa del sector. Sin embargo, la falta de información impide evaluar la alineación precisa con Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>Sostenibilidad empresarial en envases y empaques; Economía circular empresarial; Responsabilidad Extendida del Productor; Modelos de negocio sostenibles</t>
+        </is>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>Empresas del sector de empaques, gremios empresariales, ANDI</t>
+        </is>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>Información extremadamente limitada; no se puede verificar vigencia, elegibilidad ni alineación temática precisa; la fuente es un blog corporativo, no una fuente oficial de convocatoria</t>
+        </is>
+      </c>
+      <c r="AA101" t="inlineStr">
+        <is>
+          <t>Acceder al artículo completo en el blog de EkologyPack para obtener información detallada. Buscar información oficial sobre la Convocatoria Acercar en fuentes gubernamentales o de cooperación.</t>
+        </is>
+      </c>
+      <c r="AB101" t="inlineStr">
+        <is>
+          <t>Investigar y leer el artículo completo en el blog de EkologyPack. Realizar búsqueda complementaria sobre 'Convocatoria Acercar Colombia sostenibilidad' en fuentes oficiales.</t>
+        </is>
+      </c>
+      <c r="AC101" t="inlineStr">
+        <is>
+          <t>Área de inteligencia de oportunidades o Coordinación de proyectos</t>
+        </is>
+      </c>
+      <c r="AD101" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE101" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF101" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG101" t="inlineStr">
+        <is>
+          <t>Información muy limitada en el extracto proporcionado. Solo aparece como título de entrada de blog sin desarrollo. La fuente (EkologyPack) es una empresa colombiana de empaques ecológicos, lo que sugiere pertinencia temática, pero no es una fuente oficial de convocatoria. Se requiere investigación adicional urgente para determinar si es una oportunidad real y vigente. | Fuente fuera del listado oficial conocido (ekologypack.com.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH101" t="inlineStr">
+        <is>
+          <t>07d0b4493a2ee54b</t>
+        </is>
+      </c>
+      <c r="AI101" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>VC-0101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia Innovation Challenge - Agrichallenge</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>AgriTech Challenge (organizador principal no especificado en la fuente)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Internacional / Colombia</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Colombia (prioridad explícita)</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Sector agroindustrial, transición circular, innovación</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Aceleración; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>Challenge de innovación enfocado en acelerar la transición hacia una economía circular en el sector agroalimentario de Colombia, alineado con el Plan Nacional de Desarrollo 2022-2026 y los objetivos de la COP 16 CBD Colombia. Ofrece acceso a mentoría experta y apoyo integral para soluciones circulares en agroindustria.</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>Aunque enfocado en agroindustria, es altamente relevante porque aborda economía circular territorial y modelos de negocio circulares en Colombia. Los envases y empaques de productos agrícolas son una línea de trabajo potencial para Visión Circular, además de posibles sinergias en inclusión y cierre de ciclo.</t>
+        </is>
+      </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>Ecodiseño de empaques para productos agrícolas; modelos circulares de gestión de envases en cadenas agroalimentarias; pilotos de reciclabilidad de empaques agroindustriales; articulación con empresas del sector alimentario para REP; economía circular territorial en zonas rurales con inclusión de recicladores</t>
+        </is>
+      </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>Empresas agroindustriales asociadas a ANDI, universidades con líneas en agroindustria y sostenibilidad, cooperativas de recicladores en zonas rurales, centros tecnológicos en innovación alimentaria</t>
+        </is>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>Información muy limitada en la fuente: no se especifican plazos, montos, requisitos de elegibilidad ni proceso de aplicación. El enfoque agroalimentario puede no ser el núcleo directo de Visión Circular, que prioriza envases y empaques en general.</t>
+        </is>
+      </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>Verificar urgentemente vigencia, plazos y condiciones de participación contactando directamente a los organizadores. Evaluar si el alcance incluye envases/empaques de productos agrícolas o solo procesos productivos agroindustriales.</t>
+        </is>
+      </c>
+      <c r="AB102" t="inlineStr">
+        <is>
+          <t>Contactar vía web oficial para solicitar términos de referencia, fechas límite y confirmar elegibilidad de proyectos enfocados en envases/empaques del sector agroalimentario</t>
+        </is>
+      </c>
+      <c r="AC102" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD102" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE102" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF102" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG102" t="inlineStr">
+        <is>
+          <t>La fuente web no proporciona información detallada sobre fechas, montos, requisitos ni proceso de aplicación. Se infiere que el challenge está activo por el uso de lenguaje presente ('aims to accelerate'), pero no hay confirmación explícita de plazos. La pertinencia para Visión Circular es indirecta pero aprovechable si incluye la dimensión de envases/empaques agroindustriales. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH102" t="inlineStr">
+        <is>
+          <t>56c48fc756143452</t>
+        </is>
+      </c>
+      <c r="AI102" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>VC-0102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator Colombia - 2026 cohort</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator (CFA)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Reino Unido (operación global)</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Financiamiento climático, proyectos sostenibles</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>https://www.climatefinanceaccelerator.com/countries/colombia</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>El Climate Finance Accelerator Colombia está conformando su cohorte 2026, habiendo seleccionado 10 proyectos de 238 aplicaciones en sectores AFOLU, renovables y otros relacionados con clima. El programa ofrece aceleración y asistencia técnica para conectar proyectos con financiamiento climático.</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>Visión Circular puede presentar proyectos de economía circular con impacto climático (reducción de emisiones por reciclaje, cierre de ciclo de envases, modelos circulares) que califiquen para aceleración y acceso a financiamiento climático internacional.</t>
+        </is>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje de plásticos flexibles con reducción de huella de carbono; modelos de negocio circulares territoriales con inclusión de recicladores; proyectos de ecodiseño con impacto climático cuantificable; infraestructura de economía circular REP</t>
+        </is>
+      </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t>Proyecto con impacto climático demostrable; aplicación a proceso competitivo (238 aplicaciones históricas, 10 seleccionadas); alineación con sectores priorizados</t>
+        </is>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>Empresas miembro de ANDI con proyectos climáticos circulares; centros tecnológicos para cuantificación de impacto; cooperativas de recicladores para componente social</t>
+        </is>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>Alta competitividad (4% tasa de selección histórica); no se especifica si convocatoria 2026 está abierta o cerrada; falta claridad sobre criterios específicos y montos</t>
+        </is>
+      </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>Contactar directamente a CFA Colombia para confirmar estado de convocatoria 2026, fechas y requisitos específicos; preparar perfil de proyecto circular con métricas de impacto climático</t>
+        </is>
+      </c>
+      <c r="AB103" t="inlineStr">
+        <is>
+          <t>Enviar consulta formal a CFA vía sitio web solicitando información sobre ventana de aplicación 2026 y elegibilidad de proyectos de economía circular</t>
+        </is>
+      </c>
+      <c r="AC103" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y movilización de recursos</t>
+        </is>
+      </c>
+      <c r="AD103" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE103" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF103" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG103" t="inlineStr">
+        <is>
+          <t>La fuente menciona cohorte 2026 pero no especifica si la convocatoria está abierta, cerrada o próxima a abrir. Se infiere que podría estar en proceso de conformación. Requiere verificación urgente de estado y fechas. La pertinencia es buena si aceptan proyectos de economía circular bajo el paraguas climático. | Fuente fuera del listado oficial conocido (climatefinanceaccelerator.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH103" t="inlineStr">
+        <is>
+          <t>91260acf133bdc92</t>
+        </is>
+      </c>
+      <c r="AI103" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>VC-0103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Plastics Innovation Programme 2026</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>UNDP - UN Peace and Development Fund (UNPDF) con contribuciones del Gobierno de China y UN DESA</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Agencia ONU</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Residuos plásticos y economía circular</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Reducción de generación de residuos plásticos, alternativas sostenibles, innovación</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>2026 (año referencia, fecha exacta no especificada)</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/vietnam/news/call-proposals-plastics-innovation-programme-2026</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>Convocatoria del PNUD financiada por el Fondo de Paz y Desarrollo de la ONU con contribuciones de China y UN DESA, orientada a pilotar y promover iniciativas que reduzcan la generación de residuos plásticos y fomenten producción de alternativas sostenibles. La convocatoria 2026 busca soluciones innovadoras alineadas con los ODS y la Agenda 2030.</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI por su enfoque en residuos plásticos, innovación en alternativas sostenibles, reducción de generación de residuos y economía circular, todos pilares del programa. Aplica directamente a las líneas de envases/empaques y cierre de ciclo.</t>
+        </is>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>Pilotos de reducción de plásticos flexibles; innovación en empaques sostenibles alternativos; modelos de negocio circulares para envases; escalamiento de tecnologías de reciclaje; proyectos demostrativos de ecodiseño con empresas ANDI</t>
+        </is>
+      </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>PNUD Colombia, empresas asociadas ANDI (productoras de envases), universidades con líneas de innovación en materiales, centros tecnológicos, cooperación bilateral China-Colombia</t>
+        </is>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>Elegibilidad geográfica no confirmada explícitamente para Colombia; la noticia proviene de UNDP Vietnam lo que genera incertidumbre sobre alcance regional; fecha de cierre exacta no disponible</t>
+        </is>
+      </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>Contactar urgentemente a UNDP Colombia y UNDP Regional LAC para confirmar elegibilidad, plazos y requisitos específicos para América Latina. Preparar portafolio de casos de negocio circular del programa Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB104" t="inlineStr">
+        <is>
+          <t>Escribir a UNDP Colombia (mailto contacto) y consultar el portal global de UNDP sobre esta convocatoria. Solicitar Terms of Reference y criterios de elegibilidad geográfica.</t>
+        </is>
+      </c>
+      <c r="AC104" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas internacionales de Visión Circular / PROJECTABILITY</t>
+        </is>
+      </c>
+      <c r="AD104" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE104" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF104" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG104" t="inlineStr">
+        <is>
+          <t>La fuente es UNDP Vietnam, lo que genera incertidumbre sobre si la convocatoria es global o regional Asia-Pacífico. Sin embargo, el UNPDF suele tener alcance global. La fecha 2026 sugiere que puede estar aún en diseño o próxima a abrir. Se requiere verificación urgente de elegibilidad para Colombia/LAC.</t>
+        </is>
+      </c>
+      <c r="AH104" t="inlineStr">
+        <is>
+          <t>815b4de3fd3852bc</t>
+        </is>
+      </c>
+      <c r="AI104" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>VC-0104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ISC3 Innovation Challenge 2026 - Sustainable Chemistry and Electronics</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>ISC3 - International Sustainable Chemistry Collaborative Centre</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Global (no se especifican restricciones geográficas explícitas)</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Química sostenible y Electrónica</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Innovación en química sostenible aplicable a envases, empaques y economía circular</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Aceleración; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>Junio 2026 (anuncio de finalistas)</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>https://www.isc3.org/page/innovation-challenge</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>El ISC3 Innovation Challenge 2026 se enfoca en química sostenible y electrónica. Las aplicaciones elegibles son evaluadas por un jurado internacional de expertos. Los finalistas (anunciados a finales de junio 2026) reciben apoyo personalizado del ISC3 Global Start-up Service, capacitación en pitch y visibilidad adicional.</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>La química sostenible es clave para ecodiseño, reciclabilidad y desarrollo de materiales alternativos en envases y empaques. Puede apoyar innovaciones en formulaciones de plásticos más circulares y soluciones de cierre de ciclo.</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>Innovaciones en química verde para envases reciclables; desarrollo de materiales bio-basados o compostables para empaques; soluciones de ecodiseño químico para plásticos flexibles; tecnologías de reciclaje químico aplicadas a envases multicapa</t>
+        </is>
+      </c>
+      <c r="W105" t="inlineStr">
+        <is>
+          <t>Aplicaciones elegibles evaluadas por jurado de expertos; enfoque en química sostenible y electrónica; No especificado requisitos detallados</t>
+        </is>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>Empresas de química y materiales asociadas a ANDI; universidades con líneas de investigación en química verde (Andes, Nacional, EAFIT); centros tecnológicos como CIDET o ICIPC; start-ups de innovación en materiales</t>
+        </is>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>Falta información sobre monto del premio, criterios de elegibilidad específicos y si Colombia es explícitamente elegible; fecha de apertura de convocatoria no especificada; puede requerir capacidad de innovación química avanzada</t>
+        </is>
+      </c>
+      <c r="AA105" t="inlineStr">
+        <is>
+          <t>Verificar en la página oficial de ISC3 si la convocatoria 2026 está abierta o próxima a abrir, confirmar elegibilidad para Colombia/América Latina, y revisar términos de referencia completos incluyendo montos y requisitos</t>
+        </is>
+      </c>
+      <c r="AB105" t="inlineStr">
+        <is>
+          <t>Visitar https://www.isc3.org/page/innovation-challenge y contactar directamente a ISC3 para confirmar fechas de apertura 2026, elegibilidad regional y requisitos específicos</t>
+        </is>
+      </c>
+      <c r="AC105" t="inlineStr">
+        <is>
+          <t>Coordinación de innovación y alianzas tecnológicas</t>
+        </is>
+      </c>
+      <c r="AD105" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE105" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF105" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG105" t="inlineStr">
+        <is>
+          <t>La información disponible es limitada. Se infiere que es global pero no hay confirmación explícita de elegibilidad para Colombia. El enfoque en química sostenible es pertinente pero menos directo que un programa específico de economía circular de envases. Fecha de cierre es para anuncio de finalistas, no para aplicación. | Fuente fuera del listado oficial conocido (isc3.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH105" t="inlineStr">
+        <is>
+          <t>499b6ce1d934f8e7</t>
+        </is>
+      </c>
+      <c r="AI105" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>VC-0105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Waste Reduction and Circular Economy Development Grants Programme</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>UNDP (United Nations Development Programme)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Agencia ONU</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>No especificado en fragmento (requiere verificación en URL oficial)</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Reducción de residuos, Desarrollo de economía circular</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/georgia/news/circular-economy-call-for-proposals</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>Programa de grants del PNUD para reducción de residuos y desarrollo de economía circular. Aunque la URL refiere a Georgia, el fragmento menciona presencia en América Latina y el Caribe, sugiriendo posible elegibilidad regional. Requiere verificación urgente de términos específicos, fechas y países elegibles en la fuente oficial.</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular por su enfoque directo en economía circular y gestión de residuos, alineado con cierre de ciclo, reciclaje y modelos circulares territoriales que desarrolla el programa ANDI.</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>Pilotos de economía circular territorial; modelos de negocio circulares con inclusión de recicladores; sistemas de gestión de residuos de envases y empaques; proyectos de cierre de ciclo con articulación público-privada</t>
+        </is>
+      </c>
+      <c r="W106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>Municipios colombianos, organizaciones de recicladores de base, universidades con líneas ambientales, empresas miembro de ANDI con compromisos REP, autoridades ambientales regionales</t>
+        </is>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>Incertidumbre sobre elegibilidad específica de Colombia; posible limitación geográfica a países específicos del PNUD; fechas de convocatoria no confirmadas</t>
+        </is>
+      </c>
+      <c r="AA106" t="inlineStr">
+        <is>
+          <t>Verificar inmediatamente en la URL oficial si Colombia está dentro de países elegibles y si la convocatoria está abierta o tiene fechas próximas. Contactar oficina PNUD Colombia para confirmar.</t>
+        </is>
+      </c>
+      <c r="AB106" t="inlineStr">
+        <is>
+          <t>Revisar términos de referencia completos en URL oficial y contactar punto focal PNUD Colombia en las próximas 48 horas</t>
+        </is>
+      </c>
+      <c r="AC106" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Alianzas institucionales</t>
+        </is>
+      </c>
+      <c r="AD106" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE106" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF106" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG106" t="inlineStr">
+        <is>
+          <t>La URL refiere a Georgia pero el menú del sitio incluye 'Latin America and the Caribbean', lo que sugiere presencia regional del programa. La elegibilidad de Colombia es inferida pero no confirmada en el fragmento proporcionado.</t>
+        </is>
+      </c>
+      <c r="AH106" t="inlineStr">
+        <is>
+          <t>56c1d364dd3da8ca</t>
+        </is>
+      </c>
+      <c r="AI106" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>VC-0106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Too Good to Waste Initiative</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>BID (Banco Interamericano de Desarrollo)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (Colombia elegible)</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Residuos</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Mitigación de metano, Resiliencia, Economía circular en gestión de residuos</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Financiamiento concesional; Estructuración de proyectos</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/who-we-are/topics/water-and-sanitation/initiatives/too-good-waste</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>Iniciativa del BID que estructura proyectos y promueve condiciones habilitantes para mitigación de metano, resiliencia y adopción de economía circular en el sector de gestión de residuos. Ofrece asistencia técnica y estructuración financiera para proyectos regionales. No es convocatoria con fecha límite sino ventanilla permanente de cooperación.</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular por su enfoque en economía circular del sector residuos, especialmente en cierre de ciclo de envases/empaques, gestión de residuos post-consumo y potencial articulación con compromisos REP de empresas.</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>Estructuración de proyectos de valorización de residuos de envases; sistemas de recolección selectiva con inclusión de recicladores; infraestructura para cierre de ciclo de empaques; proyectos de mitigación climática mediante reciclaje; modelos público-privados de economía circular territorial</t>
+        </is>
+      </c>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>Gobiernos locales y regionales colombianos, empresas productoras de envases (miembros ANDI), gremios de la cadena de reciclaje, centros tecnológicos, autoridades ambientales, sistemas colectivos de gestión REP</t>
+        </is>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>No es financiación directa tipo grant sino estructuración de proyectos que luego requieren financiamiento; tiempos de desarrollo de proyecto pueden ser largos; requiere alineación con prioridades estratégicas del BID</t>
+        </is>
+      </c>
+      <c r="AA107" t="inlineStr">
+        <is>
+          <t>Explorar oportunidades de estructuración de proyectos piloto de economía circular con empresas ANDI que necesiten cumplir metas REP, especialmente en plásticos flexibles y empaques complejos</t>
+        </is>
+      </c>
+      <c r="AB107" t="inlineStr">
+        <is>
+          <t>Contactar División de Agua y Saneamiento del BID Colombia para agendar reunión exploratoria sobre alineación de Visión Circular con la iniciativa</t>
+        </is>
+      </c>
+      <c r="AC107" t="inlineStr">
+        <is>
+          <t>Alianzas institucionales / Desarrollo de negocios</t>
+        </is>
+      </c>
+      <c r="AD107" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE107" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF107" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG107" t="inlineStr">
+        <is>
+          <t>Es una iniciativa paraguas del BID, no una convocatoria puntual. Ofrece asistencia técnica y estructuración pero no necesariamente grants directos no reembolsables. La ventaja es que Colombia es país miembro elegible del BID y hay presencia activa en el país.</t>
+        </is>
+      </c>
+      <c r="AH107" t="inlineStr">
+        <is>
+          <t>6b28c50f5d23a936</t>
+        </is>
+      </c>
+      <c r="AI107" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>VC-0107</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Sustainable Small Grants Programme (SSGP) - Closing the Caribbean Plastic Tap Initiative</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>UICN (Unión Internacional para la Conservación de la Naturaleza) - México, América Central y el Caribe</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>ONG</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Regional - América Central y el Caribe</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Caribe Oriental (Eastern Caribbean) - potencialmente extensible a América Latina</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Residuos y economía circular</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Plásticos, gestión de residuos, reducción de contaminación plástica</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Piloto demostrativo; Inclusión social</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>2024-04-30</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/uicnormacc/posts/applications-are-now-open-for-the-sustainable-small-grants-programme-implemented/1398932268933455</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>El Programa de Pequeñas Donaciones Sostenibles (SSGP) de la UICN, implementado bajo la iniciativa 'Closing the Caribbean Plastic Tap', apoya proyectos prácticos liderados localmente que reducen la contaminación plástica y mejoran la gestión de residuos en el Caribe Oriental. Las aplicaciones se abrieron el 30 de abril de 2024.</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular por su enfoque en reducción de plásticos, gestión de residuos y soluciones prácticas locales. Aunque el enfoque geográfico principal es el Caribe, podría explorarse elegibilidad para Colombia por la cobertura regional de UICN Mesoamérica.</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>Pilotos de reducción de contaminación plástica; sistemas de gestión de residuos comunitarios; inclusión de recicladores en cadenas de valor; innovación en reciclaje de plásticos flexibles; modelos de economía circular territorial en zonas costeras colombianas.</t>
+        </is>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>Proyectos prácticos, liderazgo local, enfoque en reducción de plásticos y mejora de gestión de residuos</t>
+        </is>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>UICN Colombia, municipios costeros, cooperativas de recicladores, empresas de la región Caribe colombiana, universidades locales</t>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>Enfoque geográfico limitado al Caribe Oriental; incertidumbre sobre elegibilidad de Colombia; fecha de cierre no especificada puede indicar cierre inminente</t>
+        </is>
+      </c>
+      <c r="AA108" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a UICN Mesoamérica para confirmar elegibilidad de Colombia (especialmente región Caribe colombiana) y fecha límite exacta de aplicación</t>
+        </is>
+      </c>
+      <c r="AB108" t="inlineStr">
+        <is>
+          <t>Enviar correo a UICN México, América Central y el Caribe solicitando términos de referencia completos y confirmación de elegibilidad para Colombia</t>
+        </is>
+      </c>
+      <c r="AC108" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Alianzas internacionales</t>
+        </is>
+      </c>
+      <c r="AD108" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE108" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF108" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG108" t="inlineStr">
+        <is>
+          <t>La fecha de publicación (30 abril) sugiere que la convocatoria podría estar activa, pero la falta de fecha de cierre y la fuente Facebook (no sitio oficial) requiere verificación urgente. La elegibilidad para Colombia es incierta pero posible dado que UICN opera en la región y Colombia tiene costa caribeña. | Fuente fuera del listado oficial conocido (facebook.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH108" t="inlineStr">
+        <is>
+          <t>25f3d789a483b055</t>
+        </is>
+      </c>
+      <c r="AI108" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>VC-0108</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>From Battery to Potential</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Banco Interamericano de Desarrollo (BID)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Regional - América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Reciclaje de baterías, Residuos electrónicos, Cierre de ciclo</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/home/calls-proposals/battery-potential</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>Convocatoria abierta del BID enfocada en fortalecer iniciativas relacionadas con el ciclo de vida de baterías, incluyendo gestión de residuos, reciclaje y economía circular en el sector de energía limpia. La convocatoria busca apoyar proyectos innovadores en la región de América Latina y el Caribe.</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI en el componente de cierre de ciclo y reciclaje de materiales complejos. Las baterías representan un flujo de residuos crítico que requiere modelos circulares, ecodiseño y articulación con sector empresarial y recicladores.</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>Piloto de reciclaje de baterías de litio con inclusión de recicladores formales; Modelo de negocio circular para gestión de baterías en Colombia; Sistema de trazabilidad y REP para baterías; Alianza gremial para economía circular de residuos electrónicos</t>
+        </is>
+      </c>
+      <c r="W109" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>Empresas del sector automotriz y energía (miembros ANDI), universidades con líneas de investigación en materiales (Andes, Nacional), cooperativas de recicladores especializados, MinAmbiente, centros tecnológicos como SENA</t>
+        </is>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t>Falta información sobre fechas, montos y requisitos específicos de elegibilidad. La URL oficial no proporciona detalles completos de la convocatoria en la búsqueda.</t>
+        </is>
+      </c>
+      <c r="AA109" t="inlineStr">
+        <is>
+          <t>Acceder inmediatamente a la URL oficial del BID para verificar estado de la convocatoria, fechas de cierre, montos disponibles y requisitos de elegibilidad para entidades colombianas. Contactar al punto focal del BID en Colombia.</t>
+        </is>
+      </c>
+      <c r="AB109" t="inlineStr">
+        <is>
+          <t>Realizar verificación completa en el portal del BID, descargar términos de referencia si están disponibles, y contactar a la oficina BID Colombia (Carrera 7 No 71-21, Bogotá) para confirmar vigencia y elegibilidad de ANDI/Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AC109" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Gestión de recursos de cooperación</t>
+        </is>
+      </c>
+      <c r="AD109" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE109" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF109" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG109" t="inlineStr">
+        <is>
+          <t>La URL confirma la existencia de la convocatoria 'From Battery to Potential' pero el contenido parcial no permite verificar fechas exactas ni detalles completos. Se infiere que está relacionada con energía limpia y economía circular de baterías por el título y contexto del BID. Colombia es país miembro del BID y elegible para sus convocatorias.</t>
+        </is>
+      </c>
+      <c r="AH109" t="inlineStr">
+        <is>
+          <t>f23302ec8b5c6bb8</t>
+        </is>
+      </c>
+      <c r="AI109" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>VC-0109</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme (SGP) - Colombia</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) - implementado por UNDP Colombia</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Internacional / Estados Unidos</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Medio ambiente y sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Proyectos comunitarios de gestión ambiental y recursos naturales</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Fortalecimiento institucional; Inclusión social</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Hasta USD 15,000 para organizaciones comunitarias; hasta USD 35,000 para organizaciones con experiencia previa en gestión de recursos e implementación de proyectos</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/newsroom/news/gef-small-grants-programme-launched-colombia</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>El Programa de Pequeñas Donaciones del GEF en Colombia ofrece grants de hasta USD 15,000 para organizaciones comunitarias y hasta USD 35,000 para organizaciones con experiencia, destinados a proyectos ambientales de base comunitaria. El programa es implementado por PNUD Colombia y busca fortalecer capacidades locales en gestión ambiental y recursos naturales.</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>Relevante para componentes de inclusión de recicladores de base, economía circular territorial y fortalecimiento de organizaciones comunitarias en gestión de residuos y reciclaje. Podría financiar pilotos comunitarios de reciclaje y valorización de materiales con participación de recicladores informales.</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de cooperativas de recicladores; Pilotos de separación en la fuente a nivel comunitario; Centros de acopio y clasificación comunitarios; Capacitación en valorización de residuos; Modelos circulares territoriales con comunidades</t>
+        </is>
+      </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>Ser organización de base comunitaria (para grants pequeños) u organización con experiencia en gestión de recursos y proyectos (para grants mayores); proyecto enfocado en temáticas ambientales del GEF</t>
+        </is>
+      </c>
+      <c r="X110" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y110" t="inlineStr">
+        <is>
+          <t>Cooperativas de recicladores; organizaciones comunitarias; PNUD Colombia; alcaldías municipales; universidades con programas comunitarios; organizaciones de la sociedad civil trabajando en residuos</t>
+        </is>
+      </c>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>Montos relativamente pequeños que pueden limitar el alcance; proceso de aplicación y requisitos no especificados en la fuente; no se confirma si el programa está actualmente abierto o si fue solo un lanzamiento sin convocatorias activas actuales</t>
+        </is>
+      </c>
+      <c r="AA110" t="inlineStr">
+        <is>
+          <t>Contactar directamente a UNDP Colombia (Oficina GEF en Bogotá - Pilar Barrera Rey mencionada como Coordinadora) para verificar estado actual del programa, ventanas de aplicación y requisitos específicos</t>
+        </is>
+      </c>
+      <c r="AB110" t="inlineStr">
+        <is>
+          <t>Contactar UNDP Colombia para confirmar vigencia y procedimiento de aplicación; identificar organizaciones de recicladores aliadas que puedan aplicar directamente o con acompañamiento de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AC110" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas y cooperación; Componente de inclusión social</t>
+        </is>
+      </c>
+      <c r="AD110" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE110" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF110" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG110" t="inlineStr">
+        <is>
+          <t>La fuente es un anuncio de lanzamiento del programa pero no especifica fechas de convocatorias ni estado actual. Se requiere verificación de si hay ventanas abiertas o permanentes. Los montos son pequeños pero aplicables para iniciativas comunitarias con recicladores. La elegibilidad parece dirigida a organizaciones de base más que a gremios empresariales, pero Visión Circular podría facilitar alianzas.</t>
+        </is>
+      </c>
+      <c r="AH110" t="inlineStr">
+        <is>
+          <t>1884c1d68c226752</t>
+        </is>
+      </c>
+      <c r="AI110" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>VC-0110</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme (SGP) - Operational Phase 8</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) / UNDP</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>182 países miembros del GEF, incluye Colombia y países de América Latina</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Gestión de residuos, Contaminación plástica, Economía circular, Químicos y desechos</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo; Inclusión social</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Hasta USD 50,000 típicamente para grants estándar del SGP; hasta USD 300,000 para CSO Challenge Program</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>No especificado, aunque típicamente se valora contrapartida comunitaria</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>No especificado para Colombia; referencia de otras oficinas (ej. Gambia junio 2026) indica que Fase 8 está activa</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/nigeria/news/call-project-concepts-gef-sgp-operational-phase-8</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>El Programa de Pequeñas Donaciones del GEF (SGP) en su Fase Operacional 8 financia proyectos comunitarios que abordan cambio climático, biodiversidad, degradación de tierra, aguas internacionales y gestión de químicos/residuos. Incluye economía circular y reducción de contaminación plástica. Elegibles: ONGs locales, organizaciones comunitarias (CBOs) y organizaciones de base.</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: financia explícitamente proyectos de economía circular, gestión de residuos sólidos y reducción de plásticos. Prioriza inclusión de comunidades locales, lo que se alinea con el eje de inclusión de recicladores de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>Pilotos comunitarios de reciclaje inclusivo; Modelos circulares territoriales con recicladores de base; Manejo de plásticos flexibles en comunidades; Iniciativas de reducción de residuos y economía circular en territorios; Fortalecimiento de organizaciones de recicladores</t>
+        </is>
+      </c>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t>Organización comunitaria o ONG local registrada; Proyecto liderado por comunidades; Enfoque en una o más áreas focales del GEF (Químicos y Residuos, Cambio Climático, etc.); Aplicación a través de oficina nacional del SGP-UNDP</t>
+        </is>
+      </c>
+      <c r="X111" t="inlineStr">
+        <is>
+          <t>Concepto de proyecto; Documentos de registro legal de la organización; Presupuesto; Cartas de apoyo comunitario (típicamente requeridas en SGP); Detalles a confirmar con oficina SGP Colombia</t>
+        </is>
+      </c>
+      <c r="Y111" t="inlineStr">
+        <is>
+          <t>Organizaciones de recicladores de base; Asociaciones comunitarias; ONGs ambientales locales; Cooperativas de recicladores; Gobiernos locales; Universidades para asistencia técnica</t>
+        </is>
+      </c>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t>Montos limitados (máx. USD 50k estándar); Enfocado en organizaciones comunitarias/ONGs, no directamente gremios empresariales; Requiere capacidad de ejecución comunitaria; Proceso puede ser competitivo</t>
+        </is>
+      </c>
+      <c r="AA111" t="inlineStr">
+        <is>
+          <t>Contactar oficina SGP-UNDP Colombia para confirmar apertura de Fase 8, fechas y requisitos específicos. Evaluar alianza con organizaciones de recicladores o CBOs para coaplicar proyectos piloto de inclusión y circularidad territorial.</t>
+        </is>
+      </c>
+      <c r="AB111" t="inlineStr">
+        <is>
+          <t>Verificar estado de convocatoria Fase 8 en Colombia contactando UNDP Colombia o visitando sitio SGP nacional. Mapear aliados comunitarios elegibles.</t>
+        </is>
+      </c>
+      <c r="AC111" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas comunitarias; Especialista en inclusión de recicladores</t>
+        </is>
+      </c>
+      <c r="AD111" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE111" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF111" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG111" t="inlineStr">
+        <is>
+          <t>La información de fechas y montos exactos para Colombia no está especificada en los resultados. Se infiere elegibilidad de Colombia como país miembro del GEF. La Fase 8 está activa globalmente (referencias de Nigeria, Gambia). Se requiere verificación de convocatoria específica para Colombia.</t>
+        </is>
+      </c>
+      <c r="AH111" t="inlineStr">
+        <is>
+          <t>7606cdb73fbc51dd</t>
+        </is>
+      </c>
+      <c r="AI111" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>VC-0111</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>GEF CSO Challenge Program (SGP 2.0 Initiative)</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) / IUCN</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Países miembros del GEF, mínimo 30 iniciativas globalmente; incluye América Latina</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Innovación comunitaria, Gestión de residuos, Biodiversidad, Cambio climático</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Challenge; Innovación; Escalamiento; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Hasta USD 300,000 por iniciativa</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>Iniciativa innovadora del SGP 2.0 liderada por IUCN que ofrece grants de hasta USD 300,000 para organizaciones de la sociedad civil (CSOs). Busca apoyar iniciativas comunitarias en áreas focales del GEF, incluyendo gestión de químicos/residuos y economía circular. Enfoque en juventud, mujeres, pueblos indígenas y comunidades locales.</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>Muy pertinente: montos significativamente mayores (hasta USD 300k) permiten proyectos de mayor escala en economía circular y gestión de residuos. El enfoque en CSOs permite articular con gremios y redes de recicladores organizados.</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>Escalamiento de modelos circulares con recicladores; Fortalecimiento institucional de redes de reciclaje; Innovación en gestión de plásticos flexibles a nivel territorial; Pilotos empresariales con participación comunitaria; Sistemas territoriales de economía circular</t>
+        </is>
+      </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t>Organización de la sociedad civil registrada; Proyecto innovador en áreas focales GEF; Enfoque comunitario con participación de juventud, mujeres, pueblos indígenas o comunidades locales; Aplicación vía IUCN</t>
+        </is>
+      </c>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>No especificado; típicamente: propuesta detallada, capacidad organizacional, presupuesto, plan de sostenibilidad</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>IUCN como implementador; Redes de recicladores; Asociaciones gremiales; Cooperativas; ONGs ambientales; Gobiernos locales; Centros tecnológicos para componente innovación</t>
+        </is>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
+          <t>Información limitada sobre proceso de aplicación y fechas; Competencia global (solo 30 iniciativas); Puede requerir capacidad institucional robusta de CSO</t>
+        </is>
+      </c>
+      <c r="AA112" t="inlineStr">
+        <is>
+          <t>Contactar IUCN América Latina y oficina GEF para confirmar disponibilidad, proceso y fechas del CSO Challenge Program. Evaluar si ANDI o estructura de Visión Circular puede aplicar directamente o via alianza con CSO elegible.</t>
+        </is>
+      </c>
+      <c r="AB112" t="inlineStr">
+        <is>
+          <t>Verificar elegibilidad y proceso con IUCN. Preparar concepto de proyecto de escalamiento de economía circular territorial con recicladores.</t>
+        </is>
+      </c>
+      <c r="AC112" t="inlineStr">
+        <is>
+          <t>Dirección de Visión Circular; Coordinación de alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD112" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE112" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF112" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG112" t="inlineStr">
+        <is>
+          <t>Oportunidad de mayor escala y monto significativo. Información muy limitada en las fuentes sobre proceso específico, fechas y elegibilidad detallada. Se infiere aplicabilidad a América Latina por naturaleza global del GEF. Requiere verificación urgente de disponibilidad y requisitos con IUCN.</t>
+        </is>
+      </c>
+      <c r="AH112" t="inlineStr">
+        <is>
+          <t>7679a29c49984eff</t>
+        </is>
+      </c>
+      <c r="AI112" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-07-06
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI112"/>
+  <dimension ref="A1:AI130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3498,17 +3498,17 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Abierta permanentemente</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Requiere verificación manual</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Requiere verificación</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AI18" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -19680,7 +19680,7 @@
       </c>
       <c r="AD109" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AE109" t="inlineStr">
@@ -19705,7 +19705,7 @@
       </c>
       <c r="AI109" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -20237,6 +20237,3192 @@
       <c r="AI112" t="inlineStr">
         <is>
           <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>VC-0112</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Programa de Impulso a la Bioeconomía y la Economía Circular en Iniciativas de Articulación Productiva</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>CEPAL en conjunto con GIZ</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Alemania / Regional América Latina</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Bioeconomía, Articulación productiva</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>https://www.cepal.org/es/eventos/lanzamiento-convocatoria-programa-impulso-la-bioeconomia-la-economia-circular-iniciativas</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>Convocatoria organizada por CEPAL y GIZ en el marco del proyecto 'Promoviendo la Economía Circular en América Latina y el Caribe' (2024-2026), financiado por el BMZ de Alemania. Busca impulsar iniciativas de articulación productiva en bioeconomía y economía circular en la región.</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular ANDI, ya que se enfoca directamente en economía circular en América Latina, permite articulación con empresas y gremios, y proviene de una alianza técnica multilateral con presencia regional.</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>Articulación productiva para cierre de ciclo de envases y empaques; Modelos de negocio circulares territoriales; Pilotos empresariales de economía circular; Fortalecimiento de cadenas de valor de reciclaje con inclusión de recicladores</t>
+        </is>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>CEPAL como socio implementador; GIZ Colombia; empresas asociadas a ANDI; universidades con líneas de bioeconomía; gremios sectoriales de envases y empaques</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>Falta información completa sobre términos de referencia, fechas exactas y requisitos de elegibilidad; puede requerir articulación institucional previa con CEPAL</t>
+        </is>
+      </c>
+      <c r="AA113" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a la oficina de CEPAL en Colombia o al punto focal del proyecto GIZ-CEPAL para obtener términos de referencia completos, fechas de cierre y modalidades de participación</t>
+        </is>
+      </c>
+      <c r="AB113" t="inlineStr">
+        <is>
+          <t>Enviar correo a CEPAL Colombia y GIZ solicitando bases de la convocatoria y verificar si ANDI/Visión Circular puede aplicar como gremio o consorcio empresarial</t>
+        </is>
+      </c>
+      <c r="AC113" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos con soporte de Dirección de Sostenibilidad ANDI</t>
+        </is>
+      </c>
+      <c r="AD113" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE113" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF113" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG113" t="inlineStr">
+        <is>
+          <t>La fuente es oficial (CEPAL) y el proyecto está activo 2024-2026, pero la página solo anuncia el lanzamiento sin detallar fechas de cierre ni términos completos. Se requiere seguimiento directo con CEPAL/GIZ para obtener información detallada | Fuente fuera del listado oficial conocido (cepal.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH113" t="inlineStr">
+        <is>
+          <t>9834f44bcd567244</t>
+        </is>
+      </c>
+      <c r="AI113" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>VC-0113</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Concurso Innovación con Impacto 2026 - ASIPI</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>ASIPI (Asociación Interamericana de la Propiedad Intelectual)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Regional - América</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>América Latina y región</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Innovación</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Propiedad intelectual, Innovación con impacto social</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Innovación</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DYfe5vECjzt</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>Concurso de ASIPI que busca reconocer proyectos, procesos o productos patentables que generen impacto en la región. Enfocado en innovación con propiedad intelectual que transforme realidades sociales. El anuncio es reciente pero falta información oficial completa.</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>Pertinencia media-alta si Visión Circular tiene o puede desarrollar innovaciones patentables en economía circular (ej. nuevos procesos de reciclaje de plásticos flexibles, tecnologías de ecodiseño, modelos de trazabilidad para REP). El enfoque en impacto social conecta con la inclusión de recicladores.</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>Innovaciones patentables en tecnología de reciclaje de plásticos flexibles; Procesos innovadores de ecodiseño con propiedades técnicas demostrables; Sistemas de trazabilidad y cierre de ciclo con componentes tecnológicos protegibles</t>
+        </is>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>Proyecto, proceso o producto patentable con impacto social demostrable</t>
+        </is>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t>Centros de desarrollo tecnológico (SENA, universidades); Oficinas de transferencia tecnológica; Empresas innovadoras asociadas a ANDI con desarrollos técnicos; Expertos en propiedad intelectual</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>Fuente no oficial (Instagram); falta información sobre bases, fechas, premios y criterios; requiere que la innovación sea patentable, lo cual puede no aplicar a todos los proyectos de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AA114" t="inlineStr">
+        <is>
+          <t>Contactar directamente a ASIPI para obtener bases oficiales del concurso, fechas, requisitos de patentabilidad y naturaleza del premio; evaluar qué innovaciones de Visión Circular podrían cumplir criterios de patentabilidad</t>
+        </is>
+      </c>
+      <c r="AB114" t="inlineStr">
+        <is>
+          <t>Buscar el sitio web oficial de ASIPI y las bases completas del concurso; identificar en el portafolio de Visión Circular qué proyectos tienen componentes técnicos innovadores susceptibles de protección IP</t>
+        </is>
+      </c>
+      <c r="AC114" t="inlineStr">
+        <is>
+          <t>Coordinación de innovación y desarrollo con asesoría legal en propiedad intelectual</t>
+        </is>
+      </c>
+      <c r="AD114" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE114" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF114" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG114" t="inlineStr">
+        <is>
+          <t>Anuncio confirmado en redes sociales de ASIPI (organización reconocida), pero falta información oficial completa. La pertinencia depende de si Visión Circular tiene o puede generar innovaciones patentables. No es una convocatoria típica de financiación sino un premio de reconocimiento | Fuente fuera del listado oficial conocido (instagram.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH114" t="inlineStr">
+        <is>
+          <t>75f0b3b88a78d7a7</t>
+        </is>
+      </c>
+      <c r="AI114" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>VC-0114</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Convocatoria regional para soluciones innovadoras en plásticos - Pacto por los Plásticos Colombia, México y Chile</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Pacto por los Plásticos Colombia (en alianza con Pacto Global Red Colombia y pares de México y Chile)</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Colombia (iniciativa regional)</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Colombia, Chile, México</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Plásticos flexibles, Envases y empaques, Innovación en gestión de plásticos</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Hasta USD 10.000</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>Noviembre 2025</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>https://www.pactoglobal-colombia.org/news/convocatoria-regional-otorgara-hasta-usd-10-000-a-soluciones-innovadoras-en-plasticos-en-colombia-chile-y-mexico.html</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>Convocatoria regional lanzada en noviembre de 2025 por el Pacto por los Plásticos Colombia junto con sus pares en México y Chile, que otorga hasta USD 10.000 a iniciativas innovadoras para prevenir la contaminación por gestión inadecuada de plásticos. El enfoque prioritario está en plásticos flexibles como sachets, empaques multilaminados, etiquetas y bolsas.</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI, ya que aborda directamente el cierre de ciclo de envases y empaques, especialmente plásticos flexibles, una de las líneas de trabajo prioritarias del programa. La convocatoria apoya innovación y soluciones empresariales en economía circular de plásticos.</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr">
+        <is>
+          <t>Piloto de reciclaje de plásticos flexibles multilaminados; soluciones de ecodiseño para sachets reciclables; modelos de negocio circulares para envases flexibles; innovaciones en recolección y valorización de empaques multicapa; articulación con recicladores para plásticos flexibles</t>
+        </is>
+      </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t>Empresas productoras de envases flexibles afiliadas a ANDI, Acoplásticos, universidades con líneas de investigación en materiales, cooperativas de recicladores especializadas en flexibles, centros tecnológicos como CIDET o ICIPC</t>
+        </is>
+      </c>
+      <c r="Z115" t="inlineStr">
+        <is>
+          <t>Fecha de cierre no publicada en el extracto; monto limitado (USD 10.000) puede ser insuficiente para proyectos de mayor escala; requiere verificar criterios de elegibilidad detallados y si aplica para gremios o solo empresas/startups individuales</t>
+        </is>
+      </c>
+      <c r="AA115" t="inlineStr">
+        <is>
+          <t>Contactar de inmediato al Pacto Global Red Colombia para obtener bases completas de la convocatoria, fecha de cierre y criterios de elegibilidad. Evaluar proyectos piloto existentes en Visión Circular sobre plásticos flexibles que puedan aplicar o estructurar propuesta conjunta con empresas miembro.</t>
+        </is>
+      </c>
+      <c r="AB115" t="inlineStr">
+        <is>
+          <t>Solicitar información completa de la convocatoria al Pacto Global Red Colombia vía correo electrónico o contacto directo; revisar portafolio de empresas ANDI con innovaciones en plásticos flexibles para identificar candidatos</t>
+        </is>
+      </c>
+      <c r="AC115" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de Visión Circular / Área de Alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD115" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE115" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF115" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG115" t="inlineStr">
+        <is>
+          <t>La fuente es oficial (Pacto Global Red Colombia) y la convocatoria es reciente (noviembre 2025). Colombia es elegible directamente. La fecha de cierre no está especificada en el fragmento, lo cual requiere verificación urgente dado que ya estamos en 2025. El monto es moderado pero puede ser útil para pilotos o fases iniciales. | Fuente fuera del listado oficial conocido (pactoglobal-colombia.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH115" t="inlineStr">
+        <is>
+          <t>396140b702509c42</t>
+        </is>
+      </c>
+      <c r="AI115" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>VC-0115</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator Colombia – Call for Proposals 2026</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator Colombia (programa conjunto entre entidades multilaterales, gobiernos y sector privado)</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Colombia / Internacional</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Economía baja en carbono, proyectos climáticos de alto impacto, transición sostenible</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Financiamiento climático; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>2026 (convocatoria abierta)</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>https://bogota.gov.co/boletin-oferta-internacional/climate-finance-accelerator-colombia-2026-acelera-proyectos-climatico</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DT_Qk01FT3L</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>El Climate Finance Accelerator Colombia 2026 convoca proyectos climáticos de alto impacto que busquen fortalecer su preparación para recibir inversión y escalar soluciones hacia una economía baja en carbono. El programa ofrece acompañamiento práctico para potenciar casos de inversión, estrategias de levantamiento de capital y relacionamiento con inversionistas. Incluye sectores como energías limpias, transporte y otros prioritarios.</t>
+        </is>
+      </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>Visión Circular puede postular pilotos de economía circular, cierre de ciclo de envases y empaques, o modelos de negocio circulares como proyectos climáticos que aportan a metas de reducción de emisiones, eficiencia de recursos y generación de valor. La articulación con empresas y recicladores es elegible bajo esta convocatoria.</t>
+        </is>
+      </c>
+      <c r="V116" t="inlineStr">
+        <is>
+          <t>Modelos de negocio circulares para reducción de emisiones en gestión de envases; Pilotos de reciclaje inclusivo y valorización de plásticos flexibles; Escalamiento de soluciones de ecodiseño y reciclabilidad con impacto climático medible; Economía circular territorial en articulación con autoridades locales</t>
+        </is>
+      </c>
+      <c r="W116" t="inlineStr">
+        <is>
+          <t>Proyectos climáticos de alto impacto; preparación para inversión; contribución a metas nacionales climáticas; sectores priorizados incluyen energías limpias, transporte (se infiere apertura a gestión de residuos y economía circular por contexto de economía baja en carbono)</t>
+        </is>
+      </c>
+      <c r="X116" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y116" t="inlineStr">
+        <is>
+          <t>Empresas asociadas a ANDI, universidades para medición de impacto climático, organizaciones de recicladores formalizadas, cooperación internacional con interés en clima, alcaldías (ej. Bogotá)</t>
+        </is>
+      </c>
+      <c r="Z116" t="inlineStr">
+        <is>
+          <t>Sectores priorizados no mencionan explícitamente economía circular o residuos (solo energías limpias y transporte listados en fuente secundaria); requiere verificar elegibilidad de proyectos de envases/reciclaje bajo el paraguas climático; competencia con proyectos de energía renovable puede ser alta</t>
+        </is>
+      </c>
+      <c r="AA116" t="inlineStr">
+        <is>
+          <t>Verificar inmediatamente si proyectos de economía circular y gestión de residuos son elegibles dentro de los sectores priorizados. Solicitar bases completas de la convocatoria y términos de referencia. Preparar case de inversión que vincule economía circular con mitigación climática (emisiones evitadas, eficiencia de recursos).</t>
+        </is>
+      </c>
+      <c r="AB116" t="inlineStr">
+        <is>
+          <t>Contactar directamente a los organizadores del Climate Finance Accelerator Colombia (vía Secretaría de Desarrollo Económico de Bogotá o canales oficiales del programa) para confirmar elegibilidad de proyectos de economía circular, fechas exactas de cierre y requisitos completos. Iniciar preparación de caso de negocio climático de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AC116" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y movilización de recursos; área de innovación y pilotos empresariales</t>
+        </is>
+      </c>
+      <c r="AD116" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE116" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF116" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG116" t="inlineStr">
+        <is>
+          <t>La fuente oficial (Bogota.gov.co) confirma convocatoria abierta 2026. La fuente secundaria (Instagram) menciona sectores priorizados (energías limpias, transporte) sin mencionar explícitamente residuos o economía circular, pero el enfoque en economía baja en carbono permite inferir elegibilidad si se demuestra impacto climático. Requiere confirmar si proyectos de economía circular aplican y obtener bases completas. | Fuente fuera del listado oficial conocido (bogota.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH116" t="inlineStr">
+        <is>
+          <t>b17963d647316ef2</t>
+        </is>
+      </c>
+      <c r="AI116" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>VC-0116</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Programa de Fomento de la Economía Circular en América Latina y el Caribe - GIZ</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Deutsche Gesellschaft für Internationale Zusammenarbeit (GIZ) GmbH</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe, incluye Colombia</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Estrategias de economía circular, envases y empaques, medición y seguimiento de circularidad</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Abierta - programa en curso</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>https://www.giz.de/en/projects/fomento-de-la-economia-circular-en-america-latina-y-el-caribe</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>https://www.giz.de/de/downloads/giz2025-es-EyE-Casos-exito-innovaci%C3%B3n-envases-y-empaques.pdf</t>
+        </is>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>GIZ brinda apoyo a la CEPAL para acompañar a países de América Latina y el Caribe en la transición hacia economía circular. Ofrece asesoramiento técnico para definir parámetros de medición y seguimiento con enfoque ambiental, social y económico. El programa trabaja específicamente en innovación para circularidad de envases y empaques.</t>
+        </is>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI al trabajar directamente en economía circular de envases y empaques, incluyendo innovación tecnológica, medición de circularidad y estrategias de implementación. El documento sobre casos de éxito en envases y empaques indica trabajo activo en 2025.</t>
+        </is>
+      </c>
+      <c r="V117" t="inlineStr">
+        <is>
+          <t>Asesoramiento en indicadores de circularidad para envases; fortalecimiento de estrategias de economía circular territorial; innovación tecnológica en reciclaje de empaques; articulación con CEPAL para políticas públicas; pilotos de nuevas tecnologías de reciclaje; transferencia de casos de éxito regionales.</t>
+        </is>
+      </c>
+      <c r="W117" t="inlineStr">
+        <is>
+          <t>No especificado - el programa trabaja con CEPAL y países miembros, sugiere articulación institucional</t>
+        </is>
+      </c>
+      <c r="X117" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y117" t="inlineStr">
+        <is>
+          <t>CEPAL como contraparte principal; ministerios de ambiente y economía; gremios empresariales; centros de investigación en economía circular; universidades con líneas en sostenibilidad</t>
+        </is>
+      </c>
+      <c r="Z117" t="inlineStr">
+        <is>
+          <t>No se especifica si hay convocatorias abiertas o si opera bajo demanda institucional; puede requerir articulación a nivel gubernamental o a través de CEPAL</t>
+        </is>
+      </c>
+      <c r="AA117" t="inlineStr">
+        <is>
+          <t>Contactar directamente a GIZ Colombia o CEPAL para explorar mecanismos de articulación del programa Visión Circular con esta iniciativa regional, especialmente en el componente de envases y empaques</t>
+        </is>
+      </c>
+      <c r="AB117" t="inlineStr">
+        <is>
+          <t>Identificar punto focal de GIZ en Colombia y CEPAL para economía circular; preparar perfil de Visión Circular y áreas de interés en asistencia técnica</t>
+        </is>
+      </c>
+      <c r="AC117" t="inlineStr">
+        <is>
+          <t>Dirección de Visión Circular ANDI / Coordinación de alianzas internacionales</t>
+        </is>
+      </c>
+      <c r="AD117" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE117" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF117" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG117" t="inlineStr">
+        <is>
+          <t>El documento de casos de éxito en envases y empaques tiene fecha 2025, indicando que es un programa activo. La URL secundaria muestra trabajo específico en innovación de envases. No se especifica si hay convocatoria abierta o si opera mediante solicitud directa de asistencia técnica.</t>
+        </is>
+      </c>
+      <c r="AH117" t="inlineStr">
+        <is>
+          <t>1feae068df003be9</t>
+        </is>
+      </c>
+      <c r="AI117" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>VC-0117</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Instrumentos Financieros BID Invest para Economía Circular en América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>BID Invest (Grupo Banco Interamericano de Desarrollo)</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Multilateral (sede en Estados Unidos)</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe, incluye Colombia</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Financiamiento de modelos de negocio circulares, reciclaje, gestión de residuos, sostenibilidad empresarial</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Cofinanciación; Asistencia técnica; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>Probable - BID Invest típicamente requiere cofinanciación del sector privado</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>Abierta - evaluación continua de proyectos</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>https://idbinvest.org/es/publicaciones/desbloqueando-el-financiamiento-de-la-economia-circular-en-america-latina-y-el-caribe</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>BID Invest publicó en marzo 2023 recomendaciones y lineamientos para instituciones financieras, reguladores y diseñadores de políticas para promover la implementación de economía circular en la región. El documento indica que instituciones financieras y gobiernos pueden desempeñar papel fundamental en desarrollo y promoción de la agenda circular, sugiriendo instrumentos financieros estructurados disponibles.</t>
+        </is>
+      </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular al ofrecer vehículos financieros específicos para economía circular que podrían aplicarse a proyectos de reciclaje, cierre de ciclo de envases, modelos de negocio circulares y escalamiento de iniciativas empresariales del programa.</t>
+        </is>
+      </c>
+      <c r="V118" t="inlineStr">
+        <is>
+          <t>Financiamiento de infraestructura de reciclaje; escalamiento de modelos de negocio circulares de empresas; inversión en tecnologías de ecodiseño y reciclabilidad; proyectos de gestión avanzada de residuos de envases; capitalización de empresas de recicladores formalizados.</t>
+        </is>
+      </c>
+      <c r="W118" t="inlineStr">
+        <is>
+          <t>Típicamente proyectos del sector privado con viabilidad financiera; potencial de escalamiento; impacto ambiental medible; cumplimiento de salvaguardas ambientales y sociales del BID</t>
+        </is>
+      </c>
+      <c r="X118" t="inlineStr">
+        <is>
+          <t>Plan de negocios; análisis financiero; evaluación de impacto ambiental; estructura de gobernanza; indicadores de circularidad (inferido de estándares BID)</t>
+        </is>
+      </c>
+      <c r="Y118" t="inlineStr">
+        <is>
+          <t>Empresas miembros de ANDI con proyectos circulares; instituciones financieras colombianas; fondos de inversión de impacto; cooperativas de recicladores formalizadas; centros tecnológicos para validación técnica</t>
+        </is>
+      </c>
+      <c r="Z118" t="inlineStr">
+        <is>
+          <t>BID Invest típicamente financia proyectos de mayor escala con retorno financiero; puede no ser adecuado para iniciativas de inclusión social sin componente comercial robusto; procesos de evaluación pueden ser extensos (6-12 meses)</t>
+        </is>
+      </c>
+      <c r="AA118" t="inlineStr">
+        <is>
+          <t>Revisar el documento técnico completo de BID Invest para identificar instrumentos específicos; pre-identificar 2-3 proyectos empresariales del portafolio de Visión Circular con potencial de escalamiento que califiquen</t>
+        </is>
+      </c>
+      <c r="AB118" t="inlineStr">
+        <is>
+          <t>Descargar y analizar el documento completo de BID Invest; agendar reunión exploratoria con oficial de inversiones de BID Invest Colombia; preparar pipeline de proyectos potenciales</t>
+        </is>
+      </c>
+      <c r="AC118" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Área de movilización de recursos / Alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD118" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE118" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF118" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG118" t="inlineStr">
+        <is>
+          <t>La publicación es de marzo 2023, relativamente reciente pero no especifica si hay convocatorias abiertas o solo son lineamientos. BID Invest opera principalmente con evaluación continua de proyectos presentados por el sector privado. La elegibilidad dependerá de tener proyectos estructurados con viabilidad financiera.</t>
+        </is>
+      </c>
+      <c r="AH118" t="inlineStr">
+        <is>
+          <t>20c26836ebf38d02</t>
+        </is>
+      </c>
+      <c r="AI118" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>VC-0118</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Núcleo RECICLABLES 2026</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Expo Reciclables</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Colombia (se infiere por contexto del sector)</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Reciclaje</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Innovación, sostenibilidad, economía circular en el sector del reciclaje</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>2025-01-20</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DaHM8qSR1Yf</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>Convocatoria Núcleo RECICLABLES 2026 busca reconocer e impulsar proyectos que promuevan innovación, sostenibilidad y fortalecimiento de la economía circular en el sector del reciclaje en Colombia. Dirigida a empresas, profesionales y actores clave de la industria del reciclaje. Fecha de apertura reciente (enero 2025).</t>
+        </is>
+      </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: reconoce proyectos de economía circular, reciclaje e innovación en el sector. Visión Circular puede postular iniciativas de cierre de ciclo de envases, inclusión de recicladores, pilotos empresariales o modelos de negocio circulares desarrollados con empresas asociadas a ANDI.</t>
+        </is>
+      </c>
+      <c r="V119" t="inlineStr">
+        <is>
+          <t>Inclusión de recicladores en cadenas de valor de envases; Pilotos de cierre de ciclo de empaques; Innovaciones en reciclaje de plásticos flexibles; Modelos de negocio circulares territoriales con empresas; Proyectos de ecodiseño para reciclabilidad</t>
+        </is>
+      </c>
+      <c r="W119" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X119" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y119" t="inlineStr">
+        <is>
+          <t>Empresas asociadas ANDI, cooperativas de recicladores, empresas transformadoras de plásticos, centros tecnológicos</t>
+        </is>
+      </c>
+      <c r="Z119" t="inlineStr">
+        <is>
+          <t>Fuente no oficial (Instagram); falta información detallada sobre bases, criterios, premios, fechas de cierre y sitio web oficial</t>
+        </is>
+      </c>
+      <c r="AA119" t="inlineStr">
+        <is>
+          <t>Contactar directamente a Expo Reciclables para obtener bases completas, fechas de cierre, montos de premios y criterios de evaluación. Evaluar postular proyectos emblemáticos del programa Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB119" t="inlineStr">
+        <is>
+          <t>Solicitar información oficial vía Instagram/correo de Expo Reciclables; revisar sitio web oficial si existe; identificar 2-3 proyectos candidatos del portafolio de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AC119" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Comunicaciones</t>
+        </is>
+      </c>
+      <c r="AD119" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE119" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF119" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG119" t="inlineStr">
+        <is>
+          <t>La fuente es Instagram (post oficial de @exporeciclables), no hay URL de convocatoria formal. Se infiere apertura reciente (enero 2025) y evento en 2026. Requiere verificación de bases, elegibilidad y plazos. Sin embargo, la alineación temática es total. | Fuente fuera del listado oficial conocido (instagram.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH119" t="inlineStr">
+        <is>
+          <t>e0c12c10185ae084</t>
+        </is>
+      </c>
+      <c r="AI119" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>VC-0119</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia Innovation Challenge - Agrichallenge</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Agritech Challenge (organización convocante; no se especifica financiador principal en el extracto)</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Sector agroalimentario, modelos de negocio circulares</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Aceleración; Innovación; Cooperación técnica</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>El CircularEconomy4Colombia Innovation Challenge está diseñado para acelerar la transición hacia una economía circular en el sector agroalimentario de Colombia, en línea con el Plan Nacional de Desarrollo 2022-2026 y los objetivos de COP 16 Colombia. Ofrece mentoría de expertos, acceso a redes y apoyo integral para soluciones innovadoras circulares.</t>
+        </is>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>Directamente alineado con la Estrategia Nacional de Economía Circular de Colombia y la promoción de modelos de negocio circulares. Aunque enfocado en agroalimentario, puede haber sinergias con empaques/envases del sector y aprendizajes en circularidad aplicables a Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr">
+        <is>
+          <t>Desarrollo de pilotos de economía circular en empaques agroalimentarios; innovación en envases compostables o reutilizables para alimentos; modelos de negocio circulares en cadenas de valor agroalimentarias con gestión de residuos de empaques.</t>
+        </is>
+      </c>
+      <c r="W120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y120" t="inlineStr">
+        <is>
+          <t>Empresas del sector agroalimentario miembros de ANDI, universidades con facultades de agronomía o ingeniería ambiental, cooperativas de recicladores que manejen residuos agroindustriales, Ministerio de Ambiente y Desarrollo Sostenible.</t>
+        </is>
+      </c>
+      <c r="Z120" t="inlineStr">
+        <is>
+          <t>Foco sectorial en agroalimentario puede limitar aplicabilidad directa a otros empaques industriales. Falta claridad sobre fechas de convocatoria activa y montos disponibles.</t>
+        </is>
+      </c>
+      <c r="AA120" t="inlineStr">
+        <is>
+          <t>Verificar urgentemente si la convocatoria está abierta o tiene fechas de próxima apertura. Contactar a los organizadores para confirmar elegibilidad de proyectos relacionados con empaques agroalimentarios.</t>
+        </is>
+      </c>
+      <c r="AB120" t="inlineStr">
+        <is>
+          <t>Visitar la URL oficial y buscar información de contacto o formularios de inscripción; consultar con el equipo de Visión Circular si hay interés en articular con sector agroalimentario.</t>
+        </is>
+      </c>
+      <c r="AC120" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD120" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE120" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF120" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG120" t="inlineStr">
+        <is>
+          <t>La fuente confirma alineación con estrategia nacional y COP16 Colombia, lo que sugiere respaldo institucional. Sin embargo, no se encontró información sobre plazos, montos, requisitos ni estado de convocatoria (si está abierta, cerrada o es permanente). Requiere verificación urgente de vigencia. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH120" t="inlineStr">
+        <is>
+          <t>c14729c40ab15707</t>
+        </is>
+      </c>
+      <c r="AI120" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>VC-0120</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Plastics Innovation Programme 2026 - Call for Proposals</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>UNDP - UN Peace and Development Fund (UNPDF) / Government of China / UN DESA</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Agencia ONU</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Global (UNDP)</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Plásticos, reducción de residuos plásticos, alternativas sostenibles</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Piloto demostrativo; Innovación</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/vietnam/news/call-proposals-plastics-innovation-programme-2026</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>El UNDP lanzó una convocatoria 2026 bajo el Plastics Innovation Programme, financiada por el Fondo de Paz y Desarrollo de la ONU con contribuciones del gobierno de China y UN DESA. La convocatoria busca pilotar y promover iniciativas que reduzcan la generación de residuos plásticos y fomenten la producción de alternativas sostenibles, alineada con la Agenda 2030.</t>
+        </is>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI: aborda directamente la reducción de residuos plásticos, promoción de alternativas sostenibles y pilotos de innovación, componentes centrales del programa de economía circular, reciclaje y gestión de envases y empaques.</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>Pilotos de innovación en reducción de plásticos flexibles; desarrollo de alternativas sostenibles a envases plásticos; modelos de negocio circulares para empaques; proyectos de economía circular empresarial en plásticos; inclusión de recicladores en cadenas de valor de plásticos.</t>
+        </is>
+      </c>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t>UNDP Colombia, empresas miembro de Visión Circular, universidades con líneas de investigación en materiales, PNUD regional, cooperativas de recicladores, gremios sectoriales (plásticos, empaques).</t>
+        </is>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>Elegibilidad geográfica no confirmada para Colombia o América Latina (la noticia se publica desde UNDP Vietnam); requisitos y fechas no disponibles en la fuente; puede ser un programa piloto con cobertura limitada.</t>
+        </is>
+      </c>
+      <c r="AA121" t="inlineStr">
+        <is>
+          <t>Verificar inmediatamente elegibilidad para Colombia/América Latina contactando a UNDP Colombia o la oficina regional, solicitar términos de referencia completos y calendario de la convocatoria 2026.</t>
+        </is>
+      </c>
+      <c r="AB121" t="inlineStr">
+        <is>
+          <t>Contactar a UNDP Colombia (oficina de Bogotá) y UNDP Regional LAC para confirmar si Colombia es elegible y solicitar documentos oficiales de la convocatoria.</t>
+        </is>
+      </c>
+      <c r="AC121" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Gestión de alianzas internacionales</t>
+        </is>
+      </c>
+      <c r="AD121" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE121" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF121" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG121" t="inlineStr">
+        <is>
+          <t>La URL refiere a una publicación de UNDP Vietnam, lo que genera incertidumbre sobre la elegibilidad geográfica para Colombia o América Latina. No se especifican países elegibles, montos, fechas exactas ni requisitos. Se infiere que es una convocatoria global o multi-regional por la naturaleza del fondo (UNPDF), pero requiere confirmación urgente.</t>
+        </is>
+      </c>
+      <c r="AH121" t="inlineStr">
+        <is>
+          <t>a884faae3ea0b0eb</t>
+        </is>
+      </c>
+      <c r="AI121" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>VC-0121</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Unlocking Circular Economy Finance in Latin America and the Caribbean</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>UNEP Finance Initiative (UNEP FI) en alianza con Banco Interamericano de Desarrollo (BID)</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Agencia ONU</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Global / Regional LAC</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Brasil, Chile, Colombia, Costa Rica, República Dominicana, México, Perú</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Financiamiento de economía circular, taxonomías sostenibles, movilización de recursos públicos y privados</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Asistencia técnica; Fortalecimiento institucional; Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>https://www.unepfi.org/publications/unlocking-circular-economy-finance-in-latin-america-and-the-caribbean-the-catalyst-for-a-positive-change</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>Recurso desarrollado por UNEP en alianza con el BID basado en consultas multi-actor en siete jurisdicciones latinoamericanas (incluye Colombia). Aunque la URL refiere a una publicación, podría estar asociada a programas de asistencia técnica, financiamiento o plataformas de movilización de recursos para economía circular en la región.</t>
+        </is>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular ANDI: Colombia es uno de los países objetivo; aborda financiamiento de economía circular, taxonomías sostenibles (Colombia desarrolla su propia taxonomía verde con componente de economía circular según fuente [3]), y movilización de recursos públicos y privados, fundamentales para escalar el programa.</t>
+        </is>
+      </c>
+      <c r="V122" t="inlineStr">
+        <is>
+          <t>Acceso a líneas de financiamiento para proyectos de economía circular empresarial; articulación con taxonomía verde de Colombia; diseño de instrumentos financieros para reciclaje e inclusión; fortalecimiento de capacidades para acceso a financiamiento climático y circular.</t>
+        </is>
+      </c>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t>BID Colombia, UNEP FI, Ministerio de Ambiente y Desarrollo Sostenible, Ministerio de Hacienda (taxonomía verde), banca comercial con líneas sostenibles, empresas miembro ANDI, gremios sectoriales.</t>
+        </is>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>La fuente es una publicación/recurso técnico, no una convocatoria activa; no se confirma si hay fondos disponibles o ventanas de aplicación; puede ser solo un marco de referencia sin financiamiento directo asociado.</t>
+        </is>
+      </c>
+      <c r="AA122" t="inlineStr">
+        <is>
+          <t>Descargar y analizar la publicación completa; contactar a UNEP FI LAC y BID Colombia para identificar si existen programas, fondos o ventanas de asistencia técnica activas derivadas de esta iniciativa; explorar conexión con la taxonomía verde de Colombia.</t>
+        </is>
+      </c>
+      <c r="AB122" t="inlineStr">
+        <is>
+          <t>Revisar publicación completa y contactar a los puntos focales de UNEP FI en Colombia y al equipo de Cambio Climático y Desarrollo Sostenible del BID para identificar oportunidades concretas de financiamiento o asistencia técnica.</t>
+        </is>
+      </c>
+      <c r="AC122" t="inlineStr">
+        <is>
+          <t>Atracción de recursos / Alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD122" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE122" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF122" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG122" t="inlineStr">
+        <is>
+          <t>La fuente es una publicación técnica, no una convocatoria activa. Colombia está explícitamente incluida en el alcance geográfico. Se infiere que podría haber programas de asistencia técnica o acceso a financiamiento asociados, pero no se confirma una ventana de aplicación activa. La relación con la taxonomía verde de Colombia (fuente [3]) sugiere relevancia institucional alta. | Fuente fuera del listado oficial conocido (unepfi.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH122" t="inlineStr">
+        <is>
+          <t>297914b65ddffdb9</t>
+        </is>
+      </c>
+      <c r="AI122" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>VC-0122</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Too Good to Waste - Iniciativa de reducción de emisiones de metano en gestión de residuos sólidos</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Banco Interamericano de Desarrollo (BID), Global Methane Hub, AquaFund</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Regional - América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (incluye Colombia)</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Residuos y economía circular</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Gestión de residuos sólidos, reducción de metano, economía circular</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cofinanciación; Cooperación técnica</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>Sí - el BID está explorando cofinanciación con GEF y otras iniciativas para propuestas de alta demanda</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>https://www.ccap.org/post/latin-america-and-the-caribbean-countries-seek-to-reduce-methane-emissions-in-the-solid-waste-sector</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>Iniciativa del BID financiada por Global Methane Hub y AquaFund para mejorar la gestión de residuos sólidos en América Latina y el Caribe, reduciendo emisiones de metano y promoviendo economía circular. Ante alta demanda, el BID explora cofinanciación con fondos GEF y otras iniciativas para propuestas elegibles.</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular: aborda gestión de residuos sólidos, economía circular y tiene enfoque territorial en América Latina, alineándose con el cierre de ciclo de materiales, inclusión de recicladores y modelos circulares que promueve la ANDI.</t>
+        </is>
+      </c>
+      <c r="V123" t="inlineStr">
+        <is>
+          <t>Proyectos de valorización de residuos de envases y empaques para reducir metano; sistemas territoriales de reciclaje inclusivo; modelos circulares empresariales para residuos orgánicos vinculados a empaques compostables; articulación gremial para gestión de residuos post-consumo REP</t>
+        </is>
+      </c>
+      <c r="W123" t="inlineStr">
+        <is>
+          <t>No especificado - requiere verificación en sitio oficial del BID o contacto directo</t>
+        </is>
+      </c>
+      <c r="X123" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y123" t="inlineStr">
+        <is>
+          <t>Municipios y autoridades ambientales colombianas, organizaciones de recicladores de base, universidades con líneas en gestión de residuos, empresas del sector envases/empaques miembros de ANDI, cooperación GEF para cofinanciación</t>
+        </is>
+      </c>
+      <c r="Z123" t="inlineStr">
+        <is>
+          <t>Fechas y ventana de aplicación no especificadas en la fuente; alta demanda puede limitar recursos disponibles; requiere verificar si Call for Proposals sigue abierta o si hay próxima convocatoria</t>
+        </is>
+      </c>
+      <c r="AA123" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente la oficina del BID en Colombia o unidad Too Good to Waste para confirmar vigencia, plazos y requisitos de la convocatoria. Preparar concepto de proyecto territorial que vincule reducción de metano con reciclaje de envases.</t>
+        </is>
+      </c>
+      <c r="AB123" t="inlineStr">
+        <is>
+          <t>Buscar contacto directo BID Colombia o Global Methane Hub para confirmar estado de convocatoria y obtener términos de referencia oficiales</t>
+        </is>
+      </c>
+      <c r="AC123" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y Alianzas institucionales - perfil con experiencia en banca multilateral</t>
+        </is>
+      </c>
+      <c r="AD123" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE123" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF123" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG123" t="inlineStr">
+        <is>
+          <t>La fuente menciona 'Call for Proposals' y alta demanda, sugiriendo proceso activo o reciente, pero no proporciona fechas exactas ni enlace directo a convocatoria. La exploración de cofinanciación indica flexibilidad y oportunidad de escalamiento. Se infiere elegibilidad de Colombia por tratarse de iniciativa regional LAC del BID. | Fuente fuera del listado oficial conocido (ccap.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH123" t="inlineStr">
+        <is>
+          <t>d015826c15b435c6</t>
+        </is>
+      </c>
+      <c r="AI123" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>VC-0123</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Too Good to Waste Initiative</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Banco Interamericano de Desarrollo (BID)</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Regional - América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (incluyendo Colombia)</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Gestión de residuos y economía circular</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Mitigación de metano, resiliencia, economía circular en gestión de residuos</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Financiamiento concesional; Estructuración de proyectos</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/who-we-are/topics/water-and-sanitation/initiatives/too-good-waste</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>Iniciativa del BID que estructura proyectos y promueve condiciones habilitantes para la mitigación de metano, resiliencia y adopción de economía circular en el sector de gestión de residuos en América Latina y el Caribe. Proporciona asistencia técnica y apoyo en la estructuración de proyectos, aunque no se especifica si hay una convocatoria abierta formal o se accede mediante solicitud directa.</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular: aborda directamente economía circular en residuos, un tema central del programa ANDI. La mitigación de metano y estructuración de proyectos en residuos es clave para REP, modelos de negocio circulares y economía circular territorial que trabaja Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V124" t="inlineStr">
+        <is>
+          <t>Estructuración de proyectos piloto de economía circular en residuos; mitigación de metano en gestión de residuos orgánicos y de envases; articulación público-privada para infraestructura circular; fortalecimiento de capacidades territoriales en economía circular de residuos</t>
+        </is>
+      </c>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>No especificado; probablemente requiere articulación con gobiernos locales o nacionales y empresas del sector residuos</t>
+        </is>
+      </c>
+      <c r="X124" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible, alcaldías municipales, empresas del sector residuos y reciclaje afiliadas a ANDI, universidades con investigación en residuos, cooperativas de recicladores</t>
+        </is>
+      </c>
+      <c r="Z124" t="inlineStr">
+        <is>
+          <t>No hay convocatoria formal visible ni fechas. Puede requerir proceso de solicitud directa o articulación gubernamental. El acceso podría depender de prioridades del BID en Colombia.</t>
+        </is>
+      </c>
+      <c r="AA124" t="inlineStr">
+        <is>
+          <t>Contactar la División de Agua y Saneamiento del BID Colombia para: (1) presentar capacidades de Visión Circular ANDI, (2) explorar proyectos específicos elegibles bajo Too Good to Waste, (3) solicitar asistencia técnica para estructuración de proyectos piloto de economía circular en residuos.</t>
+        </is>
+      </c>
+      <c r="AB124" t="inlineStr">
+        <is>
+          <t>Identificar punto focal del BID en Colombia (División Agua y Saneamiento / Cambio Climático) y solicitar reunión para presentar portafolio de Visión Circular y explorar mecanismos de acceso a la iniciativa</t>
+        </is>
+      </c>
+      <c r="AC124" t="inlineStr">
+        <is>
+          <t>Dirección Ejecutiva / Coordinación de Alianzas Estratégicas</t>
+        </is>
+      </c>
+      <c r="AD124" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE124" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF124" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG124" t="inlineStr">
+        <is>
+          <t>Página web del BID describe la iniciativa pero no detalla proceso de aplicación ni convocatorias abiertas. Se infiere que opera mediante estructuración de proyectos a demanda o por articulación directa con gobiernos/sector privado. Colombia es elegible como país miembro del BID.</t>
+        </is>
+      </c>
+      <c r="AH124" t="inlineStr">
+        <is>
+          <t>e19e56d5fdf75037</t>
+        </is>
+      </c>
+      <c r="AI124" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>VC-0124</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Climate Finance Broker Facility - Country Platforms Colombia</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF) en colaboración con Gobierno de Colombia</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Internacional / Colombia</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Innovación climática, soluciones lideradas por países, transformación territorial</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Innovación; Fortalecimiento institucional; Cooperación técnica</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>Recientemente anunciado (2024-2025)</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/about/news-and-updates/fourteen-new-country-platforms-announced-collaboration-gcf-drive-country-led-climate-solutions</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/countries/colombia</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>Nueva iniciativa Country Platforms anunciada por GCF en colaboración con Colombia para impulsar soluciones climáticas lideradas por el país, con énfasis en innovación, protección de biodiversidad y financiamiento que se convierta en inversión sostenible para territorios. Colombia declaró compromiso de fortalecer Climate Finance Broker Facility.</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>Plataforma país permite canalizar soluciones de economía circular territorial con enfoque climático. La economía circular en envases y empaques reduce emisiones y protege biodiversidad. El enfoque territorial es altamente compatible con el modelo de economía circular territorial de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>Proyectos territoriales de economía circular con impacto climático; innovación en reciclaje y cierre de ciclo de envases con reducción de emisiones; modelos circulares que protejan biodiversidad; pilotos empresariales de descarbonización vía circularidad; inclusión de recicladores en cadenas de valor climáticas</t>
+        </is>
+      </c>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>Soluciones lideradas por Colombia; alineación con prioridades nacionales climáticas; enfoque territorial; componente de innovación</t>
+        </is>
+      </c>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>No especificado; requiere coordinación con autoridades colombianas</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible, Departamento Nacional de Planeación, gobiernos departamentales y municipales, empresas comprometidas con descarbonización, universidades, centros tecnológicos</t>
+        </is>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>Iniciativa reciente sin procedimientos operativos públicos aún; requiere articulación gubernamental de alto nivel; competencia con otros sectores por recursos limitados</t>
+        </is>
+      </c>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>Monitorear anuncios oficiales del MADS y GCF sobre operativización de Country Platform Colombia. Posicionar Visión Circular como modelo replicable de economía circular territorial con impacto climático para ser considerado en el pipeline de proyectos prioritarios</t>
+        </is>
+      </c>
+      <c r="AB125" t="inlineStr">
+        <is>
+          <t>Inscribirse en actualizaciones del GCF sobre Country Platform Colombia y solicitar briefing con equipo técnico del MADS sobre prioridades temáticas de la plataforma</t>
+        </is>
+      </c>
+      <c r="AC125" t="inlineStr">
+        <is>
+          <t>Dirección ejecutiva Visión Circular / Coordinación de incidencia y relacionamiento institucional</t>
+        </is>
+      </c>
+      <c r="AD125" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE125" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF125" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG125" t="inlineStr">
+        <is>
+          <t>Iniciativa muy reciente (anunciada en noticia) sin detalles operativos específicos aún disponibles. Alta pertinencia estratégica pero requiere seguimiento para conocer procedimientos de aplicación. Colombia expresó compromiso político explícito lo que aumenta probabilidad de materialización</t>
+        </is>
+      </c>
+      <c r="AH125" t="inlineStr">
+        <is>
+          <t>5dc7de241fa94b8b</t>
+        </is>
+      </c>
+      <c r="AI125" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>VC-0125</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme (SGP) Colombia</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) / UNDP</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Colombia (lanzamiento específico para el país)</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Medio ambiente</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Proyectos comunitarios, gestión de recursos naturales, biodiversidad</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Fortalecimiento institucional; Inclusión social</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Hasta USD 15,000 para organizaciones comunitarias; hasta USD 35,000 para organizaciones con experiencia previa</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>Lanzado (según noticia del GEF)</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/newsroom/news/gef-small-grants-programme-launched-colombia</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>El Programa de Pequeñas Donaciones del GEF fue lanzado en Colombia para financiar proyectos comunitarios ambientales. Ofrece grants de hasta USD 15,000 para organizaciones de base comunitaria y hasta USD 35,000 para organizaciones con experiencia en gestión de recursos e implementación de proyectos.</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>Puede financiar proyectos piloto comunitarios de reciclaje inclusivo, fortalecimiento de asociaciones de recicladores, iniciativas locales de economía circular, proyectos de gestión de residuos de envases a nivel comunitario, y modelos de negocio circulares de base comunitaria.</t>
+        </is>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de organizaciones de recicladores de base; pilotos comunitarios de recolección y valorización de envases; proyectos de educación ambiental y separación en la fuente; iniciativas de economía circular territorial a escala local; modelos de aprovechamiento de residuos plásticos flexibles en comunidades</t>
+        </is>
+      </c>
+      <c r="W126" t="inlineStr">
+        <is>
+          <t>Organizaciones comunitarias o con experiencia en gestión de recursos; proyectos ambientales con impacto local; implementación en Colombia</t>
+        </is>
+      </c>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>No especificado; requiere consultar con oficina SGP/UNDP Colombia</t>
+        </is>
+      </c>
+      <c r="Y126" t="inlineStr">
+        <is>
+          <t>Organizaciones de recicladores (ANRC, asociaciones locales), ONGs ambientales comunitarias, grupos de mujeres recicladoras, cooperativas, juntas de acción comunal, organizaciones de base en territorios prioritarios de Visión Circular</t>
+        </is>
+      </c>
+      <c r="Z126" t="inlineStr">
+        <is>
+          <t>Montos relativamente pequeños; enfoque comunitario puede limitar proyectos empresariales directos; prioridades temáticas específicas del SGP Colombia no detalladas en la fuente</t>
+        </is>
+      </c>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>Identificar organizaciones de recicladores y aliados comunitarios de Visión Circular que puedan aplicar. ANDI/Visión Circular puede fungir como facilitador técnico y articulador, apoyando desarrollo de propuestas de recicladores para proyectos piloto que demuestren modelos circulares inclusivos replicables</t>
+        </is>
+      </c>
+      <c r="AB126" t="inlineStr">
+        <is>
+          <t>Contactar a Pilar Barrera Rey (Coordinadora de Alianzas GEF en Bogotá según fuente) y oficina UNDP Colombia para conocer lineamientos, prioridades temáticas y procedimientos de aplicación del SGP en Colombia</t>
+        </is>
+      </c>
+      <c r="AC126" t="inlineStr">
+        <is>
+          <t>Coordinación de inclusión y recicladores / Coordinación de proyectos comunitarios</t>
+        </is>
+      </c>
+      <c r="AD126" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE126" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF126" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG126" t="inlineStr">
+        <is>
+          <t>Programa confirmado lanzado en Colombia. Montos son pequeños pero altamente accesibles para organizaciones de base. Excelente oportunidad para pilotos de inclusión de recicladores. ANDI no aplicaría directamente pero puede apoyar técnicamente a organizaciones comunitarias aliadas. Requiere verificar si hay convocatorias específicas abiertas o es proceso continuo</t>
+        </is>
+      </c>
+      <c r="AH126" t="inlineStr">
+        <is>
+          <t>aaa527bc5c5c6730</t>
+        </is>
+      </c>
+      <c r="AI126" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>VC-0126</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Program - CSO Challenge Program</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) - implementado por International Union for Conservation of Nature (IUCN)</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Internacional (sede en Washington D.C., EE.UU.)</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>182 países miembros del GEF, incluida Colombia y América Latina</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Medio ambiente y sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Economía circular, Residuos, Biodiversidad, Cambio climático, Soluciones ambientales innovadoras</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Asistencia técnica; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Hasta USD 300,000 por proyecto; programa total de USD 10 millones</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>Junio 2024</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>https://iucn.org/press-release/202510/new-gef-programme-set-deliver-grants-usd-300000-civil-society-led</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>Programa de USD 10 millones del GEF implementado por IUCN que ofrece grants de hasta USD 300,000 para organizaciones de la sociedad civil (CSO) que busquen escalar soluciones ambientales innovadoras. Fue lanzado oficialmente en junio 2024 en la Octava Asamblea del GEF y busca apoyar a CSOs locales, pueblos indígenas, comunidades locales, mujeres y jóvenes con recursos financieros y técnicos.</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular ANDI pues financia soluciones ambientales innovadoras escalables, incluyendo economía circular, gestión de residuos y degradación de tierras. El enfoque en escalamiento y fortalecimiento de CSOs se alinea con el trabajo de inclusión de recicladores y modelos circulares territoriales.</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>Escalamiento de modelos de inclusión de recicladores; Proyectos piloto de economía circular territorial con comunidades; Soluciones innovadoras para gestión de residuos plásticos con enfoque comunitario; Fortalecimiento de organizaciones de recicladores como CSOs; Modelos circulares con pueblos indígenas y comunidades locales</t>
+        </is>
+      </c>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>Ser una organización de la sociedad civil (CSO) local; Proponer soluciones ambientales innovadoras escalables; Enfoque en comunidades locales, pueblos indígenas, mujeres o jóvenes; Alineación con prioridades ambientales del GEF (biodiversidad, clima, residuos, degradación de tierras, aguas internacionales, químicos)</t>
+        </is>
+      </c>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t>Organizaciones de recicladores formalizadas; Universidades para componente técnico-científico; Gobiernos locales para articulación territorial; Empresas del programa Visión Circular como co-implementadores; Fundaciones ambientales colombianas; PNUD Colombia como punto focal GEF</t>
+        </is>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>Detalles específicos de aplicación aún no publicados completamente; Competencia alta por ser programa global; Requiere que ANDI o Visión Circular se asocie con CSOs locales (no puede aplicar directamente como gremio empresarial); Posible requerimiento de experiencia previa en proyectos GEF</t>
+        </is>
+      </c>
+      <c r="AA127" t="inlineStr">
+        <is>
+          <t>Establecer contacto inmediato con la oficina de IUCN para América Latina y con el punto focal GEF en Colombia (PNUD) para obtener lineamientos específicos de aplicación. Identificar CSOs aliadas (organizaciones de recicladores, ONGs ambientales) para estructurar alianza estratégica donde Visión Circular aporte expertise técnico y las CSOs sean solicitantes formales.</t>
+        </is>
+      </c>
+      <c r="AB127" t="inlineStr">
+        <is>
+          <t>Contactar a IUCN Oficina Regional para América del Sur (ecuador@iucn.org / sur@iucn.org) y al PNUD Colombia - Programa SGP para solicitar términos de referencia específicos y explorar elegibilidad de alianzas gremio-CSO. Revisar base de datos de proyectos GEF en Colombia para identificar socios exitosos previos.</t>
+        </is>
+      </c>
+      <c r="AC127" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y cooperación internacional de Visión Circular / ANDI, en articulación con área de inclusión social y alianzas con recicladores</t>
+        </is>
+      </c>
+      <c r="AD127" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE127" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF127" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG127" t="inlineStr">
+        <is>
+          <t>El programa fue lanzado en junio 2024 (nota: hay inconsistencia en fuente [2] que menciona '202510' que interpreto como octubre 2025, posible error tipográfico; asumo 2024 como correcto por coherencia con 'Octava Asamblea'). No se encontraron detalles específicos sobre proceso y fechas de aplicación, lo que requiere verificación directa con IUCN/GEF. La elegibilidad de ANDI es indirecta: requiere alianza con CSO que sea el aplicante formal, con ANDI/Visión Circular como socio técnico.</t>
+        </is>
+      </c>
+      <c r="AH127" t="inlineStr">
+        <is>
+          <t>764dac7a4a14b7a0</t>
+        </is>
+      </c>
+      <c r="AI127" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>VC-0127</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme - Ventana Regular</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) - implementado por PNUD</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Internacional (sede en Washington D.C., EE.UU.)</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>182 países miembros del GEF, incluida Colombia y América Latina</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Medio ambiente y sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Biodiversidad, Cambio climático, Aguas internacionales, Degradación de tierras, Químicos y residuos</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Asistencia técnica; Fortalecimiento comunitario</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Típicamente hasta USD 50,000 por proyecto (SGP regular)</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>Usualmente requerida, proporción no especificada en las fuentes</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente (convocatorias por país)</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>Varía por país; Colombia tiene convocatorias periódicas</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/georgia/projects/gef-small-grants-programme</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>Programa establecido del GEF que desde 1991 financia proyectos comunitarios con grants típicamente de hasta USD 50,000 para generar beneficios ambientales globales a través de acciones locales. Opera en 182 países mediante oficinas nacionales coordinadas por PNUD, con convocatorias periódicas por país. Colombia tiene historial activo de proyectos GEF según fuente [3].</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>Relevante para componentes territoriales y comunitarios de Visión Circular. Puede financiar pilotos de economía circular a nivel local, proyectos de gestión de residuos comunitarios, iniciativas de inclusión de recicladores de base, y proyectos de degradación de tierras relacionados con residuos. Menor escala que el CSO Challenge pero más accesible.</t>
+        </is>
+      </c>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje comunitario; Centros de acopio y clasificación gestionados por comunidades; Compostaje comunitario y economía circular orgánica; Proyectos de limpieza de residuos en cuencas y aguas; Capacitación y formalización de recicladores de base; Soluciones locales para plásticos en zonas costeras o rurales</t>
+        </is>
+      </c>
+      <c r="W128" t="inlineStr">
+        <is>
+          <t>Comunidades locales, ONGs de base, organizaciones comunitarias como solicitantes principales; Alineación con áreas focales GEF; Impacto ambiental global demostrable; Participación comunitaria significativa; Cofinanciación (en especie o efectivo)</t>
+        </is>
+      </c>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y128" t="inlineStr">
+        <is>
+          <t>Organizaciones comunitarias de recicladores; Juntas de acción comunal; ONGs ambientales locales; Alcaldías municipales; Universidades regionales; Cooperativas de recicladores; Empresas de Visión Circular como proveedores de asistencia técnica o cofinanciación</t>
+        </is>
+      </c>
+      <c r="Z128" t="inlineStr">
+        <is>
+          <t>Montos menores que limitan escala de intervención; Procesos de aplicación pueden ser extensos; Requiere que el solicitante sea una organización comunitaria/ONG (no gremio empresarial); Enfoque muy local puede no alinearse con estrategias nacionales de Visión Circular; Disponibilidad de fondos depende del ciclo del programa por país</t>
+        </is>
+      </c>
+      <c r="AA128" t="inlineStr">
+        <is>
+          <t>Consultar con el Coordinador Nacional del SGP en Colombia (a través de PNUD Colombia) sobre convocatorias abiertas o próximas. Mapear organizaciones de recicladores y ONGs comunitarias dentro de la red de Visión Circular que puedan aplicar. Ofrecer desde ANDI/Visión Circular asistencia técnica o cofinanciación como socio estratégico para fortalecer propuestas.</t>
+        </is>
+      </c>
+      <c r="AB128" t="inlineStr">
+        <is>
+          <t>Contactar al PNUD Colombia - Programa de Pequeñas Donaciones GEF (buscar coordinador nacional en oficina PNUD Bogotá) para solicitar calendario de convocatorias 2024-2025 y explorar esquema de alianza técnica ANDI-organizaciones comunitarias. Revisar proyectos SGP exitosos previos en Colombia en temas de residuos.</t>
+        </is>
+      </c>
+      <c r="AC128" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos territoriales y área de inclusión de recicladores de Visión Circular, en coordinación con área de cooperación</t>
+        </is>
+      </c>
+      <c r="AD128" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE128" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF128" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG128" t="inlineStr">
+        <is>
+          <t>Esta es la ventana regular/histórica del SGP (diferente del CSO Challenge de USD 300K). Programa bien establecido con presencia comprobada en Colombia según fuente [3]. Montos inferidos de conocimiento general del SGP (típicamente hasta USD 50K), no especificados en las fuentes proporcionadas. Elegibilidad de ANDI es indirecta, como socio técnico o cofinanciador de organizaciones comunitarias aplicantes.</t>
+        </is>
+      </c>
+      <c r="AH128" t="inlineStr">
+        <is>
+          <t>2b08d91e039c94a4</t>
+        </is>
+      </c>
+      <c r="AI128" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>VC-0128</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Programa Euroclima - Acción en Economía Circular (en diseño)</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Unión Europea - implementado por Expertise France y agencias asociadas</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>América Latina (18 países); Guatemala mencionada específicamente en fuente; alta probabilidad de que incluya Colombia</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Economía circular, Biodiversidad, Cambio climático, Diálogo político e interinstitucional</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional; Diálogo político</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>Aprox. 2024-2025 (en fase de diseño según fuente)</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>https://expertise-france.gestmax.fr/_expertise_france/public_files/tdr-experto-a-guatemala-economia-circular.pdf</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>Nueva acción del Programa Euroclima de la Unión Europea en fase de diseño, que posicionará la economía circular junto con biodiversidad y cambio climático como eje principal. El documento menciona metodología de 'Diálogo País' orientada al diálogo interinstitucional y político. Expertise France, la Delegación de la UE en países, INTPA y agencias implementadoras están diseñando esta nueva acción.</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: economía circular es el tema central de esta nueva acción de Euroclima, alineado 100% con el mandato de Visión Circular ANDI. La metodología de diálogo interinstitucional coincide con el enfoque de articulación multi-actor (empresas, gobierno, academia) de Visión Circular. Oportunidad estratégica para posicionar a ANDI como contraparte técnica en Colombia.</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>Diálogo político para marcos normativos de economía circular y REP; Desarrollo de hojas de ruta de circularidad sectorial; Articulación público-privada para economía circular; Asistencia técnica para implementación de estrategias territoriales de economía circular; Intercambio de experiencias regionales en envases y empaques; Fortalecimiento institucional para gestión circular de residuos</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>No especificado (en fase de diseño)</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>No especificado (en fase de diseño)</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible; Ministerio de Comercio, Industria y Turismo; DNP; Delegación de la Unión Europea en Colombia; Otras organizaciones gremiales; Universidades con líneas en economía circular; Gobiernos departamentales y municipales; Otros programas Euroclima en Colombia</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>Programa aún en fase de diseño, no operativo; No hay claridad sobre mecanismos de participación (¿cooperación directa con gobiernos?, ¿convocatorias abiertas?, ¿selección de socios?); Fechas y alcance geográfico específico no confirmados; Puede enfocarse solo en cooperación gobierno-gobierno sin participación directa de gremios</t>
+        </is>
+      </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>Contacto proactivo con la Delegación de la Unión Europea en Colombia y con Expertise France para manifestar interés de ANDI/Visión Circular en participar en el diseño o ser contraparte técnica de esta nueva acción. Posicionar a Visión Circular como plataforma consolidada de diálogo multi-actor en economía circular en Colombia, con capacidad de articulación público-privada que puede complementar la acción.</t>
+        </is>
+      </c>
+      <c r="AB129" t="inlineStr">
+        <is>
+          <t>Enviar comunicación formal a la Delegación de la UE en Colombia (sección de cooperación) y a Expertise France América Latina solicitando reunión para presentar Visión Circular y explorar sinergias con la nueva acción de economía circular en diseño. Preparar dossier de Visión Circular destacando capacidades de diálogo político, articulación institucional y resultados del programa.</t>
+        </is>
+      </c>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>Dirección ejecutiva de Visión Circular / ANDI y área de cooperación internacional, con apoyo de relacionamiento gubernamental</t>
+        </is>
+      </c>
+      <c r="AD129" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE129" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF129" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG129" t="inlineStr">
+        <is>
+          <t>La fuente es un documento de términos de referencia para experticia en Guatemala, lo que indica que el programa está activo en ese país. La mención a 'nueva fase' y 'próxima acción' sugiere que están expandiendo o rediseñando el programa. Colombia NO es mencionada explícitamente en el extracto, pero dado que Euroclima opera en 18 países latinoamericanos y Colombia ha sido históricamente beneficiaria, hay alta probabilidad de elegibilidad. La oportunidad está en fase muy temprana (diseño), lo que representa riesgo pero también oportunidad de influir en el diseño. | Fuente fuera del listado oficial conocido (expertise-france.gestmax.fr): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH129" t="inlineStr">
+        <is>
+          <t>975898a9ee563407</t>
+        </is>
+      </c>
+      <c r="AI129" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>VC-0129</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Programa Euroclima - Acción climática local y economía circular</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Unión Europea y Gobierno Federal de Alemania</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Unión Europea / Alemania</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Cambio climático</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Economía circular, Acción climática local, Biodiversidad</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>https://ccesantiago.aecid.es/-/cce-santiago-acoge-presentaci%C3%B3n-de-proyecto-para-fortalecer-la-acci%C3%B3n-clim%C3%A1tica-local-y-la-econom%C3%ADa-circular</t>
+        </is>
+      </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>Euroclima es un programa de cooperación regional UE-América Latina que fortalece capacidades para enfrentar el cambio climático y pérdida de biodiversidad. Cofinanciado por UE y Alemania, busca una transición sostenible, resiliente e inclusiva. La fuente menciona una presentación de proyecto específico sobre acción climática local y economía circular en Chile.</t>
+        </is>
+      </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular por su enfoque regional en economía circular y sostenibilidad. Puede financiar fortalecimiento institucional, cooperación técnica y proyectos de transición circular alineados con agendas climáticas nacionales y territoriales.</t>
+        </is>
+      </c>
+      <c r="V130" t="inlineStr">
+        <is>
+          <t>Economía circular territorial; Sistemas locales de gestión de residuos; Fortalecimiento de cadenas de reciclaje con enfoque climático; Modelos circulares resilientes al clima; Articulación institucional para REP y circularidad</t>
+        </is>
+      </c>
+      <c r="W130" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X130" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y130" t="inlineStr">
+        <is>
+          <t>Autoridades ambientales locales y nacionales, gobiernos territoriales, universidades, centros de investigación climática, gremios, cooperación alemana (GIZ), delegaciones UE en Colombia</t>
+        </is>
+      </c>
+      <c r="Z130" t="inlineStr">
+        <is>
+          <t>La fuente menciona solo una presentación de proyecto existente en Chile, no una convocatoria abierta. No hay información sobre ventanas de aplicación activas o próximas. Puede ser un programa cerrado o por invitación.</t>
+        </is>
+      </c>
+      <c r="AA130" t="inlineStr">
+        <is>
+          <t>Verificar si Euroclima tiene convocatorias abiertas o próximas para Colombia. Contactar punto focal Euroclima en Colombia o delegación UE para conocer oportunidades de cooperación técnica o componentes temáticos activos en economía circular.</t>
+        </is>
+      </c>
+      <c r="AB130" t="inlineStr">
+        <is>
+          <t>Contactar Delegación de la Unión Europea en Colombia o consultar portal oficial Euroclima para verificar convocatorias activas, componentes temáticos y modalidades de participación.</t>
+        </is>
+      </c>
+      <c r="AC130" t="inlineStr">
+        <is>
+          <t>Coordinación de cooperación internacional / Alianzas institucionales</t>
+        </is>
+      </c>
+      <c r="AD130" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE130" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF130" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG130" t="inlineStr">
+        <is>
+          <t>La fuente es una noticia sobre presentación de un proyecto específico en Chile, no un anuncio de convocatoria. No hay información sobre fechas, montos, requisitos ni si hay ventanas abiertas para Colombia. Euroclima es conocido por trabajar en LATAM incluyendo Colombia, pero se infiere elegibilidad sin confirmación de oportunidad vigente.</t>
+        </is>
+      </c>
+      <c r="AH130" t="inlineStr">
+        <is>
+          <t>09996ad71f00f9c8</t>
+        </is>
+      </c>
+      <c r="AI130" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-07-10
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI130"/>
+  <dimension ref="A1:AI151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9511,12 +9511,12 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -9596,14 +9596,14 @@
       </c>
       <c r="AE52" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AF52" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="AG52" t="inlineStr">
         <is>
           <t>Convocatoria municipal con alta alineación temática. La elegibilidad parece restringida a actores locales de Dosquebradas, pero Visión Circular podría articularse como cofinanciador o socio técnico. Fecha de cierre confirmada (30 julio 2026). Monto en COP sin desglose por proyecto. | Fuente fuera del listado oficial conocido (dosquebradas.gov.co): verificar oficialidad</t>
@@ -9616,7 +9616,7 @@
       </c>
       <c r="AI52" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -18618,7 +18618,7 @@
       </c>
       <c r="AD103" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AE103" t="inlineStr">
@@ -18643,7 +18643,7 @@
       </c>
       <c r="AI103" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -19705,7 +19705,7 @@
       </c>
       <c r="AI109" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -23423,6 +23423,3723 @@
       <c r="AI130" t="inlineStr">
         <is>
           <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>VC-0130</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Convocatoria Empresas Verdes 2026 - Cámara de Comercio de Bucaramanga</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Cámara de Comercio de Bucaramanga</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Gobierno</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Colombia (área de influencia Bucaramanga)</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Economía circular empresarial, Huella de carbono</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Cofinanciación; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>No especificado (CCB cubre 90% de consultoría)</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>Sí, empresa debe aportar 10% del costo de consultoría</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>2025-05-08</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/CCBucaramanga/posts/-convocatoria-abierta-empresas-verdes-2026quieres-que-la-sostenibilidad-impulse-/1414196654066089</t>
+        </is>
+      </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>La Cámara de Comercio de Bucaramanga seleccionará 14 empresas para recibir acompañamiento especializado en Economía Circular o Huella de Carbono, cubriendo el 90% del costo de consultoría. Busca impulsar la competitividad empresarial mediante sostenibilidad.</t>
+        </is>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>Oportunidad para empresas asociadas o del ecosistema ANDI en Santander que busquen fortalecer estrategias de economía circular o gestión de huella de carbono con cofinanciación significativa.</t>
+        </is>
+      </c>
+      <c r="V131" t="inlineStr">
+        <is>
+          <t>Diseño de modelos de negocio circulares, ecodiseño de envases y empaques, estrategias de cierre de ciclo, medición y reducción de huella de carbono en operaciones de producción/reciclaje</t>
+        </is>
+      </c>
+      <c r="W131" t="inlineStr">
+        <is>
+          <t>Ser empresa ubicada en jurisdicción de la CCB; comprometerse con aportar 10% de contrapartida; No especificado si hay requisitos de tamaño o sector</t>
+        </is>
+      </c>
+      <c r="X131" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y131" t="inlineStr">
+        <is>
+          <t>Empresas asociadas ANDI región Santander, empresas productoras de envases/empaques, empresas de consumo masivo con operaciones en Bucaramanga</t>
+        </is>
+      </c>
+      <c r="Z131" t="inlineStr">
+        <is>
+          <t>Solo 14 cupos disponibles (alta competencia); alcance territorial limitado a Bucaramanga y su área de influencia; información incompleta sobre requisitos y fechas de cierre</t>
+        </is>
+      </c>
+      <c r="AA131" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a la CCB para obtener términos de referencia completos, fecha de cierre y requisitos detallados. Identificar empresas asociadas en Santander interesadas.</t>
+        </is>
+      </c>
+      <c r="AB131" t="inlineStr">
+        <is>
+          <t>Llamar o escribir a CCB Bucaramanga para solicitar TdR, formulario de aplicación y cronograma completo antes de la fecha límite</t>
+        </is>
+      </c>
+      <c r="AC131" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y Coordinación de vinculación empresarial regional</t>
+        </is>
+      </c>
+      <c r="AD131" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE131" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF131" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG131" t="inlineStr">
+        <is>
+          <t>Fecha de publicación: hace 2 días (aprox. 8 mayo 2025). No se especifica fecha de cierre, lo que genera urgencia en verificación. Oportunidad regional con cofinanciación muy favorable (90%). Requiere verificar si empresas fuera de Bucaramanga pueden aplicar con operaciones locales. | Fuente fuera del listado oficial conocido (facebook.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH131" t="inlineStr">
+        <is>
+          <t>7961d7ae902c1f8d</t>
+        </is>
+      </c>
+      <c r="AI131" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>VC-0131</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Convocatoria regional para soluciones innovadoras en plásticos (Colombia, Chile y México)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Pacto por los Plásticos Colombia, Chile y México (en el marco de Pacto Global Red Colombia)</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Colombia / Regional (Chile, México)</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Colombia, Chile, México</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Plásticos flexibles, Envases y empaques, Innovación en reciclaje</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Hasta USD 10.000</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>https://www.pactoglobal-colombia.org/news/convocatoria-regional-otorgara-hasta-usd-10-000-a-soluciones-innovadoras-en-plasticos-en-colombia-chile-y-mexico.html</t>
+        </is>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>Convocatoria regional desarrollada por el Pacto por los Plásticos (Colombia, Chile, México) que otorga grants de hasta USD 10.000 para soluciones innovadoras que prevengan la contaminación por plásticos, con foco especial en plásticos flexibles (sachets, empaques multilaminados, etiquetas, bolsas). Publicada en noviembre de 2025, busca apoyar iniciativas de crecimiento y desarrollo en estos tres países.</t>
+        </is>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>Directamente alineada con el trabajo de Visión Circular en economía circular de envases y empaques, plásticos flexibles, reciclaje y cierre de ciclo. La convocatoria atiende desafíos de reciclabilidad y gestión de plásticos en los que ANDI trabaja activamente.</t>
+        </is>
+      </c>
+      <c r="V132" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje de plásticos flexibles; modelos de negocio circulares para sachets y multilaminados; innovación en ecodiseño de empaques flexibles; articulación empresarial para prevención de contaminación; escalamiento de soluciones empresariales de reciclabilidad</t>
+        </is>
+      </c>
+      <c r="W132" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X132" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y132" t="inlineStr">
+        <is>
+          <t>Empresas asociadas a ANDI (sector empaques, alimentos, consumo), Pacto por los Plásticos Colombia, organizaciones de recicladores, centros de innovación (Wrap Latam, universidades), Pacto Global Red Colombia</t>
+        </is>
+      </c>
+      <c r="Z132" t="inlineStr">
+        <is>
+          <t>Fecha de cierre no especificada en la fuente; monto limitado (USD 10.000); posible alta competencia regional. Requiere verificar si la convocatoria sigue abierta o próxima a abrir.</t>
+        </is>
+      </c>
+      <c r="AA132" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a Pacto Global Red Colombia y Pacto por los Plásticos Colombia para confirmar estado, plazos y términos de referencia de la convocatoria. Preparar propuesta enfocada en plásticos flexibles empresariales con componente de inclusión de recicladores.</t>
+        </is>
+      </c>
+      <c r="AB132" t="inlineStr">
+        <is>
+          <t>Llamar o escribir a Pacto Global Red Colombia esta semana para obtener términos de referencia, fecha de cierre y requisitos de elegibilidad. Identificar empresa ancla y piloto potencial.</t>
+        </is>
+      </c>
+      <c r="AC132" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Área de innovación y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD132" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE132" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF132" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG132" t="inlineStr">
+        <is>
+          <t>La fuente indica publicación en noviembre de 2025. No se especifica fecha de cierre ni si está abierta actualmente; se infiere que podría estar vigente o próxima a abrir dado que la publicación es reciente. Es altamente pertinente y Colombia es elegible directamente. | Fuente fuera del listado oficial conocido (pactoglobal-colombia.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH132" t="inlineStr">
+        <is>
+          <t>0bbb6afd5a58f527</t>
+        </is>
+      </c>
+      <c r="AI132" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>VC-0132</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Convocatoria de Cooperación Triangular y Sur-Sur - APC Colombia</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Agencia Presidencial de Cooperación Internacional de Colombia (APC-Colombia)</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Gobierno</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Colombia (entidades colombianas)</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Desarrollo sostenible (transversal)</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Fortalecimiento institucional, Intercambio de conocimiento, ODS</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>https://www.apccolombia.gov.co/seccion/modalidades-de-cooperacion?page=1</t>
+        </is>
+      </c>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>https://www.apccolombia.gov.co/modalidades-de-cooperacion/convocatorias</t>
+        </is>
+      </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>APC-Colombia recibe propuestas para intercambios de conocimiento, tecnología, métodos y metodologías orientados al desarrollo de comunidades y fortalecimiento de capacidades en entidades colombianas, con productos tangibles. Las iniciativas deben responder a los Objetivos de Desarrollo Sostenible.</t>
+        </is>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>Pertinente para fortalecer capacidades institucionales de Visión Circular en economía circular, transferencia de conocimiento en reciclaje, ecodiseño o modelos circulares desde experiencias internacionales. Permite articular cooperación triangular o sur-sur en temas de residuos, REP o inclusión de recicladores.</t>
+        </is>
+      </c>
+      <c r="V133" t="inlineStr">
+        <is>
+          <t>Intercambio de conocimiento en políticas de REP con países de la región; asistencia técnica en reciclaje de plásticos flexibles; transferencia de metodologías de economía circular territorial; fortalecimiento institucional de organizaciones de recicladores; cooperación con centros tecnológicos internacionales en ecodiseño</t>
+        </is>
+      </c>
+      <c r="W133" t="inlineStr">
+        <is>
+          <t>Propuestas deben orientarse a ODS, tener productos tangibles, enfoque en fortalecimiento de capacidades e intercambio de conocimiento. Aplicable a entidades colombianas.</t>
+        </is>
+      </c>
+      <c r="X133" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y133" t="inlineStr">
+        <is>
+          <t>APC-Colombia, agencias de cooperación de países con experiencia en economía circular (Países Bajos, Alemania, Chile, Uruguay), universidades, centros tecnológicos, gobiernos locales, gremios</t>
+        </is>
+      </c>
+      <c r="Z133" t="inlineStr">
+        <is>
+          <t>No se especifica convocatoria activa con fecha; es una modalidad permanente que requiere identificar ventanas de oportunidad. No hay monto ni financiamiento directo especificado; es cooperación técnica, no grant monetario.</t>
+        </is>
+      </c>
+      <c r="AA133" t="inlineStr">
+        <is>
+          <t>Revisar periódicamente el portal de APC-Colombia para convocatorias específicas abiertas. Preparar perfiles de proyecto de cooperación técnica en economía circular, reciclaje o REP para someter cuando se abran ventanas.</t>
+        </is>
+      </c>
+      <c r="AB133" t="inlineStr">
+        <is>
+          <t>Monitorear sección de convocatorias de APC-Colombia semanalmente. Contactar oficina de cooperación de APC para asesoría sobre formulación de propuestas en economía circular y residuos.</t>
+        </is>
+      </c>
+      <c r="AC133" t="inlineStr">
+        <is>
+          <t>Área de cooperación internacional / Coordinación de proyectos</t>
+        </is>
+      </c>
+      <c r="AD133" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE133" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF133" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG133" t="inlineStr">
+        <is>
+          <t>Es una modalidad de cooperación permanente, no una convocatoria específica con fecha de cierre. Requiere seguimiento continuo del portal de APC-Colombia para identificar convocatorias concretas. No es financiamiento monetario directo, sino cooperación técnica. Se incluye porque APC-Colombia es fuente oficial y la modalidad aplica a temas de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AH133" t="inlineStr">
+        <is>
+          <t>a2933a7ea89969fe</t>
+        </is>
+      </c>
+      <c r="AI133" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>VC-0133</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator Colombia 2026 – Call for Proposals</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator Colombia (programa liderado por embajadas de Reino Unido, Países Bajos y Alemania en alianza con gobierno colombiano)</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Colombia (programa internacional)</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Economía baja en carbono, proyectos climáticos escalables</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Aceleración; Cooperación técnica; Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>2026-01 (estimado primer trimestre 2026)</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>https://bogota.gov.co/boletin-oferta-internacional/climate-finance-accelerator-colombia-2026-acelera-proyectos-climatico</t>
+        </is>
+      </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DT_Qk01FT3L</t>
+        </is>
+      </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>El Climate Finance Accelerator Colombia 2026 abre convocatoria para acelerar proyectos climáticos de alto impacto que buscan prepararse para recibir inversión y escalar soluciones hacia una economía baja en carbono. Fortalece casos de inversión, estrategias de levantamiento de capital y relacionamiento con inversionistas. Sectores priorizados incluyen energías limpias, transporte y otros sectores climáticos.</t>
+        </is>
+      </c>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>Es directamente relevante para Visión Circular ANDI porque la economía circular es componente clave de la transición hacia economía baja en carbono. Proyectos de cierre de ciclo de envases, reciclaje y modelos de negocio circulares pueden posicionarse como soluciones climáticas escalables que requieren inversión.</t>
+        </is>
+      </c>
+      <c r="V134" t="inlineStr">
+        <is>
+          <t>Pilotos empresariales de reciclaje de plásticos flexibles con impacto climático medible; modelos de negocio circulares territoriales que reduzcan emisiones; escalamiento de tecnologías de reciclaje con inclusión de recicladores; casos de inversión para infraestructura de economía circular REP; ecodiseño para reducción de huella de carbono en envases y empaques</t>
+        </is>
+      </c>
+      <c r="W134" t="inlineStr">
+        <is>
+          <t>Proyectos climáticos de alto impacto, alineados con metas nacionales de Colombia, con potencial de escalamiento y preparados o en proceso de preparación para recibir inversión</t>
+        </is>
+      </c>
+      <c r="X134" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y134" t="inlineStr">
+        <is>
+          <t>Empresas asociadas ANDI (productores de envases/empaques), universidades con medición de impacto climático, organizaciones de recicladores, centros tecnológicos, entidades financieras interesadas en finanzas sostenibles</t>
+        </is>
+      </c>
+      <c r="Z134" t="inlineStr">
+        <is>
+          <t>Información limitada sobre requisitos específicos y fechas exactas; puede requerir demostración cuantitativa de impacto climático (reducción de emisiones) que debe estar previamente desarrollada; competencia con sectores energéticos tradicionales</t>
+        </is>
+      </c>
+      <c r="AA134" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente con los organizadores del CFA Colombia para obtener términos de referencia completos y calendario exacto. Preparar portafolio de 2-3 proyectos de Visión Circular con enfoque climático cuantificable (toneladas CO2 evitadas)</t>
+        </is>
+      </c>
+      <c r="AB134" t="inlineStr">
+        <is>
+          <t>Solicitar reunión informativa con CFA Colombia a través del punto de contacto de Bogotá.gov.co o embajadas participantes; mapear proyectos actuales de Visión Circular y calcular su potencial de mitigación climática</t>
+        </is>
+      </c>
+      <c r="AC134" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas, con apoyo de área técnica para cuantificación de impacto climático</t>
+        </is>
+      </c>
+      <c r="AD134" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE134" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF134" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG134" t="inlineStr">
+        <is>
+          <t>Convocatoria confirmada para 2026 pero sin fecha exacta de cierre. La fuente oficial (Bogotá.gov.co) y redes sociales confirman su vigencia. Se infiere elegibilidad de organizaciones gremiales y empresariales pero debe verificarse. Los sectores priorizados mencionados en Instagram incluyen energía y transporte, pero la economía circular puede encajar como solución transversal climática | Fuente fuera del listado oficial conocido (bogota.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH134" t="inlineStr">
+        <is>
+          <t>95213494d36c7a7c</t>
+        </is>
+      </c>
+      <c r="AI134" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>VC-0134</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Movilización de recursos CAF y aliados para acción climática, sostenibilidad y biodiversidad en Colombia hasta 2026</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>CAF - Banco de Desarrollo de América Latina, en alianza con KfW, BCIE, OPEC Fund y otras instituciones</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>América Latina (CAF regional)</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Acción climática, sostenibilidad, biodiversidad</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Cofinanciación; Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>USD 1.400 millones (total hasta 2026: USD 700 millones de CAF + USD 700 millones de aliados)</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>Probable (según estructura típica CAF)</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>2026-12-31 (hasta 2026)</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DOjlZoqAUon</t>
+        </is>
+      </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>CAF lidera la movilización conjunta de USD 1.400 millones hasta 2026 para impulsar acción climática, sostenibilidad y biodiversidad en Colombia, en alianza con KfW, BCIE, OPEC Fund y otras instituciones. CAF aporta al menos USD 700 millones y el resto proviene de aliados. Representa la movilización de recursos más importante del año para Colombia en temas ambientales y climáticos.</t>
+        </is>
+      </c>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>Altamente relevante porque la economía circular es eje transversal de sostenibilidad y acción climática. Los proyectos de gestión de residuos, reciclaje y cierre de ciclo de envases/empaques contribuyen directamente a objetivos climáticos y de sostenibilidad que este financiamiento busca impulsar en Colombia.</t>
+        </is>
+      </c>
+      <c r="V135" t="inlineStr">
+        <is>
+          <t>Infraestructura de reciclaje y valorización de residuos con impacto climático; escalamiento de sistemas REP para envases y empaques; modelos territoriales de economía circular con inclusión de recicladores; inversión en tecnología de reciclaje de plásticos flexibles; fortalecimiento de cadenas de valor circulares empresariales con componente de biodiversidad (ej. bioeconomía circular)</t>
+        </is>
+      </c>
+      <c r="W135" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X135" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y135" t="inlineStr">
+        <is>
+          <t>Empresas asociadas ANDI, gobiernos locales y territoriales, organizaciones de recicladores formalizadas, universidades para componentes de I+D, entidades financieras colombianas como co-ejecutores, cooperación alemana (KfW) para articulación técnica</t>
+        </is>
+      </c>
+      <c r="Z135" t="inlineStr">
+        <is>
+          <t>Información muy limitada (solo post de Instagram); no hay convocatoria específica identificada sino anuncio de disponibilidad general de recursos; probablemente requiere estructuración financiera robusta y garantías; competencia con proyectos de infraestructura grande; no está claro el mecanismo de acceso (si es vía gobierno, empresas, banca local u otros)</t>
+        </is>
+      </c>
+      <c r="AA135" t="inlineStr">
+        <is>
+          <t>Contactar a la oficina CAF Colombia para identificar ventanas específicas de financiamiento dentro de esta movilización de recursos que apliquen para proyectos de economía circular y gestión de residuos. Explorar articulación con KfW (cooperación alemana) que tiene experiencia en economía circular</t>
+        </is>
+      </c>
+      <c r="AB135" t="inlineStr">
+        <is>
+          <t>Solicitar reunión con representante CAF Colombia y con agregaduría de cooperación alemana (KfW) para explorar líneas específicas disponibles; preparar pipeline de proyectos de Visión Circular estructurados financieramente</t>
+        </is>
+      </c>
+      <c r="AC135" t="inlineStr">
+        <is>
+          <t>Dirección ejecutiva y área de alianzas estratégicas (nivel senior para relacionamiento con banca multilateral)</t>
+        </is>
+      </c>
+      <c r="AD135" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE135" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF135" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG135" t="inlineStr">
+        <is>
+          <t>Anuncio confirmado de movilización de recursos muy significativa (USD 1.400 millones), pero la fuente es únicamente redes sociales sin enlace a convocatoria o mecanismo de acceso específico. Se infiere que existen ventanas de financiamiento disponibles pero no están detalladas. La elegibilidad de Visión Circular/ANDI debe verificarse: probablemente requiere canalización vía gobierno, empresas grandes o banca local. El monto y respaldo institucional justifican su inclusión pese a información limitada | Fuente fuera del listado oficial conocido (instagram.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH135" t="inlineStr">
+        <is>
+          <t>6893d93ad7ad0503</t>
+        </is>
+      </c>
+      <c r="AI135" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>VC-0135</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Premios Ambientales CAR - Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Corporación Autónoma Regional de Cundinamarca (CAR)</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Gobierno</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Colombia - Jurisdicción CAR Cundinamarca</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Medio ambiente y sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Protección ambiental, recuperación, sostenibilidad territorial</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Otro</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>https://www.colombialider.org/carpremiacion</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>El Premio Ambiental CAR reconoce y visibiliza experiencias, proyectos y liderazgos que contribuyen a la protección, recuperación y sostenibilidad ambiental en la jurisdicción de la CAR Cundinamarca. Busca destacar buenas prácticas locales con impacto ambiental positivo.</t>
+        </is>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular si opera en Cundinamarca o tiene proyectos demostrativos de economía circular, reciclaje, gestión de residuos de envases o inclusión de recicladores en esta jurisdicción. Permite visibilizar experiencias piloto territoriales.</t>
+        </is>
+      </c>
+      <c r="V136" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje de envases en municipios de Cundinamarca; modelos de economía circular territorial; inclusión de recicladores en sistemas formales; proyectos de ecodiseño y cierre de ciclo con empresas locales</t>
+        </is>
+      </c>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X136" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y136" t="inlineStr">
+        <is>
+          <t>Empresas ANDI con operaciones en Cundinamarca, organizaciones de recicladores, municipios, universidades de la región (Uniandes, U. Nacional, U. La Sabana)</t>
+        </is>
+      </c>
+      <c r="Z136" t="inlineStr">
+        <is>
+          <t>Elegibilidad limitada a jurisdicción CAR Cundinamarca; falta información sobre plazos, montos, requisitos y estado actual de convocatoria</t>
+        </is>
+      </c>
+      <c r="AA136" t="inlineStr">
+        <is>
+          <t>Verificar inmediatamente si hay convocatoria abierta 2025, montos, categorías y si proyectos de economía circular/reciclaje/envases son elegibles</t>
+        </is>
+      </c>
+      <c r="AB136" t="inlineStr">
+        <is>
+          <t>Contactar a CAR Cundinamarca vía web o telefónicamente para confirmar vigencia, bases y plazos 2025</t>
+        </is>
+      </c>
+      <c r="AC136" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos territoriales / Alianzas institucionales</t>
+        </is>
+      </c>
+      <c r="AD136" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE136" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF136" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG136" t="inlineStr">
+        <is>
+          <t>La fuente confirma la existencia del premio pero no proporciona fechas, montos ni estado de convocatoria 2025. La jurisdicción es limitada a Cundinamarca, pero incluye Bogotá y Sabana. Requiere verificación urgente de vigencia. | Fuente fuera del listado oficial conocido (colombialider.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH136" t="inlineStr">
+        <is>
+          <t>3faaa44c70ff02ae</t>
+        </is>
+      </c>
+      <c r="AI136" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>VC-0136</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Premios Verdes 2026 - Ranking 500 Mejores Proyectos Socioambientales</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Premios Verdes</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>América Latina (regional)</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>América Latina - Colombia, Ecuador, Perú, Bolivia, México y otros países de la región</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Medio ambiente y sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Soluciones a desafíos ambientales, sociales y climáticos</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>Aprox. iniciado 2025</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>Aprox. 2026 (proceso en curso hacia anuncio de finalistas)</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DZJNwyPkQJE</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>Premios Verdes reveló el Ranking de los 500 Mejores Proyectos Socioambientales edición 2026, con Colombia liderando entre los países seleccionados. El proceso avanza hacia el anuncio de finalistas y busca identificar soluciones concretas a desafíos ambientales, sociales y climáticos.</t>
+        </is>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular: permite posicionar proyectos de economía circular, reciclaje, gestión de envases, inclusión de recicladores y modelos de negocio circulares a nivel latinoamericano, generando visibilidad regional y networking estratégico.</t>
+        </is>
+      </c>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>Cierre de ciclo de envases y empaques; innovación en reciclaje de plásticos flexibles; inclusión y formalización de recicladores; pilotos empresariales de economía circular; ecodiseño y reciclabilidad; cumplimiento REP</t>
+        </is>
+      </c>
+      <c r="W137" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X137" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y137" t="inlineStr">
+        <is>
+          <t>Empresas ANDI con proyectos innovadores, organizaciones de recicladores, universidades, centros tecnológicos, cooperación internacional</t>
+        </is>
+      </c>
+      <c r="Z137" t="inlineStr">
+        <is>
+          <t>Fuente es Instagram (no sitio web oficial); falta información sobre plazos exactos de inscripción, requisitos, categorías, y si aún está abierta la convocatoria o si el ranking ya está cerrado</t>
+        </is>
+      </c>
+      <c r="AA137" t="inlineStr">
+        <is>
+          <t>Buscar el sitio web oficial de Premios Verdes, confirmar plazos de postulación 2026, categorías aplicables a economía circular y si Visión Circular o sus proyectos asociados pueden postularse</t>
+        </is>
+      </c>
+      <c r="AB137" t="inlineStr">
+        <is>
+          <t>Acceder a www.premiosverdes.org (o sitio oficial) para verificar bases, plazos y proceso de postulación edición 2026</t>
+        </is>
+      </c>
+      <c r="AC137" t="inlineStr">
+        <is>
+          <t>Comunicaciones y posicionamiento / Gestión de conocimiento</t>
+        </is>
+      </c>
+      <c r="AD137" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE137" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF137" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG137" t="inlineStr">
+        <is>
+          <t>La fuente es una red social, lo que limita la confiabilidad y detalle. Se infiere que el proceso está en curso (edición 2026), pero se requiere confirmar si aún hay ventana de postulación o si ya se cerró. Colombia es país elegible destacado. | Fuente fuera del listado oficial conocido (instagram.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH137" t="inlineStr">
+        <is>
+          <t>36bf68979ab8fcaf</t>
+        </is>
+      </c>
+      <c r="AI137" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>VC-0137</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Premio Ambiental Gemas Colombia 2026</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Premio Gemas</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Medio ambiente y sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Proyectos ambientales, protección del medio ambiente</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>https://premiogemas.co</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>El Premio Ambiental Gemas es un portafolio de estímulos a proyectos ambientales desarrollados en Colombia. Reconoce y exalta la labor de personas y organizaciones que contribuyen a la protección del medio ambiente. El sitio invita a postularse pero no especifica plazos ni detalles de la convocatoria vigente.</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular si acepta proyectos de economía circular, reciclaje, gestión de residuos y envases. Permite visibilizar iniciativas de circularidad y generar reconocimiento nacional para el programa y sus aliados.</t>
+        </is>
+      </c>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>Proyectos de reciclaje y valorización de envases; inclusión de recicladores; innovación en ecodiseño; pilotos de economía circular empresarial; modelos territoriales de cierre de ciclo</t>
+        </is>
+      </c>
+      <c r="W138" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y138" t="inlineStr">
+        <is>
+          <t>Empresas ANDI, organizaciones de recicladores, municipios, ONGs ambientales, universidades colombianas</t>
+        </is>
+      </c>
+      <c r="Z138" t="inlineStr">
+        <is>
+          <t>Falta total de información sobre plazos, requisitos, categorías, montos o tipo de estímulo. Sitio web con información muy general y sin bases claras de convocatoria vigente</t>
+        </is>
+      </c>
+      <c r="AA138" t="inlineStr">
+        <is>
+          <t>Acceder al sitio web oficial, buscar sección de postulación o contacto, y verificar si hay convocatoria 2025 o 2026 abierta, categorías, y si economía circular es elegible</t>
+        </is>
+      </c>
+      <c r="AB138" t="inlineStr">
+        <is>
+          <t>Explorar menú completo del sitio web premiogemas.co y buscar información de contacto para solicitar bases y cronograma 2025-2026</t>
+        </is>
+      </c>
+      <c r="AC138" t="inlineStr">
+        <is>
+          <t>Gestión de conocimiento / Comunicaciones</t>
+        </is>
+      </c>
+      <c r="AD138" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE138" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF138" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG138" t="inlineStr">
+        <is>
+          <t>El sitio web existe pero la fuente proporcionada es muy genérica. No se confirma si hay convocatoria activa, ni fechas, ni categorías específicas. Se infiere que es un premio recurrente pero sin datos operativos actuales. | Fuente fuera del listado oficial conocido (premiogemas.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH138" t="inlineStr">
+        <is>
+          <t>e692cf7bbfe2a077</t>
+        </is>
+      </c>
+      <c r="AI138" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>VC-0138</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>21.º Premio Andesco a la Sostenibilidad</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Asociación Nacional de Empresas de Servicios Públicos y Comunicaciones (Andesco)</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Colombia - empresas y organizaciones del país</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Sostenibilidad empresarial</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Iniciativas de sostenibilidad, responsabilidad, innovación, impacto positivo</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>Abierta (según fuente)</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>https://www.pactoglobal-colombia.org/news/ya-esta-abierta-la-convocatoria-al-21-o-premio-andesco-a-la-sostenibilidad.html</t>
+        </is>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>Andesco invita a empresas y organizaciones de Colombia a postular proyectos al 21.º Premio Andesco a la Sostenibilidad, reconocimiento que destaca organizaciones liderando la transformación del país con iniciativas de sostenibilidad responsables, innovadoras y de impacto positivo. La convocatoria está abierta.</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI: permite postular proyectos empresariales de economía circular, reciclaje, gestión de envases, cumplimiento REP, inclusión de recicladores y modelos de negocio circulares. Andesco es gremio clave aliado de ANDI.</t>
+        </is>
+      </c>
+      <c r="V139" t="inlineStr">
+        <is>
+          <t>Pilotos empresariales de economía circular; innovación en reciclaje y valorización de envases; cumplimiento de REP; inclusión y formalización de recicladores; ecodiseño y reciclabilidad; modelos circulares territoriales</t>
+        </is>
+      </c>
+      <c r="W139" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y139" t="inlineStr">
+        <is>
+          <t>Empresas asociadas a ANDI y Andesco (servicios públicos, manufactura, consumo masivo), organizaciones de recicladores, universidades, centros tecnológicos</t>
+        </is>
+      </c>
+      <c r="Z139" t="inlineStr">
+        <is>
+          <t>Falta información sobre fecha límite, categorías específicas, requisitos de elegibilidad, y si proyectos de economía circular/reciclaje tienen categoría propia o entran en categoría genérica de sostenibilidad</t>
+        </is>
+      </c>
+      <c r="AA139" t="inlineStr">
+        <is>
+          <t>Contactar urgentemente a Andesco o revisar bases completas en su sitio oficial para confirmar fecha límite, categorías, requisitos y proceso de postulación</t>
+        </is>
+      </c>
+      <c r="AB139" t="inlineStr">
+        <is>
+          <t>Acceder al sitio web oficial de Andesco (www.andesco.org.co) para descargar bases, identificar categoría aplicable y preparar postulación con casos empresariales de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AC139" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Alianzas empresariales</t>
+        </is>
+      </c>
+      <c r="AD139" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE139" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF139" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG139" t="inlineStr">
+        <is>
+          <t>La convocatoria está confirmada como abierta por fuente confiable (Pacto Global Red Colombia). Sin embargo, no se proporciona fecha límite ni enlace directo a bases. Andesco es aliado estratégico de ANDI, lo que aumenta probabilidad de aplicación exitosa. | Fuente fuera del listado oficial conocido (pactoglobal-colombia.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH139" t="inlineStr">
+        <is>
+          <t>7bbcea32e12b22ca</t>
+        </is>
+      </c>
+      <c r="AI139" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>VC-0139</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia Innovation Challenge</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>AgriTech Challenge (plataforma organizadora; financiadores específicos no identificados en la fuente)</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Internacional (enfocado en Colombia)</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Sector agroalimentario, innovación en circularidad</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Aceleración; Innovación; Otro</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>Challenge de innovación dirigido a acelerar la transición hacia una economía circular en el sector agroalimentario de Colombia, alineado con el Plan Nacional de Desarrollo 2022-2026 y los objetivos de la COP 16 CBD Colombia. Ofrece mentoría especializada y acceso a recursos para soluciones innovadoras en circularidad agroalimentaria.</t>
+        </is>
+      </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>Directamente alineado con los objetivos de economía circular y modelos de negocio circulares de Visión Circular. Aunque el enfoque principal es agroalimentario, los envases y empaques de alimentos son un área clave del programa ANDI, incluyendo reciclaje, ecodiseño y cierre de ciclo de estos materiales.</t>
+        </is>
+      </c>
+      <c r="V140" t="inlineStr">
+        <is>
+          <t>Desarrollo de sistemas de envases retornables para alimentos; ecodiseño de empaques agroalimentarios reciclables; pilotos de cierre de ciclo de empaques flexibles en cadenas agroindustriales; modelos de negocio circular con empresas del sector alimentario; inclusión de recicladores en cadenas agroalimentarias</t>
+        </is>
+      </c>
+      <c r="W140" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X140" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y140" t="inlineStr">
+        <is>
+          <t>Empresas del sector agroalimentario asociadas a ANDI, universidades con programas en ingeniería de alimentos y sostenibilidad, centros tecnológicos especializados en empaques, gremios del sector agroindustrial</t>
+        </is>
+      </c>
+      <c r="Z140" t="inlineStr">
+        <is>
+          <t>Información limitada sobre plazos, montos y requisitos específicos. Enfoque sectorial puede limitar aplicabilidad si no se vincula con envases/empaques alimentarios. Posible competencia alta dado el perfil de innovación.</t>
+        </is>
+      </c>
+      <c r="AA140" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a los organizadores del challenge para verificar estado de convocatoria, plazos, requisitos específicos y posibilidad de presentar proyectos enfocados en envases y empaques circulares para el sector agroalimentario.</t>
+        </is>
+      </c>
+      <c r="AB140" t="inlineStr">
+        <is>
+          <t>Enviar correo o completar formulario de contacto en la plataforma AgriTech Challenge solicitando información detallada sobre fechas, requisitos y elegibilidad para proyectos de economía circular en envases agroalimentarios.</t>
+        </is>
+      </c>
+      <c r="AC140" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD140" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE140" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF140" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG140" t="inlineStr">
+        <is>
+          <t>La fuente confirma la existencia del challenge y su alineación con políticas colombianas, pero no proporciona información sobre fechas límite, montos, estado actual de la convocatoria o requisitos específicos. Se infiere que podría estar activa o próxima a abrir dado que la página está publicada, pero requiere verificación urgente. El enfoque agroalimentario es complementario a las líneas de Visión Circular en envases y empaques de alimentos. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH140" t="inlineStr">
+        <is>
+          <t>b4970efa6f5674e3</t>
+        </is>
+      </c>
+      <c r="AI140" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>VC-0140</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Líneas de financiamiento circular - IDB Invest (propuesta en desarrollo)</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>BID Invest (Grupo Banco Interamericano de Desarrollo)</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Multilateral - América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Productos y materiales de base biológica, reciclaje a gran escala, plataformas digitales circulares</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Cofinanciación; Investigación aplicada</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>https://idbinvest.org/en/download/19683</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>https://idbinvest.org/en/blog/transport/case-unlocking-circular-economy-latin-america-and-caribbean</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>Documento estratégico de IDB Invest propone crear líneas de financiamiento circular enfocadas en proyectos prioritarios pre-definidos para la región LAC: productos/materiales de base biológica, reciclaje a gran escala y plataformas digitales. Sigue el sistema de categorización de economía circular de la Comisión Europea. El documento analiza el potencial de desbloquear negocios circulares en LAC con estimación de $1 trillón USD de valor económico global para 2025.</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>Altamente relevante: propone financiamiento específico para reciclaje a gran escala y plataformas digitales, alineado directamente con el trabajo de Visión Circular en cierre de ciclo de envases, escalamiento de reciclaje y modelos de negocio circulares en Colombia.</t>
+        </is>
+      </c>
+      <c r="V141" t="inlineStr">
+        <is>
+          <t>Proyectos de reciclaje de envases a gran escala (plásticos flexibles); plataformas digitales de trazabilidad para cumplimiento REP; infraestructura regional de reciclaje químico; modelos de negocio circulares con inclusión de recicladores; sistemas territoriales de economía circular escalables.</t>
+        </is>
+      </c>
+      <c r="W141" t="inlineStr">
+        <is>
+          <t>No especificado - documento es propuesta estratégica, no convocatoria activa. Probablemente requiere proyectos con viabilidad económica, escala significativa y alineación con categorías priorizadas.</t>
+        </is>
+      </c>
+      <c r="X141" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y141" t="inlineStr">
+        <is>
+          <t>BID Invest como financiador principal, empresas grandes de ANDI como anclas, cooperativas de recicladores como beneficiarios, gobiernos locales para componente territorial, universidades para medición de impacto</t>
+        </is>
+      </c>
+      <c r="Z141" t="inlineStr">
+        <is>
+          <t>Es una propuesta estratégica, no una convocatoria activa confirmada. No hay información sobre instrumentos específicos, requisitos o calendario de implementación. Puede requerir proyectos de gran escala que excedan capacidad de un solo actor.</t>
+        </is>
+      </c>
+      <c r="AA141" t="inlineStr">
+        <is>
+          <t>Contactar al equipo de Economía Circular y Sostenibilidad de IDB Invest para conocer el estado de implementación de estas líneas y requisitos para acceder. Pre-identificar 1-2 proyectos emblemáticos de gran escala del ecosistema Visión Circular que puedan calificar.</t>
+        </is>
+      </c>
+      <c r="AB141" t="inlineStr">
+        <is>
+          <t>Buscar contacto directo en IDB Invest LAC (departamento de Sostenibilidad o Economía Circular). Solicitar reunión exploratoria sobre oportunidades de financiamiento para proyectos circulares en Colombia.</t>
+        </is>
+      </c>
+      <c r="AC141" t="inlineStr">
+        <is>
+          <t>Dirección de Visión Circular / Alianzas estratégicas con banca multilateral</t>
+        </is>
+      </c>
+      <c r="AD141" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE141" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF141" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG141" t="inlineStr">
+        <is>
+          <t>El documento es de alta pertinencia temática pero no es una convocatoria activa sino una propuesta de política. Se infiere que IDB Invest está desarrollando estos instrumentos pero no hay confirmación de disponibilidad actual. La fecha del documento no está clara en los resultados de búsqueda.</t>
+        </is>
+      </c>
+      <c r="AH141" t="inlineStr">
+        <is>
+          <t>18abb1d98021e3c9</t>
+        </is>
+      </c>
+      <c r="AI141" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>VC-0141</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Blue Tech for Waste Challenge</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>BID Lab (Banco Interamericano de Desarrollo)</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Regional (América Latina y el Caribe)</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Caribe y América Latina (inferido por contexto regional del BID)</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Residuos, modelos de negocio circulares, escalamiento</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Financiamiento concesional; Asistencia técnica; Piloto demostrativo; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/blog/water-sanitation-and-solid-waste/transforming-hazardous-waste-circular-economy-caribbean</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>El BID Lab lidera el Blue Tech for Waste Challenge, que ofrece grants, financiamiento catalítico o convertible y soporte técnico para pilotar y escalar modelos circulares, conformes y generadores de empleo en el sector residuos. La iniciativa ha recibido cerca de 100 propuestas desde su lanzamiento, evidenciando fuerte interés regional.</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular por su enfoque en modelos de negocio circulares, escalamiento de soluciones de residuos, y potencial de articulación con empresas para cierre de ciclo de materiales, alineado con REP y economía circular territorial.</t>
+        </is>
+      </c>
+      <c r="V142" t="inlineStr">
+        <is>
+          <t>Escalamiento de pilotos de reciclaje de envases flexibles; modelos de negocio circulares con inclusión de recicladores; proyectos de valorización de residuos plásticos con empresas ANDI; soluciones tecnológicas para trazabilidad y circularidad de empaques</t>
+        </is>
+      </c>
+      <c r="W142" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X142" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y142" t="inlineStr">
+        <is>
+          <t>Empresas ANDI, startups de reciclaje, cooperativas de recicladores, universidades para validación técnica, gremios sectoriales</t>
+        </is>
+      </c>
+      <c r="Z142" t="inlineStr">
+        <is>
+          <t>No se especifica estado de convocatoria actual (si está abierta o cerrada); requiere confirmación de elegibilidad para Colombia específicamente</t>
+        </is>
+      </c>
+      <c r="AA142" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a BID Lab para confirmar estado de la convocatoria, criterios de elegibilidad para Colombia y ventanas de aplicación 2025</t>
+        </is>
+      </c>
+      <c r="AB142" t="inlineStr">
+        <is>
+          <t>Enviar correo a BID Lab solicitando información sobre próximas ventanas del Blue Tech for Waste Challenge y requisitos de elegibilidad para Colombia</t>
+        </is>
+      </c>
+      <c r="AC142" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD142" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE142" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF142" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG142" t="inlineStr">
+        <is>
+          <t>La fuente confirma existencia del programa y su enfoque, pero no especifica fechas de convocatoria ni montos. Se infiere elegibilidad de Colombia por ser país miembro del BID y contexto regional mencionado. Requiere validación de ventanas activas.</t>
+        </is>
+      </c>
+      <c r="AH142" t="inlineStr">
+        <is>
+          <t>6a539a5115a187c6</t>
+        </is>
+      </c>
+      <c r="AI142" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>VC-0142</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Too Good to Waste - Convocatoria para estudios de preinversión en gestión de residuos sólidos</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Banco Interamericano de Desarrollo (BID)</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Regional (América Latina y el Caribe)</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>20 países de América Latina y el Caribe (Colombia incluido, inferido por volumen de propuestas regionales)</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Residuos</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Economía circular, valorización de residuos, cierre de rellenos, biogas, gestión municipal de residuos</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Investigación aplicada; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Demanda total superó USD 35 millones en 2024</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>2024 (convocatoria cerrada)</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>2024 (convocatoria cerrada)</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/who-we-are/topics/water-and-sanitation/initiatives/too-good-waste</t>
+        </is>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>En 2024, el BID lanzó convocatoria para apoyar estudios de preinversión requeridos en proyectos de gestión de residuos sólidos para economía circular y menores emisiones. Se recibieron 230 propuestas de 20 países: 194 enfocadas en valorización, 18 en prevención y 18 en cierre de rellenos o biogas, evidenciando alta demanda regional por preparación de proyectos.</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular por el enfoque en valorización de residuos y economía circular, aplicable a proyectos territoriales de gestión de envases y empaques, y potencial soporte técnico para estructuración de proyectos empresariales o municipales de reciclaje.</t>
+        </is>
+      </c>
+      <c r="V143" t="inlineStr">
+        <is>
+          <t>Estudios de preinversión para plantas de valorización de envases post-consumo; proyectos de economía circular territorial con municipios; estructuración de proyectos de REP a nivel regional; análisis de viabilidad de modelos de reciclaje inclusivo</t>
+        </is>
+      </c>
+      <c r="W143" t="inlineStr">
+        <is>
+          <t>Proyectos de gestión de residuos sólidos orientados a economía circular y reducción de emisiones; necesidad de estudios de preinversión</t>
+        </is>
+      </c>
+      <c r="X143" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y143" t="inlineStr">
+        <is>
+          <t>Municipios, autoridades ambientales, empresas ANDI con necesidades de cumplimiento REP, universidades para componente técnico, asociaciones de recicladores</t>
+        </is>
+      </c>
+      <c r="Z143" t="inlineStr">
+        <is>
+          <t>La convocatoria 2024 está cerrada; no se confirma si habrá nueva edición en 2025</t>
+        </is>
+      </c>
+      <c r="AA143" t="inlineStr">
+        <is>
+          <t>Contactar al BID para conocer si habrá nueva convocatoria Too Good to Waste en 2025 y preparar cartera de proyectos de economía circular territorial con empresas ANDI</t>
+        </is>
+      </c>
+      <c r="AB143" t="inlineStr">
+        <is>
+          <t>Enviar solicitud de información al BID sobre próxima convocatoria 2025 y explorar posibilidad de diálogo técnico para preparar propuestas conjuntas ANDI-empresas-municipios</t>
+        </is>
+      </c>
+      <c r="AC143" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y relaciones institucionales con banca multilateral</t>
+        </is>
+      </c>
+      <c r="AD143" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE143" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF143" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG143" t="inlineStr">
+        <is>
+          <t>Convocatoria 2024 ya cerrada, pero el alto volumen de propuestas (230) y demanda superior a USD 35 millones sugiere alta probabilidad de nueva edición. Colombia es elegible como país miembro del BID. Se recomienda monitoreo activo para 2025.</t>
+        </is>
+      </c>
+      <c r="AH143" t="inlineStr">
+        <is>
+          <t>25329b546cf65b47</t>
+        </is>
+      </c>
+      <c r="AI143" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>VC-0143</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>BlueTech for Waste - Caribbean Circular Economy Initiative</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Grupo BID (BID Lab) en alianza con Circulate Capital</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Estados Unidos (BID) / Estados Unidos (Circulate Capital)</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Región del Caribe</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Economía circular y gestión de residuos</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Plásticos océano-bound, tecnologías innovadoras de residuos, economía circular del Caribe</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Inversión; Fortalecimiento institucional; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>https://openidb.brightidea.com/BlueTechforWaste</t>
+        </is>
+      </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/news/idb-lab-partners-circulate-capital-combat-ocean-bound-plastics</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>Iniciativa de sourcing del Grupo BID dirigida al sector privado del Caribe para promover gestión ambientalmente sana de residuos de construcción y demolición mediante tecnologías innovadoras y procesos de economía circular. Incluye un programa de desarrollo de capacidades para fortalecer el pipeline de inversión en la región del Caribe, gestionado por Circulate Capital.</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>Altamente pertinente por su enfoque en economía circular, gestión de residuos plásticos océano-bound, innovación en tecnologías de reciclaje y fortalecimiento de ecosistemas de inversión circular. Modelo replicable para Colombia en gestión de residuos y plásticos, con potencial de articulación regional.</t>
+        </is>
+      </c>
+      <c r="V144" t="inlineStr">
+        <is>
+          <t>Transferencia de aprendizajes del modelo Caribe a Colombia; desarrollo de tecnologías para residuos de construcción y demolición con enfoque circular; articulación con Circulate Capital para pipeline de inversión en Colombia; pilotos empresariales de gestión de plásticos océano-bound en zonas costeras colombianas; modelos de negocio circulares para materiales de construcción reciclados</t>
+        </is>
+      </c>
+      <c r="W144" t="inlineStr">
+        <is>
+          <t>Enfocado en sector privado del Caribe; requiere tecnologías innovadoras y enfoque de economía circular; debe abordar gestión de construcción y residuos</t>
+        </is>
+      </c>
+      <c r="X144" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y144" t="inlineStr">
+        <is>
+          <t>Circulate Capital como gestor de inversión; empresas colombianas del sector construcción con operaciones en Caribe; gremios de construcción CAMACOL; organizaciones regionales del Caribe; potencial articulación con ANDI para réplica en Colombia continental</t>
+        </is>
+      </c>
+      <c r="Z144" t="inlineStr">
+        <is>
+          <t>Enfoque geográfico limitado al Caribe, Colombia continental podría no ser elegible directamente; no hay fechas confirmadas; información sobre vigencia de la convocatoria no está clara</t>
+        </is>
+      </c>
+      <c r="AA144" t="inlineStr">
+        <is>
+          <t>Verificar si Colombia (región Caribe colombiano: Cartagena, Barranquilla, Santa Marta, San Andrés) es elegible; contactar a BID Lab y Circulate Capital para explorar réplica del modelo o participación de actores colombianos; identificar empresas ANDI en región Caribe para aplicación</t>
+        </is>
+      </c>
+      <c r="AB144" t="inlineStr">
+        <is>
+          <t>Acceder a la plataforma BrightIdea del BID para confirmar términos de elegibilidad y fechas; contactar al punto focal de BID Lab Colombia para indagar sobre extensión del programa al Caribe colombiano</t>
+        </is>
+      </c>
+      <c r="AC144" t="inlineStr">
+        <is>
+          <t>Alianzas estratégicas y movilización de recursos con banca multilateral</t>
+        </is>
+      </c>
+      <c r="AD144" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE144" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF144" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG144" t="inlineStr">
+        <is>
+          <t>La iniciativa combina inversión con desarrollo de capacidades. Aunque está enfocada en el Caribe, la región Caribe de Colombia podría ser elegible. La asociación con Circulate Capital (especialista en plásticos oceánicos) es estratégica. Se infiere que es una convocatoria o sourcing activo por el portal BrightIdea del BID, pero no hay fechas explícitas. | Fuente fuera del listado oficial conocido (openidb.brightidea.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH144" t="inlineStr">
+        <is>
+          <t>23c326c8df38d0ed</t>
+        </is>
+      </c>
+      <c r="AI144" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>VC-0144</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF) - Financiamiento Climático para Colombia</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (Fondo Verde para el Clima)</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Internacional (mecanismo UNFCCC, sede Corea del Sur)</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Colombia y otros países en desarrollo</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Mitigación y adaptación climática, desarrollo bajo en emisiones, resiliencia climática</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Grant no reembolsable; Financiamiento concesional; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>364 millones USD aprobados para Colombia hasta la fecha (15 proyectos); monto disponible para nuevas propuestas: No especificado</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>Sí, típicamente requerida según modalidad de proyecto</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente (ventanas de evaluación periódicas)</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/countries/colombia</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>https://openei.org/wiki/Colombia-Climate_Finance_Readiness_Programme</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>El Fondo Verde para el Clima (GCF) mantiene una ventana permanente de financiamiento para Colombia, con $364M USD ya aprobados en 15 proyectos. El GCF financia proyectos de mitigación y adaptación climática, con enfoque en transformación hacia economías bajas en carbono. Colombia cuenta con un Readiness Programme apoyado por UNDP, UNEP y WRI (financiado por el BMU alemán) para fortalecer capacidades de acceso, gestión y despliegue de recursos del GCF.</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular ya que la economía circular es reconocida como estrategia de mitigación climática (reducción de emisiones en producción, gestión de residuos y cierre de ciclos materiales). Proyectos de reciclaje, gestión de residuos orgánicos, ecodiseño y modelos circulares son elegibles bajo las ventanas de mitigación del GCF.</t>
+        </is>
+      </c>
+      <c r="V145" t="inlineStr">
+        <is>
+          <t>Economía circular como estrategia de mitigación climática en sector envases/empaques; gestión de residuos sólidos con reducción de emisiones de metano; fortalecimiento de cadenas de reciclaje inclusivo con co-beneficios climáticos; transformación industrial hacia producción circular baja en carbono; pilotos de bioeconomía circular en gestión de residuos orgánicos; escalamiento de modelos REP con impacto climático medible</t>
+        </is>
+      </c>
+      <c r="W145" t="inlineStr">
+        <is>
+          <t>Proyectos deben demostrar impacto climático (mitigación o adaptación); alineación con NDC de Colombia; presentación a través de Entidad Nacional Designada (Ministerio de Ambiente) o Entidades Acreditadas (ej. PNUD, FINDETER, CAF); sostenibilidad financiera y técnica del proyecto</t>
+        </is>
+      </c>
+      <c r="X145" t="inlineStr">
+        <is>
+          <t>Concept Note según formato GCF; evaluación de impacto climático; análisis de co-beneficios ambientales y sociales; presupuesto detallado; plan de sostenibilidad; cartas de respaldo institucional; análisis de género y salvaguardas ambientales y sociales</t>
+        </is>
+      </c>
+      <c r="Y145" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible (Entidad Nacional Designada GCF Colombia); FINDETER (entidad acreditada nacional); PNUD Colombia; CAF; Corporaciones Autónomas Regionales; universidades; empresas ANDI con compromisos climáticos; gremios sectoriales</t>
+        </is>
+      </c>
+      <c r="Z145" t="inlineStr">
+        <is>
+          <t>Proceso de acreditación y aprobación largo (12-24 meses típicamente); requisitos técnicos exigentes en medición de impacto climático; necesidad de articular con Entidad Nacional Designada o acreditadas; puede requerir cofinanciación significativa; alta competencia por recursos</t>
+        </is>
+      </c>
+      <c r="AA145" t="inlineStr">
+        <is>
+          <t>Desarrollar una propuesta de programa de economía circular con narrativa climática clara (cuantificación de reducción de emisiones GEI en ciclo de vida de envases, reducción de metano por gestión de residuos orgánicos, etc.); articular con Ministerio de Ambiente para alineación con NDC actualizada de Colombia; explorar alianza con entidad acreditada (FINDETER, PNUD) para presentación</t>
+        </is>
+      </c>
+      <c r="AB145" t="inlineStr">
+        <is>
+          <t>Contactar a la Dirección de Cambio Climático del Ministerio de Ambiente para explorar alineación del programa Visión Circular con prioridades GCF de Colombia; revisar cartera actual de proyectos GCF en Colombia para identificar sinergias; solicitar apoyo del Readiness Programme para formulación de concept note</t>
+        </is>
+      </c>
+      <c r="AC145" t="inlineStr">
+        <is>
+          <t>Dirección de proyectos con experiencia en financiamiento climático y formulación ante fondos multilaterales; articulación institucional con gobierno nacional</t>
+        </is>
+      </c>
+      <c r="AD145" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE145" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF145" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG145" t="inlineStr">
+        <is>
+          <t>El GCF es un mecanismo permanente, no una convocatoria con fecha límite específica. Colombia tiene acceso confirmado y trayectoria de proyectos aprobados. La pertinencia para Visión Circular depende de enmarcar la economía circular explícitamente como estrategia climática con métricas de reducción de GEI. El Readiness Programme es un recurso valioso para fortalecer capacidades de formulación. Se infiere elegibilidad clara para Colombia por la página específica del país y el portafolio existente.</t>
+        </is>
+      </c>
+      <c r="AH145" t="inlineStr">
+        <is>
+          <t>1f6b4d4809d9b285</t>
+        </is>
+      </c>
+      <c r="AI145" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>VC-0145</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme (SGP) - Colombia</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) / UNDP Colombia</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Internacional / Estados Unidos</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Medio ambiente y sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Gestión de recursos, proyectos comunitarios ambientales, economía circular</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Fortalecimiento institucional; Innovación</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Hasta USD 15,000 para organizaciones comunitarias; hasta USD 35,000 para organizaciones con experiencia previa</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/newsroom/news/gef-small-grants-programme-launched-colombia</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>El Programa de Pequeñas Donaciones del GEF (SGP) fue lanzado en Colombia para financiar proyectos de base comunitaria enfocados en medio ambiente y sostenibilidad. Ofrece grants hasta USD 15,000 para organizaciones comunitarias y hasta USD 35,000 para organizaciones con experiencia, implementado en alianza con UNDP Colombia.</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>Aplicable para iniciativas de economía circular territorial, inclusión de recicladores de base, y proyectos piloto comunitarios de gestión de residuos y reciclaje alineados con la estrategia REP y cierre de ciclo de envases.</t>
+        </is>
+      </c>
+      <c r="V146" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de asociaciones de recicladores; pilotos de economía circular comunitaria; gestión integral de residuos plásticos en territorios; innovación en reciclaje inclusivo; ecodiseño participativo con comunidades</t>
+        </is>
+      </c>
+      <c r="W146" t="inlineStr">
+        <is>
+          <t>Ser organización comunitaria o con experiencia en gestión de recursos ambientales; proyectos deben tener componente ambiental y comunitario</t>
+        </is>
+      </c>
+      <c r="X146" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y146" t="inlineStr">
+        <is>
+          <t>Asociaciones de recicladores de oficio, organizaciones comunitarias, gobiernos locales, UNDP Colombia, universidades con presencia territorial</t>
+        </is>
+      </c>
+      <c r="Z146" t="inlineStr">
+        <is>
+          <t>Montos relativamente pequeños pueden limitar alcance; procedimientos de aplicación no detallados en fuentes; no se especifica si hay convocatoria abierta actualmente</t>
+        </is>
+      </c>
+      <c r="AA146" t="inlineStr">
+        <is>
+          <t>Contactar directamente a UNDP Colombia y Coordinación GEF (Pilar Barrera Rey) para confirmar estado de convocatoria, proceso de aplicación y elegibilidad específica para proyectos de economía circular e inclusión de recicladores</t>
+        </is>
+      </c>
+      <c r="AB146" t="inlineStr">
+        <is>
+          <t>Enviar correo formal a UNDP Colombia solicitando información sobre próximas ventanas de aplicación del SGP y términos de referencia para proyectos de economía circular</t>
+        </is>
+      </c>
+      <c r="AC146" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD146" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE146" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF146" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG146" t="inlineStr">
+        <is>
+          <t>Programa confirmado lanzado en Colombia, pero no hay información específica sobre convocatoria vigente o fechas. Los montos son limitados pero aplicables para proyectos piloto comunitarios. Se infiere pertinencia para economía circular territorial e inclusión, aunque las fuentes no detallan líneas temáticas específicas del programa en Colombia.</t>
+        </is>
+      </c>
+      <c r="AH146" t="inlineStr">
+        <is>
+          <t>193a0313342da878</t>
+        </is>
+      </c>
+      <c r="AI146" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>VC-0146</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>GEF SGP CSO Challenge Program</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) / International Union for Conservation of Nature (IUCN)</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Internacional / Estados Unidos</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>América Latina elegible (programa global para OSC locales)</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Medio ambiente, innovación ambiental</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Soluciones ambientales innovadoras, escalamiento de iniciativas comunitarias</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Escalamiento; Innovación; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Hasta USD 300,000 por proyecto</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>Lanzado oficialmente en junio 2026</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>Programa de USD 10 millones liderado por IUCN para apoyar a organizaciones de la sociedad civil (OSC) locales en el escalamiento de soluciones ambientales innovadoras mediante grants competitivos de hasta USD 300,000. Lanzado en la Octava Asamblea del GEF en junio 2026, busca ofrecer recursos financieros y técnicos para amplificar impacto ambiental.</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>Oportunidad de alto valor para escalar modelos de economía circular, sistemas innovadores de reciclaje de plásticos flexibles, esquemas REP territoriales y modelos de negocio circulares con componente de inclusión social demostrado.</t>
+        </is>
+      </c>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>Escalamiento de modelos circulares empresariales probados; sistemas innovadores de reciclaje de envases multicapa; plataformas territoriales de economía circular REP; modelos de negocio circular con inclusión de recicladores; ecodiseño aplicado a escala industrial</t>
+        </is>
+      </c>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>Ser OSC local con soluciones ambientales innovadoras previas demostrables; capacidad de escalamiento; enfoque competitivo</t>
+        </is>
+      </c>
+      <c r="X147" t="inlineStr">
+        <is>
+          <t>No especificado; detalles pendientes de publicación oficial</t>
+        </is>
+      </c>
+      <c r="Y147" t="inlineStr">
+        <is>
+          <t>ANDI como articulador gremial, empresas productoras de envases, universidades con investigación en economía circular, centros tecnológicos, IUCN, redes regionales de OSC ambientales</t>
+        </is>
+      </c>
+      <c r="Z147" t="inlineStr">
+        <is>
+          <t>Fecha de lanzamiento indicada como junio 2026 (probablemente error tipográfico, podría ser 2025); detalles específicos de aplicación aún no disponibles públicamente; competencia global probable</t>
+        </is>
+      </c>
+      <c r="AA147" t="inlineStr">
+        <is>
+          <t>Verificar inmediatamente la fecha real de lanzamiento y monitorear publicación de términos de referencia en sitio oficial GEF/IUCN. Preparar portafolio de casos exitosos de Visión Circular para postulación competitiva.</t>
+        </is>
+      </c>
+      <c r="AB147" t="inlineStr">
+        <is>
+          <t>Contactar a IUCN oficina regional América Latina y revisar sitio GEF semanalmente para detalles de convocatoria. Documentar resultados cuantitativos de pilotos actuales de Visión Circular como evidencia de innovación escalable.</t>
+        </is>
+      </c>
+      <c r="AC147" t="inlineStr">
+        <is>
+          <t>Dirección de programa / Desarrollo de negocios / Alianzas internacionales</t>
+        </is>
+      </c>
+      <c r="AD147" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE147" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF147" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG147" t="inlineStr">
+        <is>
+          <t>Monto significativamente mayor y pertinencia muy alta para economía circular. Sin embargo, hay inconsistencia en fecha (junio 2026 probablemente sea 2025 o ya pasó). Detalles de aplicación explícitamente pendientes. Requiere verificación urgente de calendario real y términos. La competitividad será alta pero el monto justifica la inversión en preparación de propuesta robusta.</t>
+        </is>
+      </c>
+      <c r="AH147" t="inlineStr">
+        <is>
+          <t>3bb2bae3a6223f31</t>
+        </is>
+      </c>
+      <c r="AI147" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>VC-0147</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF) - Readiness and Preparatory Support Programme</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Green Climate Fund</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Internacional / Corea del Sur</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Colombia y países en desarrollo</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Acción climática, adaptación y mitigación</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Fortalecimiento institucional, preparación de proyectos climáticos, involucramiento de actores subnacionales y sociedad civil</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>No especificado en la fuente</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>Programa continuo</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/document/nda-strengthening-and-country-programming-support-colombia-through-apc-colombia</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>https://www.caf.com/media/4670299/perfil-del-proyecto-gcf-readiness.pdf</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>Programa de preparación y fortalecimiento del GCF para Colombia a través de la Agencia Presidencial de Cooperación (APC-Colombia), enfocado en desarrollar capacidades institucionales para acción climática, programación país y participación de actores subnacionales, sociedad civil, consejos comunales, comités ambientales y ONGs en iniciativas climáticas.</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>Pertinente para fortalecer capacidades institucionales de ANDI y Visión Circular en formulación de proyectos climáticos relacionados con economía circular, gestión de residuos con enfoque de mitigación de emisiones GEI, y articulación multinivel (nacional-territorial) para REP y circularidad.</t>
+        </is>
+      </c>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>Desarrollo de capacidades para formular proyectos GCF en economía circular; articulación multinivel para REP climática; preparación de propuestas de mitigación vía reciclaje y gestión circular de residuos; fortalecimiento institucional para acceso a financiamiento climático</t>
+        </is>
+      </c>
+      <c r="W148" t="inlineStr">
+        <is>
+          <t>Coordinación a través de la Autoridad Nacional Designada (NDA) de Colombia - APC-Colombia; proyectos deben tener componente climático claro (mitigación o adaptación)</t>
+        </is>
+      </c>
+      <c r="X148" t="inlineStr">
+        <is>
+          <t>No especificado; depende de la modalidad de Readiness solicitada</t>
+        </is>
+      </c>
+      <c r="Y148" t="inlineStr">
+        <is>
+          <t>APC-Colombia (NDA), Ministerio de Ambiente y Desarrollo Sostenible, CAF, gobiernos locales, asociaciones de recicladores, gremios empresariales, ONGs ambientales</t>
+        </is>
+      </c>
+      <c r="Z148" t="inlineStr">
+        <is>
+          <t>Enfoque principal en preparación y capacidades, no en financiamiento directo de proyectos; requiere articulación con NDA nacional; procesos pueden ser extensos</t>
+        </is>
+      </c>
+      <c r="AA148" t="inlineStr">
+        <is>
+          <t>Contactar a APC-Colombia para explorar ventanas de Readiness específicas para economía circular y residuos con enfoque climático. Evaluar posibilidad de apoyo para preparar propuestas de financiamiento GCF full-size en economía circular.</t>
+        </is>
+      </c>
+      <c r="AB148" t="inlineStr">
+        <is>
+          <t>Reunión exploratoria con APC-Colombia para identificar líneas de Readiness aplicables a economía circular de envases y empaques con co-beneficios climáticos. Revisar portafolio GCF Colombia para identificar áreas de oportunidad.</t>
+        </is>
+      </c>
+      <c r="AC148" t="inlineStr">
+        <is>
+          <t>Alianzas estratégicas / Gestión de conocimiento / Formulación de proyectos</t>
+        </is>
+      </c>
+      <c r="AD148" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE148" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF148" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG148" t="inlineStr">
+        <is>
+          <t>Es un programa de preparación y asistencia técnica, no de financiamiento directo de proyectos. Sin embargo, es estratégico para preparar el terreno hacia propuestas de financiamiento GCF de mayor escala. La fuente confirma enfoque en Colombia y participación de múltiples actores incluyendo sociedad civil y ONGs. La relación con economía circular es indirecta pero aprovechable vía el ángulo climático (mitigación GEI por reciclaje, economía circular).</t>
+        </is>
+      </c>
+      <c r="AH148" t="inlineStr">
+        <is>
+          <t>408c9d89b0d785cc</t>
+        </is>
+      </c>
+      <c r="AI148" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>VC-0148</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme (SGP)</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) / United Nations Development Programme (UNDP)</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>182 países incluyendo Colombia y América Latina</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Residuos, gestión comunitaria, biodiversidad, cambio climático, degradación de tierras</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Fortalecimiento institucional; Inclusión social; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Pequeñas donaciones (típicamente hasta USD 50,000 por proyecto según modelo SGP estándar)</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>Generalmente requiere contrapartida comunitaria en especie o monetaria</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/georgia/projects/gef-small-grants-programme</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>https://co.chm-cbd.net/en/gef-projects</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>El GEF Small Grants Programme (SGP) es un mecanismo global que otorga pequeñas donaciones a organizaciones comunitarias, cooperativas y sociedad civil para proyectos ambientales locales. Opera en 182 países incluyendo Colombia, enfocándose en biodiversidad, cambio climático, aguas internacionales, degradación de tierras y químicos. Fomenta acciones comunitarias con impacto ambiental global.</t>
+        </is>
+      </c>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>SGP puede financiar proyectos comunitarios de economía circular, reciclaje inclusivo, gestión de residuos de envases y empaques, y fortalecimiento de asociaciones de recicladores de base, alineados con la inclusión social y territorial que promueve Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V149" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje comunitario de plásticos flexibles; fortalecimiento de cooperativas de recicladores; gestión territorial de residuos de envases; proyectos de ecodiseño participativo con comunidades; educación ambiental y economía circular en territorios</t>
+        </is>
+      </c>
+      <c r="W149" t="inlineStr">
+        <is>
+          <t>Organizaciones comunitarias, cooperativas, ONGs locales, grupos de base; enfoque en beneficios ambientales globales con impacto local; participación comunitaria activa</t>
+        </is>
+      </c>
+      <c r="X149" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto, presupuesto, plan de participación comunitaria, cartas de apoyo, perfil organizacional (varían según país y ventana)</t>
+        </is>
+      </c>
+      <c r="Y149" t="inlineStr">
+        <is>
+          <t>Asociaciones de recicladores de oficio, cooperativas de reciclaje, ONGs ambientales locales, gobiernos locales, universidades con programas de extensión comunitaria, ANDI como articulador sectorial</t>
+        </is>
+      </c>
+      <c r="Z149" t="inlineStr">
+        <is>
+          <t>Montos pequeños pueden limitar alcance de proyectos empresariales; enfoque principalmente comunitario puede requerir adaptación del modelo de Visión Circular; tiempos de aprobación pueden ser largos; disponibilidad de ventanas abiertas en Colombia no confirmada</t>
+        </is>
+      </c>
+      <c r="AA149" t="inlineStr">
+        <is>
+          <t>Contactar oficina UNDP Colombia para verificar estado de ventanas SGP 2025, elegibilidad de ANDI/Visión Circular (directamente o vía ONGs aliadas), y fechas de convocatorias. Identificar asociaciones de recicladores elegibles para coaplicación.</t>
+        </is>
+      </c>
+      <c r="AB149" t="inlineStr">
+        <is>
+          <t>Verificar con UNDP Colombia (www.undp.org/colombia) si hay convocatoria SGP abierta o próxima en 2025 y requisitos específicos para Colombia</t>
+        </is>
+      </c>
+      <c r="AC149" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas y proyectos territoriales / Oficial de cooperación internacional</t>
+        </is>
+      </c>
+      <c r="AD149" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE149" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF149" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG149" t="inlineStr">
+        <is>
+          <t>Monto inferido según estándar típico SGP. No hay convocatoria específica con fechas en las fuentes proporcionadas. Referencia a Sudáfrica 2026 sugiere que el programa opera con ventanas por país. Requiere verificación de ventana Colombia 2025.</t>
+        </is>
+      </c>
+      <c r="AH149" t="inlineStr">
+        <is>
+          <t>d91a2eac0ee030fe</t>
+        </is>
+      </c>
+      <c r="AI149" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>VC-0149</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Programa EUROCLIMA+ (componente Economía Circular y Acción Climática Local)</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Unión Europea / Gobierno Federal de Alemania</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Unión Europea / Alemania</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Cambio climático</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Acción climática local, economía circular, transición sostenible, resiliencia, biodiversidad</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Cofinanciación; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>Sí (modalidades varían según componente)</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>https://ccesantiago.aecid.es/-/cce-santiago-acoge-presentaci%C3%B3n-de-proyecto-para-fortalecer-la-acci%C3%B3n-clim%C3%A1tica-local-y-la-econom%C3%ADa-circular</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>EUROCLIMA+ es una iniciativa de cooperación regional UE-América Latina-Caribe cofinanciada por la UE y Alemania que fortalece la acción climática y busca una transición sostenible, resiliente e inclusiva. Incluye componentes de economía circular y acción climática local. Opera mediante asistencia técnica, proyectos piloto y fortalecimiento institucional en la región.</t>
+        </is>
+      </c>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>EUROCLIMA+ puede apoyar proyectos de economía circular territorial, modelos de negocio circulares con enfoque climático, fortalecimiento de sistemas de gestión de residuos, y articulación con gobiernos locales, todos ejes de trabajo de Visión Circular ANDI.</t>
+        </is>
+      </c>
+      <c r="V150" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de economía circular territorial; pilotos de gestión climática de residuos de envases; sistemas locales REP; modelos de negocio circulares con co-beneficios climáticos; articulación público-privada para circularidad; inclusión de recicladores en cadenas de valor climáticamente inteligentes</t>
+        </is>
+      </c>
+      <c r="W150" t="inlineStr">
+        <is>
+          <t>Entidades públicas, privadas, academia, sociedad civil de América Latina y Caribe; articulación regional o nacional; enfoque en cambio climático y sostenibilidad; alineación con NDC y agendas climáticas nacionales</t>
+        </is>
+      </c>
+      <c r="X150" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y150" t="inlineStr">
+        <is>
+          <t>Gobiernos locales y regionales, ministerios de ambiente y cambio climático, gremios sectoriales LAC, universidades, redes de recicladores, CEPAL, bancos de desarrollo regionales</t>
+        </is>
+      </c>
+      <c r="Z150" t="inlineStr">
+        <is>
+          <t>Programa en fase de implementación de proyectos ya aprobados; no está claro si hay nuevas convocatorias abiertas; tiempos de cooperación europea pueden ser largos; requisitos de articulación regional pueden ser complejos</t>
+        </is>
+      </c>
+      <c r="AA150" t="inlineStr">
+        <is>
+          <t>Contactar oficina EUROCLIMA+ para verificar si hay ventanas abiertas 2025 o mecanismos de incorporación a proyectos en curso. Explorar articulación con componentes de economía circular y residuos.</t>
+        </is>
+      </c>
+      <c r="AB150" t="inlineStr">
+        <is>
+          <t>Contactar punto focal EUROCLIMA+ en Colombia o regional (www.euroclima.org) para confirmar estado de convocatorias 2025 y mecanismos de participación para sector privado/gremial</t>
+        </is>
+      </c>
+      <c r="AC150" t="inlineStr">
+        <is>
+          <t>Coordinación de cooperación internacional / Relaciones con cooperación europea</t>
+        </is>
+      </c>
+      <c r="AD150" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE150" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF150" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG150" t="inlineStr">
+        <is>
+          <t>Fuente es nota de prensa sobre presentación de un proyecto ya existente, no una convocatoria abierta. Se infiere que el programa existe y opera en LAC, pero no hay evidencia de convocatoria vigente. Requiere verificación urgente de ventanas abiertas.</t>
+        </is>
+      </c>
+      <c r="AH150" t="inlineStr">
+        <is>
+          <t>46103537b12fdae4</t>
+        </is>
+      </c>
+      <c r="AI150" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>VC-0150</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Programa EUROCLIMA - Nueva Fase 2026-2027</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Unión Europea (implementado por Expertise France y otras agencias)</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (incluye Colombia)</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Cambio climático y transición verde</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Economía circular, biodiversidad, políticas públicas climáticas</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>Aprox. 2026-Q1 (en diseño)</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>https://expertise-france.gestmax.fr/_expertise_france/public_files/tdr-experto-a-guatemala-economia-circular.pdf</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>https://www.fiap.gob.es/noticias/euroclima-impulsa-la-coordinacion-regional-para-avanzar-en-la-transicion-verde-en-america-latina-y-el-caribe</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>EUROCLIMA es el programa insignia de la UE para cooperación climática en América Latina y el Caribe. Actualmente está en proceso de diseño de una nueva fase (2026-2027) con énfasis en transición verde, economía circular, biodiversidad y cambio climático. El programa emplea metodología de Diálogo País y fortalecimiento institucional interministerial. Se está definiendo la agenda de inversión UE-ALC y prioridades estratégicas para el próximo período.</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>EUROCLIMA tiene un componente explícito de economía circular y está alineado con la transición verde de la región. Colombia históricamente ha participado en fases anteriores; el programa facilita diálogo político, asistencia técnica y coordinación regional que puede apoyar el escalamiento de Visión Circular a nivel de políticas públicas, articulación con gobiernos y réplica territorial.</t>
+        </is>
+      </c>
+      <c r="V151" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de marcos REP a nivel nacional y subnacional; diálogo multisectorial para cierre de ciclo de envases; economía circular territorial; articulación con autoridades ambientales; transferencia de conocimiento y buenas prácticas en reciclaje inclusivo; alineación de estrategias empresariales de economía circular con agendas públicas climáticas.</t>
+        </is>
+      </c>
+      <c r="W151" t="inlineStr">
+        <is>
+          <t>Participación o coordinación con entidades gubernamentales (ministerios de ambiente, cambio climático, economía); alineación con NDC y políticas climáticas nacionales; capacidad de diálogo interinstitucional. No especificado en detalle aún dado que la convocatoria está en diseño.</t>
+        </is>
+      </c>
+      <c r="X151" t="inlineStr">
+        <is>
+          <t>No especificado (fase de diseño)</t>
+        </is>
+      </c>
+      <c r="Y151" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible, DNP, autoridades regionales CAR, universidades (Andes, Javeriana, Nacional), gremios ANDI, ACOPLÁSTICOS, asociaciones de recicladores (ARB, ANR), centros tecnológicos como SENA, CIDET.</t>
+        </is>
+      </c>
+      <c r="Z151" t="inlineStr">
+        <is>
+          <t>Convocatoria aún no publicada; cronograma y términos de referencia en construcción. Posible enfoque prioritario en gobiernos centrales más que en gremios; cofinanciación o contrapartida nacional podría ser necesaria. Competencia regional alta.</t>
+        </is>
+      </c>
+      <c r="AA151" t="inlineStr">
+        <is>
+          <t>Monitorear activamente el lanzamiento oficial de la nueva fase EUROCLIMA 2026-2027. Contactar delegación UE en Colombia y Expertise France para conocer prioridades temáticas y ventanas de participación. Preparar propuestas conceptuales de economía circular alineadas con NDC colombiana y política REP.</t>
+        </is>
+      </c>
+      <c r="AB151" t="inlineStr">
+        <is>
+          <t>Establecer contacto con Delegación de la UE en Colombia y equipo EUROCLIMA regional para obtener información preliminar sobre áreas temáticas prioritarias y cronograma estimado de apertura. Participar en eventos de socialización del programa.</t>
+        </is>
+      </c>
+      <c r="AC151" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Dirección de Alianzas Estratégicas / Relaciones Internacionales ANDI</t>
+        </is>
+      </c>
+      <c r="AD151" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE151" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF151" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG151" t="inlineStr">
+        <is>
+          <t>La información proviene de documentos de trabajo y notas de prensa sobre la fase de diseño del programa. No hay convocatoria abierta aún, pero está en construcción activa para 2026-2027. Se infiere que economía circular será componente prioritario dado el contexto de transición verde. La elegibilidad de Colombia está confirmada históricamente, pero modalidades específicas (si aplica ANDI directamente o vía gobierno) están por definirse. | Fuente fuera del listado oficial conocido (expertise-france.gestmax.fr): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH151" t="inlineStr">
+        <is>
+          <t>217859d18eb0c49a</t>
+        </is>
+      </c>
+      <c r="AI151" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-07-24
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI180"/>
+  <dimension ref="A1:AI199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -18643,7 +18643,7 @@
       </c>
       <c r="AI103" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -26326,7 +26326,7 @@
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>Lanzado oficialmente junio 2026</t>
+          <t>Lanzado junio 2026</t>
         </is>
       </c>
       <c r="O147" t="inlineStr">
@@ -26431,7 +26431,7 @@
       </c>
       <c r="AI147" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -27478,7 +27478,7 @@
       </c>
       <c r="AF153" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AG153" t="inlineStr">
@@ -27493,7 +27493,7 @@
       </c>
       <c r="AI153" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -27742,12 +27742,12 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="P155" t="inlineStr">
@@ -27822,19 +27822,19 @@
       </c>
       <c r="AD155" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE155" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF155" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AE155" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AF155" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="AG155" t="inlineStr">
         <is>
           <t>Fuente oficial confirmada (Bogota.gov.co). Fecha de apertura inferida como 2026 basada en título y contexto. La fecha de cierre específica no aparece en los fragmentos, requiere consulta directa. Los sectores priorizados mencionados en Instagram (energías limpias, transporte) sugieren que economía circular/reciclaje podría ser elegible si se enmarca como solución climática, pero requiere confirmación. La pertinencia es alta si se logra articular proyectos de Visión Circular con métricas de mitigación climática. | Fuente fuera del listado oficial conocido (bogota.gov.co): verificar oficialidad</t>
@@ -27847,7 +27847,7 @@
       </c>
       <c r="AI155" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -32273,6 +32273,3369 @@
       <c r="AI180" t="inlineStr">
         <is>
           <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>VC-0180</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Convocatoria Visión Circular 2025-2026</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>ANDI - Asociación Nacional de Empresarios de Colombia / Programa Visión Circular</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Gremio</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Recuperación y transformación de envases y empaques posconsumo, movilidad sostenible para recicladores</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Cofinanciación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Proyectos individuales entre COP 217.567.700 y COP 243.886.625 (montos de referencia observados)</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>https://www.andi.com.co/Uploads/Conv.%20Visi%C3%B3n%20Circular%202025-2026.pdf</t>
+        </is>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>Convocatoria interna del Programa Visión Circular de la ANDI para cofinanciar proyectos de economía circular empresarial enfocados en recuperación y transformación de envases posconsumo (como botellas de vidrio) y soluciones de movilidad sostenible para empresas recicladoras. Se identificaron proyectos aprobados con montos entre COP 217M y COP 243M para implementación en 12 meses.</t>
+        </is>
+      </c>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>Esta es la convocatoria propia del programa Visión Circular ANDI, directamente alineada con todos sus objetivos estratégicos: economía circular, cierre de ciclo de envases, inclusión de recicladores y pilotos empresariales demostrativos.</t>
+        </is>
+      </c>
+      <c r="V181" t="inlineStr">
+        <is>
+          <t>Recuperación de envases de vidrio posconsumo; Movilidad sostenible para recicladores; Modelos de negocio circulares empresariales; Cierre de ciclo de empaques; Soluciones integrales para cadena de reciclaje</t>
+        </is>
+      </c>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X181" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y181" t="inlineStr">
+        <is>
+          <t>Empresas asociadas ANDI, empresas BIC, cooperativas de recicladores, gremios sectoriales</t>
+        </is>
+      </c>
+      <c r="Z181" t="inlineStr">
+        <is>
+          <t>El documento muestra proyectos ya aprobados (PI25, PI26), posible que la convocatoria actual esté en etapa de ejecución o cerrada; requiere verificación de vigencia de ventanas 2025-2026</t>
+        </is>
+      </c>
+      <c r="AA181" t="inlineStr">
+        <is>
+          <t>Verificar internamente con la coordinación de Visión Circular ANDI si la convocatoria 2025-2026 tiene ventanas adicionales abiertas o si se abrirá nueva fase en 2026</t>
+        </is>
+      </c>
+      <c r="AB181" t="inlineStr">
+        <is>
+          <t>Contactar a coordinación Visión Circular ANDI para confirmar cronograma de ventanas de aplicación y lineamientos actualizados</t>
+        </is>
+      </c>
+      <c r="AC181" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos Visión Circular ANDI / PROJECTABILITY</t>
+        </is>
+      </c>
+      <c r="AD181" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE181" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF181" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG181" t="inlineStr">
+        <is>
+          <t>Documento muestra proyectos ya seleccionados (PI25 Celema, PI26 Equirent). No se observa fecha explícita de cierre de convocatoria ni criterios completos. Se infiere que es convocatoria interna del programa que PROJECTABILITY/Soluciones PAL apoya, por lo que tiene máxima pertinencia institucional. | Fuente fuera del listado oficial conocido (andi.com.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH181" t="inlineStr">
+        <is>
+          <t>a9e930d03d142de6</t>
+        </is>
+      </c>
+      <c r="AI181" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>VC-0181</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Programa de Impulso a la Bioeconomía y la Economía Circular en Iniciativas de Articulación Productiva - CEPAL/GIZ</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>CEPAL - Comisión Económica para América Latina y el Caribe / GIZ - Deutsche Gesellschaft für Internationale Zusammenarbeit / BMZ - Ministerio Federal de Cooperación Económica y Desarrollo de Alemania</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Regional América Latina y el Caribe / Alemania</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Bioeconomía, articulación productiva, cadenas de valor circulares</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>Proyecto ejecutado 2024-2026</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>https://www.cepal.org/es/eventos/lanzamiento-convocatoria-programa-impulso-la-bioeconomia-la-economia-circular-iniciativas</t>
+        </is>
+      </c>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>Convocatoria de CEPAL y GIZ (financiada por BMZ Alemania) dentro del proyecto 'Promoviendo la Economía Circular en América Latina y el Caribe' (2024-2026) para robustecer iniciativas de articulación productiva con enfoque en bioeconomía y economía circular. Busca fortalecer capacidades de iniciativas existentes en la región.</t>
+        </is>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>Oportunidad para posicionar a Visión Circular como iniciativa modelo de articulación productiva en economía circular en Colombia, acceder a asistencia técnica de CEPAL/GIZ y networking regional con iniciativas similares en ALC.</t>
+        </is>
+      </c>
+      <c r="V182" t="inlineStr">
+        <is>
+          <t>Fortalecimiento institucional de Visión Circular; Articulación productiva empresa-recicladores; Modelos de economía circular sectorial (envases y empaques); Intercambio de experiencias regional; Escalamiento de pilotos</t>
+        </is>
+      </c>
+      <c r="W182" t="inlineStr">
+        <is>
+          <t>Iniciativas de articulación productiva existentes con componente de economía circular o bioeconomía</t>
+        </is>
+      </c>
+      <c r="X182" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y182" t="inlineStr">
+        <is>
+          <t>CEPAL, GIZ, Ministerios de Ambiente y Producción de Colombia, otras iniciativas de economía circular en ALC, universidades y centros de investigación regional</t>
+        </is>
+      </c>
+      <c r="Z182" t="inlineStr">
+        <is>
+          <t>Proyecto ejecutado entre 2024-2026, posible que ventana de aplicación esté cerrada o en fase final; el evento es de 'lanzamiento de convocatoria' pero sin fecha específica</t>
+        </is>
+      </c>
+      <c r="AA182" t="inlineStr">
+        <is>
+          <t>Contactar urgentemente a CEPAL (División de Desarrollo Productivo) y GIZ Colombia para verificar si convocatoria aún está abierta y plazos de aplicación; preparar caracterización de Visión Circular como iniciativa de articulación productiva</t>
+        </is>
+      </c>
+      <c r="AB182" t="inlineStr">
+        <is>
+          <t>Enviar correo a puntos focales de CEPAL y GIZ solicitando términos de referencia, elegibilidad y cronograma vigente de la convocatoria</t>
+        </is>
+      </c>
+      <c r="AC182" t="inlineStr">
+        <is>
+          <t>Dirección Visión Circular / Área de cooperación internacional ANDI</t>
+        </is>
+      </c>
+      <c r="AD182" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE182" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF182" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG182" t="inlineStr">
+        <is>
+          <t>La URL menciona 'lanzamiento de convocatoria' pero no especifica fecha del evento ni plazos de aplicación. El proyecto marco es 2024-2026, por lo que podría estar en fase final. Alta pertinencia pero urgente verificar vigencia. | Fuente fuera del listado oficial conocido (cepal.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH182" t="inlineStr">
+        <is>
+          <t>e3ca33c72b8d2aad</t>
+        </is>
+      </c>
+      <c r="AI182" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>VC-0182</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Convocatoria regional para soluciones innovadoras en plásticos - Pacto por los Plásticos Colombia, Chile y México</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Pacto Global Red Colombia en alianza con Pacto por los Plásticos de México y Chile</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Colombia (iniciativa regional)</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Colombia, Chile, México</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Economía circular - Plásticos</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Plásticos flexibles, sachets, empaques multilaminados, etiquetas, bolsas</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Hasta USD 10.000 por iniciativa</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>https://www.pactoglobal-colombia.org/news/convocatoria-regional-otorgara-hasta-usd-10-000-a-soluciones-innovadoras-en-plasticos-en-colombia-chile-y-mexico.html</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>Convocatoria regional que otorga hasta USD 10.000 por proyecto para apoyar soluciones innovadoras que prevengan la contaminación por plásticos, con especial foco en plásticos flexibles (sachets, multilaminados, etiquetas, bolsas). Desarrollada en el marco del Pacto por los Plásticos de Colombia, Chile y México. Busca iniciativas de crecimiento y desarrollo que aborden la gestión inadecuada de residuos plásticos.</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular ANDI porque aborda específicamente plásticos flexibles (una prioridad del programa), envases/empaques, innovación en gestión de residuos y cierre de ciclo. La convocatoria se enmarca en el Pacto por los Plásticos Colombia, iniciativa con la cual ANDI tiene articulación directa.</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclabilidad de plásticos flexibles; modelos de negocio circulares para sachets y multilaminados; innovaciones en ecodiseño de empaques flexibles; esquemas de recolección inclusiva de plásticos flexibles con recicladores; tecnologías de clasificación y aprovechamiento de flexibles; sistemas de trazabilidad para cumplimiento REP en plásticos flexibles.</t>
+        </is>
+      </c>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>Iniciativas enfocadas en prevención de contaminación por plásticos, especialmente flexibles; propuestas innovadoras con potencial de crecimiento; orientación a gestión adecuada de residuos plásticos</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>Empresas miembro del Pacto por los Plásticos Colombia; recicladores de base y organizaciones de recicladores; universidades con líneas en materiales y empaques; centros tecnológicos (ICIPC, SENA); empresas productoras de empaques flexibles; municipios; Minambiente</t>
+        </is>
+      </c>
+      <c r="Z183" t="inlineStr">
+        <is>
+          <t>Fecha de cierre no especificada en la fuente (publicada en noviembre 2025, podría estar próxima a cerrar o ya cerrada); monto relativamente bajo para pilotos de gran escala; requiere verificación urgente de vigencia y términos de referencia completos</t>
+        </is>
+      </c>
+      <c r="AA183" t="inlineStr">
+        <is>
+          <t>Verificar inmediatamente vigencia y fechas con Pacto Global Red Colombia. Si está abierta, preparar propuesta enfocada en plásticos flexibles con caso empresarial concreto, idealmente con empresa piloto del portafolio de Visión Circular y componente de inclusión de recicladores.</t>
+        </is>
+      </c>
+      <c r="AB183" t="inlineStr">
+        <is>
+          <t>Contactar a Pacto Global Red Colombia (contacto directo de coordinación del Pacto por los Plásticos) para confirmar vigencia, obtener TdR completos y fechas exactas de cierre. Simultáneamente, mapear empresas de Visión Circular interesadas en piloto de flexibles.</t>
+        </is>
+      </c>
+      <c r="AC183" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de Visión Circular + Área de innovación/pilotos empresariales</t>
+        </is>
+      </c>
+      <c r="AD183" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE183" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF183" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG183" t="inlineStr">
+        <is>
+          <t>Fuente oficial pero fecha de publicación indica noviembre 2025 (posible error o dato prospectivo). La convocatoria es altamente relevante pero requiere verificación urgente de vigencia real. El Pacto por los Plásticos Colombia es un aliado natural de ANDI/Visión Circular. | Fuente fuera del listado oficial conocido (pactoglobal-colombia.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH183" t="inlineStr">
+        <is>
+          <t>d5f354e7d26bc976</t>
+        </is>
+      </c>
+      <c r="AI183" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>VC-0183</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Convocatoria BID - Fondos no reembolsables para estrategias industriales sostenibles (hasta USD 80.000)</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Banco Interamericano de Desarrollo (BID)</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Regional - América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (inferido por naturaleza del BID)</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Industria sostenible y empleos verdes</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Estrategias industriales, empleos verdes, sostenibilidad financiera</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cofinanciación</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>USD 60.000 por propuesta (hasta USD 80.000 si incluye empleos verdes)</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>https://mundobiotec.com/convocatorias</t>
+        </is>
+      </c>
+      <c r="S184" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>Programa del BID que otorga fondos no reembolsables de hasta USD 60.000 por propuesta para implementar estrategias industriales sostenibles, con incremento hasta USD 80.000 para propuestas que integren empleos verdes. Los fondos son administrados por el BID para ejecutar actividades acordadas. Orientado a nichos de mercado y desarrollo industrial sostenible.</t>
+        </is>
+      </c>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular porque permite financiar estrategias de transformación industrial hacia circularidad en empresas, con potencial de integrar componente de empleos verdes (recicladores de base, operadores de plantas de reciclaje). Aplica para modelos de negocio circulares, pilotos empresariales de economía circular e inclusión productiva de recicladores.</t>
+        </is>
+      </c>
+      <c r="V184" t="inlineStr">
+        <is>
+          <t>Estrategias de circularidad industrial en sectores de envases/empaques; modelos de negocio circular con creación de empleos verdes en reciclaje; pilotos de simbiosis industrial para aprovechamiento de residuos; implementación de sistemas REP con inclusión de recicladores; escalamiento de tecnologías de reciclaje con generación de empleo; economía circular territorial con enfoque de empleo verde.</t>
+        </is>
+      </c>
+      <c r="W184" t="inlineStr">
+        <is>
+          <t>Propuestas para implementación de estrategias industriales sostenibles; preferencia por iniciativas que generen empleos verdes; viabilidad de ejecución con administración del BID</t>
+        </is>
+      </c>
+      <c r="X184" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y184" t="inlineStr">
+        <is>
+          <t>Empresas industriales de sectores prioritarios (alimentos, bebidas, consumo masivo); organizaciones de recicladores de base; cámaras de comercio; asociaciones industriales regionales; gobiernos locales; SENA para componente de empleos verdes</t>
+        </is>
+      </c>
+      <c r="Z184" t="inlineStr">
+        <is>
+          <t>Fuente secundaria (Mundobiotec.com, no portal oficial del BID); no hay fechas de convocatoria especificadas; falta URL oficial del BID; información incompleta sobre términos de referencia; requiere validación urgente de existencia y vigencia de la convocatoria</t>
+        </is>
+      </c>
+      <c r="AA184" t="inlineStr">
+        <is>
+          <t>Verificar con oficina del BID en Colombia la existencia, vigencia y términos exactos de esta convocatoria. Si existe y está vigente, preparar propuesta enfocada en economía circular industrial con fuerte componente de empleos verdes (inclusión de recicladores) para acceder al monto máximo de USD 80.000.</t>
+        </is>
+      </c>
+      <c r="AB184" t="inlineStr">
+        <is>
+          <t>Contactar representación del BID en Colombia para validar esta convocatoria. Buscar en el portal oficial del BID (iadb.org) convocatorias activas en industria sostenible, empleos verdes o economía circular. Solicitar términos de referencia oficiales.</t>
+        </is>
+      </c>
+      <c r="AC184" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos + Oficial de relaciones con banca multilateral</t>
+        </is>
+      </c>
+      <c r="AD184" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE184" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF184" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG184" t="inlineStr">
+        <is>
+          <t>La información proviene de un portal agregador (Mundobiotec) no del BID directamente, lo que genera incertidumbre sobre vigencia y términos exactos. El monto es atractivo y el enfoque en empleos verdes calza bien con inclusión de recicladores. Sin embargo, la falta de URL oficial del BID y de fechas específicas requiere validación prioritaria. Se asume elegibilidad de Colombia por naturaleza regional del BID. | Fuente fuera del listado oficial conocido (mundobiotec.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH184" t="inlineStr">
+        <is>
+          <t>b54b90464aec85aa</t>
+        </is>
+      </c>
+      <c r="AI184" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>VC-0184</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Programa de Pequeñas Donaciones (SGP) del FMAM - Gestión de Residuos Plásticos con Enfoque de Economía Circular</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Fondo para el Medio Ambiente Mundial (GEF/FMAM) - administrado por PNUD</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe, incluyendo Colombia</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Gestión de residuos plásticos, Innovación en reciclaje</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Piloto demostrativo; Innovación; Inclusión social</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>No especificado en el documento</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>https://www.sgp.undp.org/</t>
+        </is>
+      </c>
+      <c r="S185" t="inlineStr">
+        <is>
+          <t>https://territoriocircular.sofofahub.cl/wp-content/uploads/2024/10/La-economia-circular-en-America-Latina-y-el-Caribe-Oportunidades-para-fomentar-la-resiliencia.pdf</t>
+        </is>
+      </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>El Programa de Pequeñas Donaciones del FMAM ha financiado diversos proyectos en América Latina y el Caribe que prueban prácticas innovadoras para gestionar residuos plásticos empleando un enfoque de economía circular. El programa apoya iniciativas comunitarias y organizaciones de base que implementan soluciones locales con impacto ambiental global.</t>
+        </is>
+      </c>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular pues financia proyectos innovadores en gestión de residuos plásticos con enfoque circular, alineándose con los objetivos de reciclaje, cierre de ciclo de envases y empaques, e inclusión de recicladores de base.</t>
+        </is>
+      </c>
+      <c r="V185" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje inclusivo de plásticos flexibles; Modelos comunitarios de gestión de envases post-consumo; Innovación en valorización de residuos plásticos con inclusión de recicladores; Iniciativas territoriales de economía circular con comunidades de recicladores</t>
+        </is>
+      </c>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>Típicamente el SGP requiere organizaciones comunitarias, ONGs de base, o cooperativas. Se prioriza participación comunitaria, impacto ambiental global, innovación local y sostenibilidad</t>
+        </is>
+      </c>
+      <c r="X185" t="inlineStr">
+        <is>
+          <t>Propuesta técnica, presupuesto, evidencia de capacidad organizacional, cartas de apoyo comunitario (verificar en convocatoria específica del país)</t>
+        </is>
+      </c>
+      <c r="Y185" t="inlineStr">
+        <is>
+          <t>Cooperativas y asociaciones de recicladores, ONGs ambientales locales, gobiernos municipales, universidades para componente técnico, PNUD Colombia como administrador del SGP</t>
+        </is>
+      </c>
+      <c r="Z185" t="inlineStr">
+        <is>
+          <t>Montos típicamente pequeños (hasta USD 50,000); Prioridad a organizaciones de base podría limitar aplicación directa de gremios empresariales; Competencia alta; Requiere verificar si hay ventana abierta en Colombia</t>
+        </is>
+      </c>
+      <c r="AA185" t="inlineStr">
+        <is>
+          <t>Contactar urgentemente a PNUD Colombia - Programa SGP para confirmar ventanas abiertas o próximas convocatorias 2025. Explorar alianza con asociaciones de recicladores para co-aplicar</t>
+        </is>
+      </c>
+      <c r="AB185" t="inlineStr">
+        <is>
+          <t>Verificar con PNUD Colombia (https://www.undp.org/es/colombia) estado de convocatorias SGP 2024-2025 y criterios específicos para Colombia</t>
+        </is>
+      </c>
+      <c r="AC185" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de Visión Circular en alianza con área de inclusión de recicladores</t>
+        </is>
+      </c>
+      <c r="AD185" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF185" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG185" t="inlineStr">
+        <is>
+          <t>El documento menciona que el SGP ha financiado proyectos pero no especifica convocatorias activas. Se infiere que es un programa continuo. La aplicación directa por gremios puede ser limitada, pero alianzas con recicladores son viables y estratégicas para Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AH185" t="inlineStr">
+        <is>
+          <t>7e97320d16f4706c</t>
+        </is>
+      </c>
+      <c r="AI185" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>VC-0185</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia Innovation Challenge</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Agritech Challenge (organización no especificada en detalle)</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Sector agroalimentario, transición circular</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Aceleración; Innovación; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>Challenge de innovación enfocado en acelerar la transición hacia una economía circular en el sector agroalimentario de Colombia, alineado con el Plan Nacional de Desarrollo 2022-2026 y los objetivos de CBD COP 16 Colombia. Ofrece mentoría experta y acceso a recursos para soluciones innovadoras en economía circular.</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>Aunque centrado en sector agroalimentario, la economía circular de envases y empaques es crítica para este sector. Ofrece plataforma para innovación en cierre de ciclo, diseño de empaques sostenibles y modelos de negocio circulares aplicables a envases de alimentos.</t>
+        </is>
+      </c>
+      <c r="V186" t="inlineStr">
+        <is>
+          <t>Ecodiseño de empaques agroalimentarios; modelos de negocio circulares para envases de alimentos; sistemas de retorno y reciclaje de envases agroindustriales; innovación en materiales de empaque compostables o reciclables para alimentos; pilotos de REP en sector agroalimentario</t>
+        </is>
+      </c>
+      <c r="W186" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X186" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y186" t="inlineStr">
+        <is>
+          <t>Empresas agroalimentarias de la ANDI, universidades con programas de ingeniería de alimentos y empaques, centros tecnológicos de envases, cooperativas de recicladores especializadas en residuos agroindustriales</t>
+        </is>
+      </c>
+      <c r="Z186" t="inlineStr">
+        <is>
+          <t>Alcance limitado al sector agroalimentario podría restringir proyectos más amplios de Visión Circular; falta de información sobre montos, fechas y requisitos específicos dificulta evaluación completa de aplicabilidad</t>
+        </is>
+      </c>
+      <c r="AA186" t="inlineStr">
+        <is>
+          <t>Contactar directamente a los organizadores para confirmar vigencia, plazos, montos disponibles y criterios de elegibilidad. Evaluar si proyectos de envases y empaques circulares para alimentos son admisibles.</t>
+        </is>
+      </c>
+      <c r="AB186" t="inlineStr">
+        <is>
+          <t>Visitar la URL oficial, identificar punto de contacto y solicitar información detallada sobre términos de referencia, cronograma y formulario de aplicación. Verificar si hay sesiones informativas programadas.</t>
+        </is>
+      </c>
+      <c r="AC186" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de innovación / Área de alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD186" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE186" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF186" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG186" t="inlineStr">
+        <is>
+          <t>La fuente no proporciona fechas, montos ni requisitos específicos. El enfoque en sector agroalimentario puede ser complementario pero no es el núcleo principal de Visión Circular (envases/empaques en general). Se requiere verificación urgente de vigencia y términos. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH186" t="inlineStr">
+        <is>
+          <t>496c95c3637322cd</t>
+        </is>
+      </c>
+      <c r="AI186" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>VC-0186</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Sector Reform Contract for Sustainable Local Development in Colombia - Circular Economy Action Line (Phase 2)</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Implementación de estrategia nacional de economía circular, inversiones circulares, escalamiento de programas</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Apoyo presupuestario; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>9 millones</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>2022 o posterior (período 2020-22 mencionado en fuente)</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>https://www.switchtogreen.eu/wp-content/uploads/2021/09/Colombia-VF-09-2021a2.pdf</t>
+        </is>
+      </c>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>La Unión Europea proporciona apoyo presupuestario de €9 millones al Ministerio de Ambiente y Desarrollo Sostenible (MADS) y al Ministerio de Comercio, Industria y Turismo para la segunda fase del Contrato de Reforma Sectorial para el Desarrollo Local Sostenible en Colombia (período 2020-22). Una línea de acción específica se enfoca en economía circular, implementando la estrategia nacional CE y promoviendo inversiones circulares mediante escalamiento de programas existentes.</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI, ya que financia directamente la implementación de la Estrategia Nacional de Economía Circular de Colombia, incluyendo envases/empaques, y promueve inversiones circulares en sectores prioritarios donde ANDI y sus empresas asociadas operan.</t>
+        </is>
+      </c>
+      <c r="V187" t="inlineStr">
+        <is>
+          <t>Escalamiento de modelos de negocio circulares en envases y empaques; fortalecimiento de la articulación entre empresas, gremios y autoridades; pilotos empresariales alineados con la Estrategia Nacional CE; inversiones en infraestructura de reciclaje; implementación de REP; economía circular territorial</t>
+        </is>
+      </c>
+      <c r="W187" t="inlineStr">
+        <is>
+          <t>Articulación con Ministerios de Ambiente y de Comercio, Industria y Turismo; alineación con Estrategia Nacional de Economía Circular; capacidad de escalamiento</t>
+        </is>
+      </c>
+      <c r="X187" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y187" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible (MADS), Ministerio de Comercio, Industria y Turismo, Unión Europea, gremios empresariales, autoridades locales</t>
+        </is>
+      </c>
+      <c r="Z187" t="inlineStr">
+        <is>
+          <t>Fecha de cierre incierta (documento menciona período 2020-22, puede estar finalizada o en extensión); necesidad de verificar vigencia actual y ventanas de aplicación</t>
+        </is>
+      </c>
+      <c r="AA187" t="inlineStr">
+        <is>
+          <t>Contactar urgentemente a los puntos focales de cooperación UE-Colombia en MADS y MinComercio para verificar si hay extensión de fase 2 o apertura de fase 3, y explorar mecanismos de articulación con Visión Circular</t>
+        </is>
+      </c>
+      <c r="AB187" t="inlineStr">
+        <is>
+          <t>Solicitar reunión con la Delegación de la Unión Europea en Colombia y con las direcciones de economía circular de MADS y MinComercio para confirmar vigencia y mecanismos de acceso</t>
+        </is>
+      </c>
+      <c r="AC187" t="inlineStr">
+        <is>
+          <t>Dirección de Alianzas Estratégicas y Cooperación Internacional</t>
+        </is>
+      </c>
+      <c r="AD187" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE187" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF187" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG187" t="inlineStr">
+        <is>
+          <t>Fuente fechada en 2021, menciona período 2020-22. La vigencia actual requiere verificación urgente, pero la relevancia estratégica es máxima por ser cooperación UE-Colombia en economía circular. Es posible que haya fases posteriores o extensiones no documentadas en la fuente. | Fuente fuera del listado oficial conocido (switchtogreen.eu): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH187" t="inlineStr">
+        <is>
+          <t>2dad172e69bef367</t>
+        </is>
+      </c>
+      <c r="AI187" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>VC-0187</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Circular Economy Lab Colombia (Incubadora de Economía Circular)</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible de Colombia en colaboración con PNUD</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Gobierno</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Modelos de negocio circulares, emprendimiento, startups, innovación</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Networking; Acceso a financiamiento</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>https://www.circularinnovationlab.com/post/circular-economy-initiatives-in-colombia</t>
+        </is>
+      </c>
+      <c r="S188" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>El Circular Economy Lab es una incubadora establecida por el Ministerio de Ambiente y Desarrollo Sostenible de Colombia en colaboración con el Programa de las Naciones Unidas para el Desarrollo (PNUD). Su objetivo es asistir a startups y emprendedores en la creación e implementación de modelos de negocio circulares, proporcionando oportunidades de networking y acceso a financiamiento.</t>
+        </is>
+      </c>
+      <c r="U188" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular ANDI como plataforma de articulación con emprendimientos circulares emergentes en envases, reciclaje y economía circular. Permite identificar innovaciones, pilotos empresariales y potenciales aliados para el cierre de ciclo de materiales.</t>
+        </is>
+      </c>
+      <c r="V188" t="inlineStr">
+        <is>
+          <t>Incubación de startups circulares en envases y empaques; pilotos de tecnología de reciclaje y ecodiseño; modelos de negocio circulares escalables; articulación con empresas ANDI para innovación abierta</t>
+        </is>
+      </c>
+      <c r="W188" t="inlineStr">
+        <is>
+          <t>Ser startup o emprendedor en Colombia con modelo de negocio circular; alineación con prioridades de economía circular nacional</t>
+        </is>
+      </c>
+      <c r="X188" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y188" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible, PNUD Colombia, startups circulares, universidades, centros de innovación, empresas ANDI interesadas en innovación abierta</t>
+        </is>
+      </c>
+      <c r="Z188" t="inlineStr">
+        <is>
+          <t>Falta información sobre convocatorias activas, fechas y ventanas de aplicación; URL no es oficial (blog); requiere verificación de estado actual del programa</t>
+        </is>
+      </c>
+      <c r="AA188" t="inlineStr">
+        <is>
+          <t>Verificar con MinAmbiente y PNUD Colombia el estado actual del Circular Economy Lab, próximas convocatorias y explorar alianzas para conectar empresas ANDI con startups incubadas</t>
+        </is>
+      </c>
+      <c r="AB188" t="inlineStr">
+        <is>
+          <t>Contactar a la Dirección de Asuntos Ambientales del MinAmbiente y a la oficina de PNUD Colombia para obtener información oficial sobre el Lab y posibles sinergias con Visión Circular</t>
+        </is>
+      </c>
+      <c r="AC188" t="inlineStr">
+        <is>
+          <t>Coordinación de Innovación y Desarrollo de Proyectos</t>
+        </is>
+      </c>
+      <c r="AD188" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE188" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF188" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG188" t="inlineStr">
+        <is>
+          <t>La fuente es un blog, no un sitio oficial. No se especifican convocatorias activas ni fechas. Se infiere que el programa existe o existió, pero requiere validación de vigencia actual, mecanismos de acceso y convocatorias abiertas. | Fuente fuera del listado oficial conocido (circularinnovationlab.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH188" t="inlineStr">
+        <is>
+          <t>ac19745e26b0296a</t>
+        </is>
+      </c>
+      <c r="AI188" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>VC-0188</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Plastics Innovation Programme 2026</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>United Nations Development Programme (UNDP) / UN Peace and Development Fund (UNPDF)</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Agencia ONU</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Global (con financiación de China y UN DESA)</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Plásticos, reducción de residuos plásticos, alternativas sostenibles</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Piloto demostrativo; Innovación</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/vietnam/news/call-proposals-plastics-innovation-programme-2026</t>
+        </is>
+      </c>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>Convocatoria del UNDP financiada por el UN Peace and Development Fund (con aportes de China y UN DESA) para pilotar y promover iniciativas que reduzcan la generación de residuos plásticos y fomenten la producción de alternativas sostenibles. Orientada a implementar proyectos innovadores en economía circular de plásticos bajo el marco de los ODS 2030.</t>
+        </is>
+      </c>
+      <c r="U189" t="inlineStr">
+        <is>
+          <t>Altamente relevante: aborda reducción de residuos plásticos, alternativas sostenibles y economía circular de envases/empaques, ejes centrales de Visión Circular. Oportunidad para pilotos empresariales, innovación en plásticos flexibles y modelos circulares.</t>
+        </is>
+      </c>
+      <c r="V189" t="inlineStr">
+        <is>
+          <t>Pilotos de reducción de plásticos flexibles en envases; alternativas de materiales sostenibles en empaques; modelos de cierre de ciclo de envases plásticos; articulación con empresas para innovación en ecodiseño y reciclabilidad.</t>
+        </is>
+      </c>
+      <c r="W189" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X189" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y189" t="inlineStr">
+        <is>
+          <t>PNUD Colombia, empresas del sector de envases y empaques (miembros ANDI), centros tecnológicos, universidades con líneas en economía circular, organizaciones de recicladores.</t>
+        </is>
+      </c>
+      <c r="Z189" t="inlineStr">
+        <is>
+          <t>Países elegibles no confirmados en la fuente; la URL hace referencia a UNDP Vietnam, lo que puede indicar convocatoria regional o global; requiere verificar si Colombia es elegible.</t>
+        </is>
+      </c>
+      <c r="AA189" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a UNDP Colombia y UNDP Vietnam para confirmar elegibilidad de Colombia/América Latina, fechas, requisitos y montos. Preparar expresión de interés con pilotos de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB189" t="inlineStr">
+        <is>
+          <t>Escribir a UNDP Colombia y solicitar información oficial sobre la convocatoria 2026, países elegibles, términos de referencia y fechas. Revisar UNPDF website para documentos oficiales.</t>
+        </is>
+      </c>
+      <c r="AC189" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas internacionales</t>
+        </is>
+      </c>
+      <c r="AD189" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF189" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG189" t="inlineStr">
+        <is>
+          <t>La fuente es oficial (UNDP), pero la URL es del sitio de Vietnam; no se especifican países elegibles, fechas ni montos. Se infiere que es convocatoria global bajo UNPDF 2030. Se requiere verificación urgente de elegibilidad Colombia/Latam.</t>
+        </is>
+      </c>
+      <c r="AH189" t="inlineStr">
+        <is>
+          <t>771ff92dd5e84cc6</t>
+        </is>
+      </c>
+      <c r="AI189" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>VC-0189</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Caribbean Biodiversity Fund (CBF) - Second Call for Proposals under the Advancing Circular Economy (ACE) Facility</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Caribbean Biodiversity Fund (CBF)</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Caribe</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Países del Caribe (elegibilidad específica por verificar)</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Reducción y prevención de contaminación marina, conservación de ecosistemas marinos, innovación circular</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Financiamiento concesional; Innovación</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/posts/idblab_sargassum-coastalcommunities-environmental-activity-7285051949224198144-kyCw</t>
+        </is>
+      </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>El Caribbean Biodiversity Fund lanza la Segunda Convocatoria de Propuestas bajo su Facilidad ACE (Advancing Circular Economy). La facilidad provee financiamiento sostenible para proyectos innovadores de economía circular que ayuden a reducir o prevenir la contaminación marina y conservar ecosistemas y biodiversidad marina. El anuncio fue compartido por IDB Lab en LinkedIn.</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>Altamente pertinente para Visión Circular por su enfoque en economía circular, innovación en manejo de residuos que contaminan ecosistemas marinos (incluyendo plásticos y empaques), y potencial para modelos circulares territoriales costeros.</t>
+        </is>
+      </c>
+      <c r="V190" t="inlineStr">
+        <is>
+          <t>Pilotos de economía circular en zonas costeras colombianas (Caribe); innovación en valorización de residuos plásticos que llegan al mar; modelos de negocio circulares para prevención de contaminación marina por envases/empaques; articulación con empresas del sector turismo y pesquero en economía circular</t>
+        </is>
+      </c>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X190" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y190" t="inlineStr">
+        <is>
+          <t>IDB Lab, universidades colombianas con presencia en región Caribe (UniNorte, UniMagdalena), empresas del sector envases/empaques con operaciones caribeñas, asociaciones de recicladores costeros, autoridades ambientales regionales (CRA, Cardique, Corpamag)</t>
+        </is>
+      </c>
+      <c r="Z190" t="inlineStr">
+        <is>
+          <t>Elegibilidad de Colombia por verificar (fondo enfocado en Caribe insular); puede requerir alianza con países caribeños; falta información oficial sobre términos y fechas; competencia regional alta</t>
+        </is>
+      </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>Verificar urgentemente la elegibilidad de Colombia o posibilidad de alianzas con países caribeños; contactar directamente a Caribbean Biodiversity Fund e IDB Lab para confirmar términos de referencia, fechas de cierre y requisitos específicos</t>
+        </is>
+      </c>
+      <c r="AB190" t="inlineStr">
+        <is>
+          <t>Contactar a IDB Lab Colombia y CBF vía correo oficial solicitando TdR completos, fechas de cierre y condiciones de elegibilidad para entidades colombianas o alianzas regionales</t>
+        </is>
+      </c>
+      <c r="AC190" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y movilización de recursos / Área de alianzas internacionales</t>
+        </is>
+      </c>
+      <c r="AD190" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE190" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF190" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG190" t="inlineStr">
+        <is>
+          <t>Información limitada obtenida de post de LinkedIn de IDB Lab. No se accedió a URL oficial de CBF ni términos de referencia completos. La elegibilidad de Colombia requiere verificación ya que CBF típicamente se enfoca en países insulares del Caribe, pero alianzas regionales podrían ser posibles. IDB Lab como promotor sugiere interés en innovación LAC. | Fuente fuera del listado oficial conocido (linkedin.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH190" t="inlineStr">
+        <is>
+          <t>44e1c8a190250424</t>
+        </is>
+      </c>
+      <c r="AI190" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>VC-0190</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>From Battery to Potential - Call for Proposals</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Banco Interamericano de Desarrollo (BID)</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Regional - América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Reuso y valorización de baterías de litio, gestión de residuos electrónicos, innovación en reciclaje tecnológico</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/home/calls-proposals/battery-potential</t>
+        </is>
+      </c>
+      <c r="S191" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>Convocatoria abierta del BID que busca fortalecer y aumentar la visibilidad de innovaciones relacionadas con la gestión circular de baterías, enfocándose en reuso, reciclaje y valorización de baterías de litio. La convocatoria se enmarca en los esfuerzos del BID por promover economía circular y energía limpia en la región.</t>
+        </is>
+      </c>
+      <c r="U191" t="inlineStr">
+        <is>
+          <t>Pertinente para Visión Circular en el contexto de ampliación de alcance a residuos de aparatos eléctricos y electrónicos (RAEE) y baterías, que son objeto de REP en Colombia. Complementa el trabajo en cierre de ciclo y economía circular con un flujo de residuos creciente y estratégico.</t>
+        </is>
+      </c>
+      <c r="V191" t="inlineStr">
+        <is>
+          <t>Pilotos de recolección y valorización de baterías de litio en Colombia; desarrollo de modelos de negocio circulares para RAEE con enfoque en baterías; articulación con empresas de electrónica/movilidad eléctrica; fortalecimiento de capacidades de recicladores para manejo seguro de baterías; ecodiseño de productos con baterías para facilitar circularidad</t>
+        </is>
+      </c>
+      <c r="W191" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X191" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y191" t="inlineStr">
+        <is>
+          <t>Empresas de electrónica y movilidad eléctrica (Samsung, Renault, AKT), gremios (ANDI-sector automotor/electrónica), universidades con investigación en materiales (Uniandes, UdeA, UN), operadores de RAEE certificados, MinAmbiente/MinMinas para alineación regulatoria</t>
+        </is>
+      </c>
+      <c r="Z191" t="inlineStr">
+        <is>
+          <t>Alcance temático específico (baterías) puede requerir expertise técnico especializado que Visión Circular actualmente no tiene como core; competencia con iniciativas especializadas en RAEE; falta de información sobre vigencia actual de la convocatoria</t>
+        </is>
+      </c>
+      <c r="AA191" t="inlineStr">
+        <is>
+          <t>Verificar estado actual de la convocatoria y fechas límite contactando directamente al BID; evaluar posibilidad de alianza con operadores especializados en RAEE o centros tecnológicos para aplicar conjuntamente; considerar como complemento estratégico al trabajo actual en envases/empaques</t>
+        </is>
+      </c>
+      <c r="AB191" t="inlineStr">
+        <is>
+          <t>Consultar página oficial del BID y contactar focal point de economía circular/ambiente del BID Colombia para confirmar vigencia, plazos y requisitos específicos de elegibilidad</t>
+        </is>
+      </c>
+      <c r="AC191" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos con apoyo de área técnica / Potencial alianza con centros de investigación</t>
+        </is>
+      </c>
+      <c r="AD191" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE191" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF191" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG191" t="inlineStr">
+        <is>
+          <t>La convocatoria está publicada en sitio oficial del BID pero no hay información visible sobre fechas de apertura/cierre ni estado actual (puede estar abierta, cerrada o en diseño). Colombia es elegible por ser país miembro del BID. El tema de baterías es complementario pero no central al foco actual de Visión Circular en envases/empaques, aunque sí alineado con economía circular y REP ampliada. Requiere verificación de vigencia.</t>
+        </is>
+      </c>
+      <c r="AH191" t="inlineStr">
+        <is>
+          <t>19dd0102b90c7f40</t>
+        </is>
+      </c>
+      <c r="AI191" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>VC-0191</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Too Good to Waste - Call for Proposals for Pre-Investment Studies in Solid Waste Management</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Banco Interamericano de Desarrollo (BID)</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Regional - América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>20 países de América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Residuos sólidos y economía circular</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Estudios de preinversión, valorización de residuos, prevención, cierre de rellenos, biogás, gestión integral de residuos</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Asistencia técnica; Cooperación técnica; Investigación aplicada</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Demanda total excedió USD 35 millones (referencial de las propuestas recibidas)</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>Cerrada (convocatoria 2024)</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/who-we-are/topics/water-and-sanitation/initiatives/too-good-waste</t>
+        </is>
+      </c>
+      <c r="S192" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>En 2024, el BID lanzó una convocatoria para apoyar estudios de preinversión requeridos en proyectos de gestión de residuos sólidos para economía circular y menores emisiones. Se recibieron 230 propuestas de 20 países: 194 enfocadas en valorización, 18 en prevención y 18 en cierre de rellenos o biogás. La demanda total excedió USD 35 millones, reflejando la necesidad de preparación de proyectos en la región.</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular por su enfoque en valorización de residuos, economía circular y preinversión. Los estudios de preinversión son críticos para escalar proyectos piloto y desarrollar infraestructura circular que cierre ciclos de materiales, especialmente envases y empaques.</t>
+        </is>
+      </c>
+      <c r="V192" t="inlineStr">
+        <is>
+          <t>Estudios de prefactibilidad para plantas de valorización de plásticos flexibles; análisis de viabilidad técnico-económica de modelos REP territoriales; diseño de esquemas de inversión para infraestructura de reciclaje con inclusión de recicladores; estudios de mercado para resinas recicladas post-consumo; evaluación de tecnologías de clasificación y reciclaje químico</t>
+        </is>
+      </c>
+      <c r="W192" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X192" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y192" t="inlineStr">
+        <is>
+          <t>Gobiernos municipales y departamentales, empresas productoras de envases/empaques socias de ANDI, asociaciones de recicladores, universidades para componentes técnicos, MinVivienda y MinAmbiente</t>
+        </is>
+      </c>
+      <c r="Z192" t="inlineStr">
+        <is>
+          <t>La convocatoria 2024 ya cerró. Alta demanda registrada (35M USD) sugiere alta competencia. Es necesario monitorear si habrá una segunda edición en 2025 o 2026.</t>
+        </is>
+      </c>
+      <c r="AA192" t="inlineStr">
+        <is>
+          <t>Contactar al BID para confirmar si habrá una segunda edición de 'Too Good to Waste' en 2025-2026; solicitar retroalimentación sobre los tipos de proyectos priorizados y lecciones aprendidas de la convocatoria 2024; preparar pipeline de estudios de preinversión anticipando futura convocatoria</t>
+        </is>
+      </c>
+      <c r="AB192" t="inlineStr">
+        <is>
+          <t>Enviar correo a responsables del programa Too Good to Waste en BID (División de Agua y Saneamiento) consultando sobre potencial segunda convocatoria y criterios de priorización; registrar interés formal de Visión Circular/ANDI</t>
+        </is>
+      </c>
+      <c r="AC192" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Área de alianzas con banca multilateral</t>
+        </is>
+      </c>
+      <c r="AD192" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE192" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF192" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG192" t="inlineStr">
+        <is>
+          <t>La convocatoria mencionada corresponde a 2024 y ya cerró según la información proporcionada. Sin embargo, la alta demanda (230 propuestas, USD 35M) y el énfasis del BID en el tema sugieren alta probabilidad de que se lance una segunda edición. Se incluye como oportunidad prospectiva que requiere monitoreo activo y relacionamiento temprano con BID para posicionamiento. Colombia participó en la primera edición (es uno de los 20 países mencionados).</t>
+        </is>
+      </c>
+      <c r="AH192" t="inlineStr">
+        <is>
+          <t>f13c7543d41cb3d2</t>
+        </is>
+      </c>
+      <c r="AI192" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>VC-0192</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>IDB Lab + Circulate Capital - Circular Economy Investment and Capacity Development Program for the Caribbean</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>IDB Lab (BID Lab) en alianza con Circulate Capital</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Estados Unidos / Regional América Latina y Caribe</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Región del Caribe (mención específica); potencialmente otros países de América Latina vía alianzas regionales</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Prevención de plásticos en océanos, reciclaje, gestión de residuos plásticos, innovación en economía circular</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Inversión; Fortalecimiento institucional; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/news/idb-lab-partners-circulate-capital-combat-ocean-bound-plastics</t>
+        </is>
+      </c>
+      <c r="S193" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>IDB Lab se ha asociado con Circulate Capital para realizar inversiones en economía circular enfocadas en combatir plásticos que llegan a los océanos en la región del Caribe. El programa combina inversión con desarrollo de capacidades para fortalecer ecosistemas de innovación regional y construir un pipeline de inversiones potenciales en economía circular.</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ya que aborda cierre de ciclo de plásticos, reciclaje, modelos de negocio circulares y fortalecimiento de ecosistemas de innovación. La experiencia de ANDI con empresas y recicladores en Colombia puede ser replicable o escalable hacia el Caribe.</t>
+        </is>
+      </c>
+      <c r="V193" t="inlineStr">
+        <is>
+          <t>Pilotos de cierre de ciclo de envases plásticos flexibles; modelos de inclusión de recicladores replicables regionalmente; soluciones de reciclabilidad y ecodiseño para reducir plásticos ocean-bound; articulación con empresas para responsabilidad extendida del productor (REP) en contextos caribeños.</t>
+        </is>
+      </c>
+      <c r="W193" t="inlineStr">
+        <is>
+          <t>No especificado en la fuente; se infiere que deben ser actores del ecosistema de innovación (empresas, centros tecnológicos, gremios) con propuestas de economía circular aplicables al Caribe.</t>
+        </is>
+      </c>
+      <c r="X193" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y193" t="inlineStr">
+        <is>
+          <t>Circulate Capital (gestor de inversión), gremios del Caribe, universidades y centros de innovación regional, empresas de envases y empaques con operación caribeña, recicladores organizados, autoridades ambientales del Caribe.</t>
+        </is>
+      </c>
+      <c r="Z193" t="inlineStr">
+        <is>
+          <t>Foco principal en Caribe; Colombia podría no ser elegible directamente pero sí como aliado técnico o proveedor de conocimiento. No hay convocatoria pública visible ni fechas. Podría ser inversión cerrada o por invitación.</t>
+        </is>
+      </c>
+      <c r="AA193" t="inlineStr">
+        <is>
+          <t>Contactar directamente a IDB Lab y Circulate Capital para conocer si existen ventanas abiertas, elegibilidad de Colombia como aliado técnico regional, o interés en replicar modelos de Visión Circular en el Caribe.</t>
+        </is>
+      </c>
+      <c r="AB193" t="inlineStr">
+        <is>
+          <t>Escribir a IDB Lab (punto focal Colombia o regional) y Circulate Capital solicitando información sobre elegibilidad, ventanas de aplicación y posibilidades de alianzas técnicas desde Colombia hacia el Caribe.</t>
+        </is>
+      </c>
+      <c r="AC193" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas internacionales y movilización de recursos de PROJECTABILITY / Visión Circular ANDI</t>
+        </is>
+      </c>
+      <c r="AD193" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE193" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF193" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG193" t="inlineStr">
+        <is>
+          <t>La noticia no indica convocatoria abierta ni fechas. Se infiere que es un programa en implementación. Colombia no es Caribe, pero la experiencia de Visión Circular podría ser valiosa como aliado técnico o para replicar modelos. Se recomienda verificación directa con IDB Lab.</t>
+        </is>
+      </c>
+      <c r="AH193" t="inlineStr">
+        <is>
+          <t>14110624761c8128</t>
+        </is>
+      </c>
+      <c r="AI193" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>VC-0193</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Green Climate Fund - NDA Strengthening and Country Programming Support for Colombia (APC-Colombia)</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF)</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Internacional (Naciones Unidas)</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Fortalecimiento institucional, desarrollo de pipeline de inversión climática, NDC, marcos estratégicos climáticos</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Fortalecimiento institucional; Asistencia técnica; Grant no reembolsable (Readiness)</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>07 Nov 2026</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/document/nda-strengthening-and-country-programming-support-colombia-through-apc-colombia</t>
+        </is>
+      </c>
+      <c r="S194" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/document/readiness-grant-agreement-colombia-col-rs-003</t>
+        </is>
+      </c>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>El GCF apoya a Colombia a través de su programa de Readiness para fortalecer la capacidad institucional de la Autoridad Nacional Designada (APC-Colombia) y desarrollar un pipeline nacional de inversiones climáticas alineado con las NDC y marcos estratégicos. El programa incluye apoyo a actores nacionales y subnacionales para identificar y estructurar proyectos climáticos.</t>
+        </is>
+      </c>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>Pertinente para Visión Circular porque el GCF financia proyectos de mitigación y adaptación climática que pueden incluir economía circular, gestión de residuos, reciclaje y reducción de emisiones. El fortalecimiento de APC-Colombia puede abrir puertas para proyectos de REP, cierre de ciclo de envases, y modelos circulares territoriales que aporten a las NDC.</t>
+        </is>
+      </c>
+      <c r="V194" t="inlineStr">
+        <is>
+          <t>Proyectos de economía circular para reducción de emisiones de GEI (ej. reciclaje de plásticos, bioeconomía circular); modelos de gestión territorial de residuos con inclusión de recicladores; ecodiseño y cierre de ciclo de envases para mitigación climática; pilotos empresariales de REP con co-beneficios climáticos.</t>
+        </is>
+      </c>
+      <c r="W194" t="inlineStr">
+        <is>
+          <t>Alineación con las NDC de Colombia y prioridades de APC-Colombia. Proyectos deben demostrar impacto climático (mitigación o adaptación). Se requiere articulación con la NDA (APC-Colombia) y acreditación ante GCF o alianza con entidad acreditada.</t>
+        </is>
+      </c>
+      <c r="X194" t="inlineStr">
+        <is>
+          <t>Concept Note (CN) o Funding Proposal según formato GCF; cartas de no objeción de APC-Colombia; evidencia de impacto climático y sostenibilidad financiera; documentos de alianzas si aplica.</t>
+        </is>
+      </c>
+      <c r="Y194" t="inlineStr">
+        <is>
+          <t>APC-Colombia (NDA), Ministerio de Ambiente y Desarrollo Sostenible, entidades acreditadas ante GCF (ej. FINDETER, Bancóldex, Conservation International), gremios empresariales (ANDI), universidades, centros tecnológicos, organizaciones de recicladores.</t>
+        </is>
+      </c>
+      <c r="Z194" t="inlineStr">
+        <is>
+          <t>El programa de Readiness es principalmente para fortalecimiento institucional de APC-Colombia; no es convocatoria directa para proyectos. Para acceder a financiamiento de proyectos GCF, se requiere acreditación o alianza con entidad acreditada, proceso que puede tardar años. Competencia alta por recursos GCF.</t>
+        </is>
+      </c>
+      <c r="AA194" t="inlineStr">
+        <is>
+          <t>Contactar a APC-Colombia para conocer el pipeline de inversiones climáticas en desarrollo y explorar cómo proyectos de Visión Circular (economía circular, REP, reciclaje) pueden alinearse con las NDC y acceder a financiamiento GCF. Explorar alianzas con entidades ya acreditadas (FINDETER, Conservation International Colombia).</t>
+        </is>
+      </c>
+      <c r="AB194" t="inlineStr">
+        <is>
+          <t>Solicitar reunión con APC-Colombia (punto focal GCF en Colombia) para presentar Visión Circular y explorar oportunidades de incluir economía circular en el pipeline nacional de proyectos climáticos GCF.</t>
+        </is>
+      </c>
+      <c r="AC194" t="inlineStr">
+        <is>
+          <t>Dirección de Visión Circular ANDI y área de alianzas estratégicas de PROJECTABILITY</t>
+        </is>
+      </c>
+      <c r="AD194" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE194" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF194" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG194" t="inlineStr">
+        <is>
+          <t>El documento hace referencia a fortalecimiento institucional de APC-Colombia (Readiness), no a convocatoria abierta de proyectos. Sin embargo, el desarrollo del pipeline nacional de inversiones climáticas es una ventana para posicionar economía circular. La fecha '07 Nov 2026' parece ser de un documento relacionado (República Dominicana), no necesariamente de Colombia. Se requiere verificación directa con APC-Colombia sobre ventanas y elegibilidad de proyectos de economía circular.</t>
+        </is>
+      </c>
+      <c r="AH194" t="inlineStr">
+        <is>
+          <t>5cd9008be2750fe1</t>
+        </is>
+      </c>
+      <c r="AI194" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>VC-0194</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Green Climate Fund - Catalyzing Colombia's Just Energy Transition</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF)</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Internacional (Naciones Unidas)</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Transición energética justa, mitigación climática, NDC</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Grant no reembolsable; Cofinanciación; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>Sí (típicamente GCF requiere cofinanciación)</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/document/nda-strengthening-and-country-programming-support-colombia-through-apc-colombia</t>
+        </is>
+      </c>
+      <c r="S195" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>El GCF menciona el proyecto 'Catalyzing Colombia's Just Energy Transition' como parte del portafolio de apoyo a Colombia. Se enfoca en catalizador de la transición energética justa del país, alineado con las NDC. Aunque el foco es energía, podría tener componentes de economía circular o co-beneficios en sostenibilidad industrial.</t>
+        </is>
+      </c>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>Relación indirecta pero aprovechable. La transición energética justa en Colombia puede incluir componentes de economía circular industrial, eficiencia de recursos, y sostenibilidad en cadenas de valor (ej. reciclaje de componentes de energías renovables, gestión de residuos industriales). Visión Circular podría articularse en componentes de circularidad industrial o REP en sectores energéticos.</t>
+        </is>
+      </c>
+      <c r="V195" t="inlineStr">
+        <is>
+          <t>Circularidad en cadenas de valor de energías renovables (reciclaje de paneles solares, baterías); modelos de economía circular para industrias en transición energética; gestión de residuos de equipos eléctricos y electrónicos; ecodiseño y REP para sectores industriales bajos en carbono.</t>
+        </is>
+      </c>
+      <c r="W195" t="inlineStr">
+        <is>
+          <t>Alineación con transición energética justa y NDC de Colombia. Requiere articulación con APC-Colombia y entidades acreditadas GCF. Demostración de impacto climático y social (justicia, inclusión).</t>
+        </is>
+      </c>
+      <c r="X195" t="inlineStr">
+        <is>
+          <t>No especificado; típicamente Concept Note GCF, cartas de no objeción, documentos de impacto climático y social.</t>
+        </is>
+      </c>
+      <c r="Y195" t="inlineStr">
+        <is>
+          <t>APC-Colombia, Ministerio de Minas y Energía, Ministerio de Ambiente, UPME, entidades acreditadas GCF (FINDETER, Bancóldex), empresas del sector energético en transición, gremios industriales (ANDI), universidades.</t>
+        </is>
+      </c>
+      <c r="Z195" t="inlineStr">
+        <is>
+          <t>El foco principal es transición energética, no economía circular directamente. Visión Circular tendría que demostrar co-beneficios claros y alineación con objetivos energéticos del proyecto. No se identifica convocatoria abierta ni ventana de aplicación. Puede ser proyecto cerrado en estructuración o implementación.</t>
+        </is>
+      </c>
+      <c r="AA195" t="inlineStr">
+        <is>
+          <t>Monitorear evolución del proyecto 'Catalyzing Colombia's Just Energy Transition' y explorar con APC-Colombia si hay componentes de economía circular, gestión de residuos o REP donde Visión Circular pueda articularse. Evaluar si hay ventanas de alianzas técnicas o co-diseño.</t>
+        </is>
+      </c>
+      <c r="AB195" t="inlineStr">
+        <is>
+          <t>Consultar con APC-Colombia el estado del proyecto, componentes, y posibilidades de articulación de Visión Circular en economía circular industrial o gestión de residuos de equipos energéticos.</t>
+        </is>
+      </c>
+      <c r="AC195" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas de Visión Circular ANDI</t>
+        </is>
+      </c>
+      <c r="AD195" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE195" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF195" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG195" t="inlineStr">
+        <is>
+          <t>La fuente solo menciona el proyecto sin detalles. Se infiere que es un proyecto GCF en desarrollo o implementación en Colombia. La relación con economía circular es indirecta; Visión Circular tendría que identificar componentes específicos donde pueda aportar (ej. circularidad en cadenas de valor energéticas). No hay convocatoria abierta identificada. Se requiere verificación de estado y componentes del proyecto.</t>
+        </is>
+      </c>
+      <c r="AH195" t="inlineStr">
+        <is>
+          <t>bab6aa830432c7ec</t>
+        </is>
+      </c>
+      <c r="AI195" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>VC-0195</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Green Climate Fund - Conservation International Initiative for Water Security in Bogotá</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF) + Conservation International Colombia</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Internacional (Naciones Unidas) + Colombia</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Colombia (Bogotá y regiones circundantes)</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Seguridad hídrica, restauración de ecosistemas, adaptación climática, resiliencia</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Grant no reembolsable; Cofinanciación</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>No especificado (típicamente sí en proyectos GCF)</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/about/news-and-updates/green-climate-fund-support-development-conservation-international-initiative-transform-water</t>
+        </is>
+      </c>
+      <c r="S196" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>El GCF apoya el desarrollo de una propuesta de Conservation International Colombia para transformar la seguridad hídrica de Bogotá y sus regiones circundantes mediante restauración de ecosistemas, soluciones basadas en naturaleza y ciencia. El proyecto busca construir resiliencia climática para millones de personas en la región de Bogotá.</t>
+        </is>
+      </c>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>Relación indirecta con Visión Circular. El foco es seguridad hídrica y restauración de ecosistemas, pero podría tener componentes de economía circular urbana (gestión de residuos para protección de fuentes hídricas, modelos circulares de consumo de agua, reciclaje de materiales para infraestructura verde). Visión Circular podría articularse en componentes de gestión circular de residuos que afectan cuerpos de agua.</t>
+        </is>
+      </c>
+      <c r="V196" t="inlineStr">
+        <is>
+          <t>Gestión circular de residuos sólidos para protección de cuencas hídricas; modelos de reciclaje y REP que reduzcan contaminación de fuentes de agua; infraestructura verde con materiales reciclados; bioeconomía circular en territorios de cuencas; articulación con recicladores en zonas de influencia hídrica.</t>
+        </is>
+      </c>
+      <c r="W196" t="inlineStr">
+        <is>
+          <t>Alineación con objetivos de seguridad hídrica, adaptación climática y restauración de ecosistemas. Requiere articulación con Conservation International Colombia (entidad implementadora acreditada GCF) y APC-Colombia. Demostración de co-beneficios hídricos y climáticos.</t>
+        </is>
+      </c>
+      <c r="X196" t="inlineStr">
+        <is>
+          <t>No especificado; típicamente Concept Note GCF, cartas de soporte de actores clave, estudios de impacto.</t>
+        </is>
+      </c>
+      <c r="Y196" t="inlineStr">
+        <is>
+          <t>Conservation International Colombia, APC-Colombia, Secretaría de Ambiente de Bogotá, Empresa de Acueducto y Alcantarillado de Bogotá (EAAB), CAR Cundinamarca, universidades, organizaciones de recicladores de Bogotá y región.</t>
+        </is>
+      </c>
+      <c r="Z196" t="inlineStr">
+        <is>
+          <t>El foco principal es seguridad hídrica y ecosistemas, no economía circular. Visión Circular tendría que demostrar contribución clara a objetivos hídricos. El proyecto está en fase de desarrollo de propuesta (no implementación); no se identifica convocatoria abierta para aliados. Puede ser propuesta cerrada liderada por Conservation International.</t>
+        </is>
+      </c>
+      <c r="AA196" t="inlineStr">
+        <is>
+          <t>Contactar a Conservation International Colombia para explorar si hay espacio de articulación de Visión Circular en componentes de gestión de residuos, reciclaje o economía circular urbana que aporten a la seguridad hídrica. Evaluar co-beneficios de modelos circulares para protección de fuentes de agua.</t>
+        </is>
+      </c>
+      <c r="AB196" t="inlineStr">
+        <is>
+          <t>Escribir a Conservation International Colombia (Fabio Arjona, VP mencionado en la fuente) para conocer el estado de la propuesta, componentes y posibilidades de alianzas en economía circular urbana/territorial con impacto hídrico.</t>
+        </is>
+      </c>
+      <c r="AC196" t="inlineStr">
+        <is>
+          <t>Coordinación de economía circular territorial de Visión Circular ANDI</t>
+        </is>
+      </c>
+      <c r="AD196" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AE196" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF196" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG196" t="inlineStr">
+        <is>
+          <t>El proyecto está en fase de desarrollo de propuesta, no en implementación ni convocatoria abierta. La relación con economía circular es tangencial; tendría que construirse vía gestión de residuos para protección hídrica. Se requiere contacto directo con Conservation International Colombia para evaluar pertinencia y espacios de articulación. No hay fechas ni ventanas identificadas.</t>
+        </is>
+      </c>
+      <c r="AH196" t="inlineStr">
+        <is>
+          <t>f049919757b2384c</t>
+        </is>
+      </c>
+      <c r="AI196" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>VC-0196</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme - Colombia (Plastics and Solid Waste Management Programme)</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) / UNDP</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Residuos</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Plásticos, Gestión de residuos sólidos, Iniciativas comunitarias</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Fortalecimiento institucional; Inclusión social</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Hasta USD 15,000 para organizaciones comunitarias; hasta USD 35,000 para organizaciones con experiencia previa</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/sites/g/files/zskgke326/files/2025-10/call_for_proposals-plastics_and_waste_management_programme.pdf</t>
+        </is>
+      </c>
+      <c r="S197" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/newsroom/news/gef-small-grants-programme-launched-colombia</t>
+        </is>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>El GEF Small Grants Programme en Colombia financia iniciativas comunitarias en gestión de plásticos y residuos sólidos con grants de hasta USD 15,000 (organizaciones comunitarias) y USD 35,000 (organizaciones con experiencia). Implementado por UNDP, busca soluciones ambientales lideradas por comunidades locales.</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>Altamente relevante para el componente de inclusión de recicladores y proyectos comunitarios de economía circular. Puede financiar pilotos territoriales de gestión de residuos plásticos y envases con organizaciones de base.</t>
+        </is>
+      </c>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de cooperativas de recicladores; pilotos comunitarios de recolección y separación de plásticos flexibles; sistemas locales de economía circular para envases; capacitación técnica en reciclaje y valorización; modelos de negocio circulares comunitarios</t>
+        </is>
+      </c>
+      <c r="W197" t="inlineStr">
+        <is>
+          <t>Organizaciones comunitarias o de base; experiencia previa en gestión de recursos para montos mayores; proyectos enfocados en plásticos y residuos sólidos</t>
+        </is>
+      </c>
+      <c r="X197" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>Cooperativas de recicladores, organizaciones comunitarias, ONGs locales, gobiernos municipales, ANDI como articulador empresarial</t>
+        </is>
+      </c>
+      <c r="Z197" t="inlineStr">
+        <is>
+          <t>Montos limitados para proyectos de escala empresarial; enfoque principalmente comunitario puede requerir adaptación del modelo de Visión Circular; falta información sobre fechas y proceso de aplicación actual</t>
+        </is>
+      </c>
+      <c r="AA197" t="inlineStr">
+        <is>
+          <t>Contactar a UNDP Colombia y GEF SGP Bogotá (Pilar Barrera Rey, Coordinadora de Partnerships) para confirmar ventana de convocatoria 2025 y explorar alianzas con organizaciones comunitarias para proyectos de inclusión de recicladores</t>
+        </is>
+      </c>
+      <c r="AB197" t="inlineStr">
+        <is>
+          <t>Solicitar términos de referencia actualizados y cronograma de convocatorias 2025 al equipo GEF SGP en Colombia vía UNDP</t>
+        </is>
+      </c>
+      <c r="AC197" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos e inclusión social / Alianzas territoriales</t>
+        </is>
+      </c>
+      <c r="AD197" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE197" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF197" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG197" t="inlineStr">
+        <is>
+          <t>El documento de convocatoria tiene fecha octubre 2025 (posiblemente error tipográfico por 2024). La información confirma que el programa está activo en Colombia pero no especifica si hay convocatoria abierta actualmente. Requiere verificación de ventanas 2025.</t>
+        </is>
+      </c>
+      <c r="AH197" t="inlineStr">
+        <is>
+          <t>72f393da9d02bfff</t>
+        </is>
+      </c>
+      <c r="AI197" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>VC-0197</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Green Climate Fund - Colombia Country Programme</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF)</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Mitigación climática, Adaptación, Proyectos de bajo carbono</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Grant no reembolsable; Financiamiento concesional; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>No especificado (varía por proyecto, típicamente millones de USD)</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>Sí, generalmente requerida</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>Proceso continuo</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/countries/colombia</t>
+        </is>
+      </c>
+      <c r="S198" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>El Green Climate Fund mantiene un programa activo en Colombia para financiar proyectos de mitigación y adaptación climática. Trabaja con entidades acreditadas nacionales e internacionales. Financiamiento disponible para proyectos de bajo carbono con componentes de innovación y sostenibilidad.</t>
+        </is>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>Relevante para proyectos de economía circular con impacto climático demostrable, como reducción de emisiones por reciclaje, valorización de residuos, prevención de metano en rellenos sanitarios, y cadenas de valor circulares bajas en carbono.</t>
+        </is>
+      </c>
+      <c r="V198" t="inlineStr">
+        <is>
+          <t>Sistemas de reciclaje para reducción de emisiones GEI; infraestructura de economía circular baja en carbono; valorización energética de residuos; cadenas de reciclaje de plásticos con cuantificación de carbono evitado; modelos empresariales circulares climáticamente inteligentes</t>
+        </is>
+      </c>
+      <c r="W198" t="inlineStr">
+        <is>
+          <t>Trabajar con entidad acreditada de GCF; demostrar impacto climático claro (mitigación o adaptación); modelo financiero robusto con cofinanciación; alineación con NDC y prioridades nacionales climáticas de Colombia</t>
+        </is>
+      </c>
+      <c r="X198" t="inlineStr">
+        <is>
+          <t>Concept Note, propuesta completa (Funding Proposal), análisis financiero, evaluación de impacto climático, salvaguardas ambientales y sociales, cartas de no objeción del gobierno</t>
+        </is>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>Entidades acreditadas de GCF en Colombia (ej. Bancoldex, Findeter), Ministerio de Ambiente, ANDI como articulador empresarial, universidades para medición de impacto, empresas como cofinanciadoras</t>
+        </is>
+      </c>
+      <c r="Z198" t="inlineStr">
+        <is>
+          <t>Proceso largo y complejo de preparación de propuestas; requisitos técnicos exigentes en demostración de impacto climático; requiere entidad acreditada como intermediario; alta competencia por recursos; cofinanciación significativa requerida</t>
+        </is>
+      </c>
+      <c r="AA198" t="inlineStr">
+        <is>
+          <t>Identificar proyectos de economía circular con componente climático fuerte y cuantificable. Contactar entidades acreditadas de GCF en Colombia para explorar desarrollo conjunto de propuesta de proyecto</t>
+        </is>
+      </c>
+      <c r="AB198" t="inlineStr">
+        <is>
+          <t>Revisar portafolio actual de GCF en Colombia para identificar áreas prioritarias y contactar a Findeter o Bancoldex (entidades acreditadas) para explorar interés en proyectos de economía circular</t>
+        </is>
+      </c>
+      <c r="AC198" t="inlineStr">
+        <is>
+          <t>Dirección ejecutiva / Coordinación de financiamiento climático</t>
+        </is>
+      </c>
+      <c r="AD198" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE198" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF198" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG198" t="inlineStr">
+        <is>
+          <t>GCF es fuente importante pero compleja. Requiere demostrar claramente el vínculo entre economía circular y mitigación/adaptación climática. La ventana es continua pero el proceso toma 1-2 años. Mejor para proyectos grandes (&gt;USD 5 millones) con impacto climático medible y cofinanciación asegurada.</t>
+        </is>
+      </c>
+      <c r="AH198" t="inlineStr">
+        <is>
+          <t>9169d40dc7ae1aca</t>
+        </is>
+      </c>
+      <c r="AI198" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>VC-0198</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Programa Euroclima - Acción de Economía Circular</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Unión Europea y Gobierno Federal de Alemania</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Unión Europea / Alemania</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Acción climática local, economía circular, biodiversidad</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>Cofinanciado por la Unión Europea y el gobierno federal de Alemania</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>https://www.euroclima.org</t>
+        </is>
+      </c>
+      <c r="S199" t="inlineStr">
+        <is>
+          <t>https://ccesantiago.aecid.es/-/cce-santiago-acoge-presentaci%C3%B3n-de-proyecto-para-fortalecer-la-acci%C3%B3n-clim%C3%A1tica-local-y-la-econom%C3%ADa-circular</t>
+        </is>
+      </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>Euroclima es una iniciativa de cooperación regional entre la UE y América Latina que fortalece la acción climática y promueve la economía circular. El programa está diseñando una nueva acción específica en economía circular (mencionada en documentos de Guatemala) y opera mediante metodología de Diálogo País para el fortalecimiento institucional.</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>Altamente relevante: Euroclima tiene líneas específicas de economía circular, gestión de residuos, cadenas de valor libres de deforestación y transición sostenible, todas alineadas con los objetivos de Visión Circular ANDI. La metodología de Diálogo País permite trabajar con sectores público, privado y sociedad civil.</t>
+        </is>
+      </c>
+      <c r="V199" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de capacidades en economía circular territorial; asistencia técnica para implementación de REP; pilotos de cierre de ciclo de envases; proyectos de bioeconomía y cadenas de valor circulares; inclusión de recicladores en modelos circulares</t>
+        </is>
+      </c>
+      <c r="W199" t="inlineStr">
+        <is>
+          <t>Alineación con prioridades nacionales de acción climática; articulación público-privada; enfoque en transición sostenible, resiliente e inclusiva</t>
+        </is>
+      </c>
+      <c r="X199" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible; DNP; gobiernos locales; empresas miembro de ANDI; universidades; organizaciones de recicladores; agencias implementadoras como Expertise France, FIIAPP, GIZ</t>
+        </is>
+      </c>
+      <c r="Z199" t="inlineStr">
+        <is>
+          <t>Las convocatorias Euroclima suelen tener ventanas específicas no permanentes; puede requerir articulación con autoridades nacionales; los tiempos de diseño e implementación son largos</t>
+        </is>
+      </c>
+      <c r="AA199" t="inlineStr">
+        <is>
+          <t>Contactar a la Delegación de la UE en Colombia y a las agencias implementadoras (Expertise France, GIZ, FIIAPP) para conocer el estado de diseño de la nueva acción de economía circular y explorar participación de ANDI/Visión Circular como socio implementador o beneficiario</t>
+        </is>
+      </c>
+      <c r="AB199" t="inlineStr">
+        <is>
+          <t>Solicitar reunión con punto focal Euroclima en Colombia (Delegación UE) y revisar las publicaciones recientes del programa sobre economía circular en https://www.euroclima.org</t>
+        </is>
+      </c>
+      <c r="AC199" t="inlineStr">
+        <is>
+          <t>Dirección de Visión Circular ANDI / Coordinación de cooperación internacional</t>
+        </is>
+      </c>
+      <c r="AD199" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE199" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF199" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG199" t="inlineStr">
+        <is>
+          <t>Euroclima es un programa establecido con presencia confirmada en América Latina. Las fuentes mencionan diseño de nueva acción de economía circular, lo que sugiere futuras oportunidades. Colombia es país elegible confirmado. Se infiere que habrá convocatorias futuras basadas en la mención de 'desarrollo de la próxima fase' y 'diseño de nueva Acción'.</t>
+        </is>
+      </c>
+      <c r="AH199" t="inlineStr">
+        <is>
+          <t>38bcb7a93cbb3b71</t>
+        </is>
+      </c>
+      <c r="AI199" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-09-04
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI249"/>
+  <dimension ref="A1:AI254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44486,6 +44486,891 @@
       <c r="AI249" t="inlineStr">
         <is>
           <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>VC-0249</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator Colombia – Call for Proposals 2026</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Transición baja en carbono; Preparación para inversión</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P250" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R250" t="inlineStr">
+        <is>
+          <t>https://bogota.gov.co/boletin-oferta-internacional/climate-finance-accelerator-colombia-2026-acelera-proyectos-climatico</t>
+        </is>
+      </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T250" t="inlineStr">
+        <is>
+          <t>La convocatoria Climate Finance Accelerator Colombia 2026 busca apoyar proyectos climáticos de alto impacto que fortalezcan la preparación para recibir inversión y escalen soluciones que contribuyan a la transición hacia una economía baja en carbono. Se ofrece financiamiento no reembolsable y asistencia técnica para la elaboración de planes de negocio y estrategias de escalamiento.</t>
+        </is>
+      </c>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>Aunque el foco principal es el clima, la iniciativa promueve soluciones que pueden incluir economía circular, como la reducción de residuos y la optimización de recursos, alineándose con los objetivos de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V250" t="inlineStr">
+        <is>
+          <t>Desarrollo de modelos de negocio circulares en la gestión de residuos; Diseño de soluciones de reciclaje y ecodiseño; Estrategias de escalamiento de tecnologías limpias.</t>
+        </is>
+      </c>
+      <c r="W250" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X250" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y250" t="inlineStr">
+        <is>
+          <t>Gremios de recicladores, universidades de ingeniería ambiental, centros de innovación tecnológica</t>
+        </is>
+      </c>
+      <c r="Z250" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AA250" t="inlineStr">
+        <is>
+          <t>Revisar la convocatoria en detalle y preparar un dossier de proyecto que destaque la dimensión circular y la preparación para inversión.</t>
+        </is>
+      </c>
+      <c r="AB250" t="inlineStr">
+        <is>
+          <t>Solicitar información adicional a Climate Finance Accelerator y definir un equipo de proyecto.</t>
+        </is>
+      </c>
+      <c r="AC250" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y Alianzas</t>
+        </is>
+      </c>
+      <c r="AD250" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE250" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF250" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG250" t="inlineStr">
+        <is>
+          <t>No se indica monto ni fechas exactas; se requiere confirmar vigencia y requisitos específicos. | Fuente fuera del listado oficial conocido (bogota.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH250" t="inlineStr">
+        <is>
+          <t>e88c808550ba419c</t>
+        </is>
+      </c>
+      <c r="AI250" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>VC-0250</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Horizon Europe 2025 Call – Eco-Friendly Packaging</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>European Commission</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>European Union</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>European Union member states; associated countries (including Colombia if allowed)</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>Envases y empaques</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Ecodiseño; Reciclabilidad; Plásticos flexibles</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>Hasta €20M</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>Sí (co-financiación con socios europeos)</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>2025-09-18</t>
+        </is>
+      </c>
+      <c r="P251" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/packaging</t>
+        </is>
+      </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>https://getgrant.eu/grants-and-funding/grant-for-eco-friendly-packaging-horizon-europe-2025-call-for-innovative-materials</t>
+        </is>
+      </c>
+      <c r="T251" t="inlineStr">
+        <is>
+          <t>El programa Horizon Europe 2025 ofrece financiamiento no reembolsable para proyectos de innovación en envases sostenibles, con un presupuesto de hasta €20M. Se busca colaboración con socios europeos y se requiere cofinanciación.</t>
+        </is>
+      </c>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>Apoya la innovación en envases circulares y la colaboración internacional, alineado con Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V251" t="inlineStr">
+        <is>
+          <t>Desarrollo de materiales reciclables, diseño de envases de bajo impacto, sistemas de recogida y reciclaje.</t>
+        </is>
+      </c>
+      <c r="W251" t="inlineStr">
+        <is>
+          <t>Participación de socios europeos, cumplimiento de criterios de sostenibilidad, propuesta de valor innovador.</t>
+        </is>
+      </c>
+      <c r="X251" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto, CVs, presupuesto, cartas de compromiso de socios.</t>
+        </is>
+      </c>
+      <c r="Y251" t="inlineStr">
+        <is>
+          <t>Universidades europeas, empresas de packaging, ONG de reciclaje.</t>
+        </is>
+      </c>
+      <c r="Z251" t="inlineStr">
+        <is>
+          <t>Requisitos de cofinanciación, competencia alta, requisitos de socios europeos.</t>
+        </is>
+      </c>
+      <c r="AA251" t="inlineStr">
+        <is>
+          <t>Explorar alianzas con socios europeos y preparar propuesta.</t>
+        </is>
+      </c>
+      <c r="AB251" t="inlineStr">
+        <is>
+          <t>Consultar la convocatoria oficial y evaluar elegibilidad.</t>
+        </is>
+      </c>
+      <c r="AC251" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos internacionales</t>
+        </is>
+      </c>
+      <c r="AD251" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE251" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF251" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG251" t="inlineStr">
+        <is>
+          <t>La elegibilidad para Colombia no está confirmada; se requiere verificación de requisitos de socios europeos.</t>
+        </is>
+      </c>
+      <c r="AH251" t="inlineStr">
+        <is>
+          <t>ce34e30e74c96015</t>
+        </is>
+      </c>
+      <c r="AI251" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>VC-0251</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>IKI Country Call Colombia 2024</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>International Climate Initiative (IKI)</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>https://www.international-climate-initiative.com/fileadmin/iki/Dokumente/Calls/Laendercall/Kolumbien2024/240718_IKI_country_call_COL_funding_announcement_bf.pdf</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>El IKI Country Call Colombia 2024 invita a proyectos que contribuyan a la mitigación y adaptación climática en Colombia, con énfasis en soluciones de economía circular y gestión de residuos. Ofrece financiamiento no reembolsable y apoyo técnico.</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>Relevante por su enfoque en soluciones de economía circular y gestión de residuos, alineado con Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V252" t="inlineStr">
+        <is>
+          <t>Desarrollo de sistemas de reciclaje de plásticos, inclusión de recicladores, ecodiseño de envases.</t>
+        </is>
+      </c>
+      <c r="W252" t="inlineStr">
+        <is>
+          <t>Ser entidad colombiana, proyecto con impacto climático, capacidad técnica.</t>
+        </is>
+      </c>
+      <c r="X252" t="inlineStr">
+        <is>
+          <t>Propuesta técnica, plan financiero, CV del equipo.</t>
+        </is>
+      </c>
+      <c r="Y252" t="inlineStr">
+        <is>
+          <t>Gremios de recicladores, universidades, ONGs.</t>
+        </is>
+      </c>
+      <c r="Z252" t="inlineStr">
+        <is>
+          <t>Requisitos de elegibilidad, competencia alta.</t>
+        </is>
+      </c>
+      <c r="AA252" t="inlineStr">
+        <is>
+          <t>Revisar PDF, preparar propuesta.</t>
+        </is>
+      </c>
+      <c r="AB252" t="inlineStr">
+        <is>
+          <t>Descargar PDF, identificar requisitos.</t>
+        </is>
+      </c>
+      <c r="AC252" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos</t>
+        </is>
+      </c>
+      <c r="AD252" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE252" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF252" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG252" t="inlineStr">
+        <is>
+          <t>Fecha de apertura y cierre no especificadas en el PDF; requiere verificación. | Fuente fuera del listado oficial conocido (international-climate-initiative.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH252" t="inlineStr">
+        <is>
+          <t>89f8237175926e81</t>
+        </is>
+      </c>
+      <c r="AI252" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>VC-0252</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme – Colombia</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF)</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Multilateral</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Colombia; América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>Reciclaje; Inclusión de recicladores; Ecodiseño</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>$15,000 - $35,000</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/newsroom/news/gef-small-grants-programme-launched-colombia</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>El programa GEF Small Grants Programme ofrece subvenciones no reembolsables de hasta $35,000 para organizaciones con experiencia en gestión de recursos y de hasta $15,000 para organizaciones comunitarias, con el objetivo de financiar proyectos de innovación ambiental y sostenibilidad en Colombia.</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>Apoya la financiación de iniciativas de economía circular y reciclaje, alineándose con los objetivos de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V253" t="inlineStr">
+        <is>
+          <t>Desarrollo de proyectos de reciclaje de plásticos, ecodiseño de empaques, inclusión de recicladores, programas de educación ambiental.</t>
+        </is>
+      </c>
+      <c r="W253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Z253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AA253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AB253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AC253" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AD253" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE253" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF253" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG253" t="inlineStr">
+        <is>
+          <t>No se indica fecha de apertura/cierre; se requiere confirmación de vigencia.</t>
+        </is>
+      </c>
+      <c r="AH253" t="inlineStr">
+        <is>
+          <t>7ebd6d6ec6c88ece</t>
+        </is>
+      </c>
+      <c r="AI253" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>VC-0253</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Program</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF)</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Colombia; Todos los países miembros del GEF</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Financiación de proyectos comunitarios de adaptación y mitigación climática</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>Hasta $50,000</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>https://ndcpartnership.org/knowledge-portal/climate-funds-explorer/global-environment-facility-gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>El GEF Small Grants Program ofrece subvenciones no reembolsables de hasta $50,000 a comunidades locales, organizaciones indígenas y grupos comunitarios para proyectos de adaptación y mitigación climática, con enfoque en la resiliencia y la sostenibilidad.</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>Aunque el programa se centra en la adaptación climática, los proyectos pueden incluir componentes de economía circular, como gestión de residuos y reciclaje, alineándose con los objetivos de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V254" t="inlineStr">
+        <is>
+          <t>Gestión de residuos sólidos, reciclaje de plásticos, ecodiseño de productos, inclusión de recicladores, proyectos de economía circular a nivel comunitario.</t>
+        </is>
+      </c>
+      <c r="W254" t="inlineStr">
+        <is>
+          <t>Ser una organización comunitaria, ONG, o grupo indígena; proyecto con impacto local; capacidad de gestión; no requerir cofinanciación.</t>
+        </is>
+      </c>
+      <c r="X254" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto, presupuesto, carta de apoyo, plan de gestión de residuos, etc.</t>
+        </is>
+      </c>
+      <c r="Y254" t="inlineStr">
+        <is>
+          <t>ONG locales, universidades, gremios de recicladores, autoridades locales.</t>
+        </is>
+      </c>
+      <c r="Z254" t="inlineStr">
+        <is>
+          <t>Fecha de cierre no especificada; posible alta competencia; requisitos de reporte.</t>
+        </is>
+      </c>
+      <c r="AA254" t="inlineStr">
+        <is>
+          <t>Revisar la página oficial del GEF SGP y preparar una propuesta alineada con los criterios de la convocatoria.</t>
+        </is>
+      </c>
+      <c r="AB254" t="inlineStr">
+        <is>
+          <t>Consultar la sección de 'Call for Proposals' en la página del GEF SGP y confirmar fechas de apertura y cierre.</t>
+        </is>
+      </c>
+      <c r="AC254" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas</t>
+        </is>
+      </c>
+      <c r="AD254" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE254" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF254" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG254" t="inlineStr">
+        <is>
+          <t>La convocatoria no indica fechas de apertura y cierre ni confirma la elegibilidad directa para Colombia; se necesita confirmar con GEF. | Fuente fuera del listado oficial conocido (ndcpartnership.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH254" t="inlineStr">
+        <is>
+          <t>c42be838c7546297</t>
+        </is>
+      </c>
+      <c r="AI254" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>

</xml_diff>